<commit_message>
fix(ai-sow-lite): keep acceptance and pending decisions inline
</commit_message>
<xml_diff>
--- a/plugins/ai-sow-lite/assets/sow-template.xlsx
+++ b/plugins/ai-sow-lite/assets/sow-template.xlsx
@@ -484,7 +484,7 @@
       <calculatedColumnFormula>IF($C5="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C5,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="10" name="校验结果">
-      <calculatedColumnFormula>IF(COUNTA($A5:$C5,$D5:$E5)=0,"",IF(OR($A5="",$B5="",$C5="",$F5="",$G5="",$D5=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C5)&gt;1,"故事名称重复",IF(OR(AND($F5&lt;&gt;"是",$F5&lt;&gt;"否"),AND($G5&lt;&gt;"是",$G5&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C5)=0,"故事缺少任务","通过")))))</calculatedColumnFormula>
+      <calculatedColumnFormula>IF(COUNTA($A5:$C5,$D5:$E5)=0,"",IF(LEFT($E5,4)="待确认：","待确认",IF(OR($A5="",$B5="",$C5="",$F5="",$G5="",$D5=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C5)&gt;1,"故事名称重复",IF(OR(AND($F5&lt;&gt;"是",$F5&lt;&gt;"否"),AND($G5&lt;&gt;"是",$G5&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C5)=0,"故事缺少任务","通过"))))))</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -515,7 +515,7 @@
       <calculatedColumnFormula>IF(COUNTA($A5:$G5)=0,"",IF($F5="",0,IF(NOT(ISNUMBER($I5)),"",IF($F5="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I5,1),IF($F5="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I5,1),"")))))</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="12" name="校验结果">
-      <calculatedColumnFormula>IF(COUNTA($A5:$G5)=0,"",IF(OR($A5="",$B5="",$C5="",$D5="",$E5=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B5))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A5))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E5="S",$E5="M",$E5="L")),"复杂度非法",IF(NOT(OR($F5="",$F5="内部集成",$F5="外部集成")),"集成类型非法",IF(AND($F5&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C5,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F5="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C5,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H5),"通过","工作类型与工作方式不适用")))))))))</calculatedColumnFormula>
+      <calculatedColumnFormula>IF(COUNTA($A5:$G5)=0,"",IF(LEFT($G5,4)="待确认：","待确认",IF(OR($A5="",$B5="",$C5="",$D5="",$E5=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B5))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A5))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E5="S",$E5="M",$E5="L")),"复杂度非法",IF(NOT(OR($F5="",$F5="内部集成",$F5="外部集成")),"集成类型非法",IF(AND($F5&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C5,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F5="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C5,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H5),"通过","工作类型与工作方式不适用"))))))))))</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -892,7 +892,7 @@
     </s:row>
     <s:row r="2" ht="34" customHeight="1">
       <s:c r="A2" t="str" s="2">
-        <s:v>每个 Story 一行；标题使用自然的角色/对象动作。每条验收条件以“• ”开头并独占一行；任务列表显示“[任务类型/工作方式/复杂度]”。备注只显示对象特有风险、假设、边界或不确定性，通用事项留在说明中。SIT/UAT适用由关联任务类型自动计算；灰色列为只读公式，请勿修改。</s:v>
+        <s:v>每个 Story 一行；标题使用自然的角色/对象动作。无待确认事项时备注留空；待确认事项以‘待确认：’开头写备注；校验结果优先显示“待确认”。SIT/UAT适用由关联任务类型自动计算；灰色列为只读公式，请勿修改。</s:v>
       </s:c>
       <s:c r="B2" s="0"/>
       <s:c r="C2" s="0"/>
@@ -969,7 +969,7 @@
         <s:f>IF($C5="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C5,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J5" t="str" s="5">
-        <s:f>IF(COUNTA($A5:$C5,$D5:$E5)=0,"",IF(OR($A5="",$B5="",$C5="",$F5="",$G5="",$D5=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C5)&gt;1,"故事名称重复",IF(OR(AND($F5&lt;&gt;"是",$F5&lt;&gt;"否"),AND($G5&lt;&gt;"是",$G5&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C5)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A5:$C5,$D5:$E5)=0,"",IF(LEFT($E5,4)="待确认：","待确认",IF(OR($A5="",$B5="",$C5="",$F5="",$G5="",$D5=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C5)&gt;1,"故事名称重复",IF(OR(AND($F5&lt;&gt;"是",$F5&lt;&gt;"否"),AND($G5&lt;&gt;"是",$G5&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C5)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="6" ht="42" customHeight="1">
@@ -991,7 +991,7 @@
         <s:f>IF($C6="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C6,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J6" t="str" s="5">
-        <s:f>IF(COUNTA($A6:$C6,$D6:$E6)=0,"",IF(OR($A6="",$B6="",$C6="",$F6="",$G6="",$D6=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C6)&gt;1,"故事名称重复",IF(OR(AND($F6&lt;&gt;"是",$F6&lt;&gt;"否"),AND($G6&lt;&gt;"是",$G6&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C6)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A6:$C6,$D6:$E6)=0,"",IF(LEFT($E6,4)="待确认：","待确认",IF(OR($A6="",$B6="",$C6="",$F6="",$G6="",$D6=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C6)&gt;1,"故事名称重复",IF(OR(AND($F6&lt;&gt;"是",$F6&lt;&gt;"否"),AND($G6&lt;&gt;"是",$G6&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C6)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="7" ht="42" customHeight="1">
@@ -1013,7 +1013,7 @@
         <s:f>IF($C7="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C7,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J7" t="str" s="5">
-        <s:f>IF(COUNTA($A7:$C7,$D7:$E7)=0,"",IF(OR($A7="",$B7="",$C7="",$F7="",$G7="",$D7=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C7)&gt;1,"故事名称重复",IF(OR(AND($F7&lt;&gt;"是",$F7&lt;&gt;"否"),AND($G7&lt;&gt;"是",$G7&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C7)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A7:$C7,$D7:$E7)=0,"",IF(LEFT($E7,4)="待确认：","待确认",IF(OR($A7="",$B7="",$C7="",$F7="",$G7="",$D7=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C7)&gt;1,"故事名称重复",IF(OR(AND($F7&lt;&gt;"是",$F7&lt;&gt;"否"),AND($G7&lt;&gt;"是",$G7&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C7)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="8" ht="42" customHeight="1">
@@ -1035,7 +1035,7 @@
         <s:f>IF($C8="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C8,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J8" t="str" s="5">
-        <s:f>IF(COUNTA($A8:$C8,$D8:$E8)=0,"",IF(OR($A8="",$B8="",$C8="",$F8="",$G8="",$D8=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C8)&gt;1,"故事名称重复",IF(OR(AND($F8&lt;&gt;"是",$F8&lt;&gt;"否"),AND($G8&lt;&gt;"是",$G8&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C8)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A8:$C8,$D8:$E8)=0,"",IF(LEFT($E8,4)="待确认：","待确认",IF(OR($A8="",$B8="",$C8="",$F8="",$G8="",$D8=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C8)&gt;1,"故事名称重复",IF(OR(AND($F8&lt;&gt;"是",$F8&lt;&gt;"否"),AND($G8&lt;&gt;"是",$G8&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C8)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="9" ht="42" customHeight="1">
@@ -1057,7 +1057,7 @@
         <s:f>IF($C9="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C9,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J9" t="str" s="5">
-        <s:f>IF(COUNTA($A9:$C9,$D9:$E9)=0,"",IF(OR($A9="",$B9="",$C9="",$F9="",$G9="",$D9=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C9)&gt;1,"故事名称重复",IF(OR(AND($F9&lt;&gt;"是",$F9&lt;&gt;"否"),AND($G9&lt;&gt;"是",$G9&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C9)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A9:$C9,$D9:$E9)=0,"",IF(LEFT($E9,4)="待确认：","待确认",IF(OR($A9="",$B9="",$C9="",$F9="",$G9="",$D9=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C9)&gt;1,"故事名称重复",IF(OR(AND($F9&lt;&gt;"是",$F9&lt;&gt;"否"),AND($G9&lt;&gt;"是",$G9&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C9)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="10" ht="42" customHeight="1">
@@ -1079,7 +1079,7 @@
         <s:f>IF($C10="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C10,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J10" t="str" s="5">
-        <s:f>IF(COUNTA($A10:$C10,$D10:$E10)=0,"",IF(OR($A10="",$B10="",$C10="",$F10="",$G10="",$D10=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C10)&gt;1,"故事名称重复",IF(OR(AND($F10&lt;&gt;"是",$F10&lt;&gt;"否"),AND($G10&lt;&gt;"是",$G10&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C10)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A10:$C10,$D10:$E10)=0,"",IF(LEFT($E10,4)="待确认：","待确认",IF(OR($A10="",$B10="",$C10="",$F10="",$G10="",$D10=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C10)&gt;1,"故事名称重复",IF(OR(AND($F10&lt;&gt;"是",$F10&lt;&gt;"否"),AND($G10&lt;&gt;"是",$G10&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C10)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="11" ht="42" customHeight="1">
@@ -1101,7 +1101,7 @@
         <s:f>IF($C11="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C11,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J11" t="str" s="5">
-        <s:f>IF(COUNTA($A11:$C11,$D11:$E11)=0,"",IF(OR($A11="",$B11="",$C11="",$F11="",$G11="",$D11=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C11)&gt;1,"故事名称重复",IF(OR(AND($F11&lt;&gt;"是",$F11&lt;&gt;"否"),AND($G11&lt;&gt;"是",$G11&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C11)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A11:$C11,$D11:$E11)=0,"",IF(LEFT($E11,4)="待确认：","待确认",IF(OR($A11="",$B11="",$C11="",$F11="",$G11="",$D11=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C11)&gt;1,"故事名称重复",IF(OR(AND($F11&lt;&gt;"是",$F11&lt;&gt;"否"),AND($G11&lt;&gt;"是",$G11&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C11)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="12" ht="42" customHeight="1">
@@ -1123,7 +1123,7 @@
         <s:f>IF($C12="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C12,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J12" t="str" s="5">
-        <s:f>IF(COUNTA($A12:$C12,$D12:$E12)=0,"",IF(OR($A12="",$B12="",$C12="",$F12="",$G12="",$D12=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C12)&gt;1,"故事名称重复",IF(OR(AND($F12&lt;&gt;"是",$F12&lt;&gt;"否"),AND($G12&lt;&gt;"是",$G12&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C12)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A12:$C12,$D12:$E12)=0,"",IF(LEFT($E12,4)="待确认：","待确认",IF(OR($A12="",$B12="",$C12="",$F12="",$G12="",$D12=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C12)&gt;1,"故事名称重复",IF(OR(AND($F12&lt;&gt;"是",$F12&lt;&gt;"否"),AND($G12&lt;&gt;"是",$G12&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C12)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="13" ht="42" customHeight="1">
@@ -1145,7 +1145,7 @@
         <s:f>IF($C13="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C13,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J13" t="str" s="5">
-        <s:f>IF(COUNTA($A13:$C13,$D13:$E13)=0,"",IF(OR($A13="",$B13="",$C13="",$F13="",$G13="",$D13=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C13)&gt;1,"故事名称重复",IF(OR(AND($F13&lt;&gt;"是",$F13&lt;&gt;"否"),AND($G13&lt;&gt;"是",$G13&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C13)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A13:$C13,$D13:$E13)=0,"",IF(LEFT($E13,4)="待确认：","待确认",IF(OR($A13="",$B13="",$C13="",$F13="",$G13="",$D13=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C13)&gt;1,"故事名称重复",IF(OR(AND($F13&lt;&gt;"是",$F13&lt;&gt;"否"),AND($G13&lt;&gt;"是",$G13&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C13)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="14" ht="42" customHeight="1">
@@ -1167,7 +1167,7 @@
         <s:f>IF($C14="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C14,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J14" t="str" s="5">
-        <s:f>IF(COUNTA($A14:$C14,$D14:$E14)=0,"",IF(OR($A14="",$B14="",$C14="",$F14="",$G14="",$D14=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C14)&gt;1,"故事名称重复",IF(OR(AND($F14&lt;&gt;"是",$F14&lt;&gt;"否"),AND($G14&lt;&gt;"是",$G14&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C14)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A14:$C14,$D14:$E14)=0,"",IF(LEFT($E14,4)="待确认：","待确认",IF(OR($A14="",$B14="",$C14="",$F14="",$G14="",$D14=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C14)&gt;1,"故事名称重复",IF(OR(AND($F14&lt;&gt;"是",$F14&lt;&gt;"否"),AND($G14&lt;&gt;"是",$G14&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C14)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="15" ht="42" customHeight="1">
@@ -1189,7 +1189,7 @@
         <s:f>IF($C15="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C15,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J15" t="str" s="5">
-        <s:f>IF(COUNTA($A15:$C15,$D15:$E15)=0,"",IF(OR($A15="",$B15="",$C15="",$F15="",$G15="",$D15=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C15)&gt;1,"故事名称重复",IF(OR(AND($F15&lt;&gt;"是",$F15&lt;&gt;"否"),AND($G15&lt;&gt;"是",$G15&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C15)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A15:$C15,$D15:$E15)=0,"",IF(LEFT($E15,4)="待确认：","待确认",IF(OR($A15="",$B15="",$C15="",$F15="",$G15="",$D15=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C15)&gt;1,"故事名称重复",IF(OR(AND($F15&lt;&gt;"是",$F15&lt;&gt;"否"),AND($G15&lt;&gt;"是",$G15&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C15)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="16" ht="42" customHeight="1">
@@ -1211,7 +1211,7 @@
         <s:f>IF($C16="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C16,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J16" t="str" s="5">
-        <s:f>IF(COUNTA($A16:$C16,$D16:$E16)=0,"",IF(OR($A16="",$B16="",$C16="",$F16="",$G16="",$D16=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C16)&gt;1,"故事名称重复",IF(OR(AND($F16&lt;&gt;"是",$F16&lt;&gt;"否"),AND($G16&lt;&gt;"是",$G16&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C16)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A16:$C16,$D16:$E16)=0,"",IF(LEFT($E16,4)="待确认：","待确认",IF(OR($A16="",$B16="",$C16="",$F16="",$G16="",$D16=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C16)&gt;1,"故事名称重复",IF(OR(AND($F16&lt;&gt;"是",$F16&lt;&gt;"否"),AND($G16&lt;&gt;"是",$G16&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C16)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="17" ht="42" customHeight="1">
@@ -1233,7 +1233,7 @@
         <s:f>IF($C17="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C17,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J17" t="str" s="5">
-        <s:f>IF(COUNTA($A17:$C17,$D17:$E17)=0,"",IF(OR($A17="",$B17="",$C17="",$F17="",$G17="",$D17=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C17)&gt;1,"故事名称重复",IF(OR(AND($F17&lt;&gt;"是",$F17&lt;&gt;"否"),AND($G17&lt;&gt;"是",$G17&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C17)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A17:$C17,$D17:$E17)=0,"",IF(LEFT($E17,4)="待确认：","待确认",IF(OR($A17="",$B17="",$C17="",$F17="",$G17="",$D17=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C17)&gt;1,"故事名称重复",IF(OR(AND($F17&lt;&gt;"是",$F17&lt;&gt;"否"),AND($G17&lt;&gt;"是",$G17&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C17)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="18" ht="42" customHeight="1">
@@ -1255,7 +1255,7 @@
         <s:f>IF($C18="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C18,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J18" t="str" s="5">
-        <s:f>IF(COUNTA($A18:$C18,$D18:$E18)=0,"",IF(OR($A18="",$B18="",$C18="",$F18="",$G18="",$D18=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C18)&gt;1,"故事名称重复",IF(OR(AND($F18&lt;&gt;"是",$F18&lt;&gt;"否"),AND($G18&lt;&gt;"是",$G18&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C18)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A18:$C18,$D18:$E18)=0,"",IF(LEFT($E18,4)="待确认：","待确认",IF(OR($A18="",$B18="",$C18="",$F18="",$G18="",$D18=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C18)&gt;1,"故事名称重复",IF(OR(AND($F18&lt;&gt;"是",$F18&lt;&gt;"否"),AND($G18&lt;&gt;"是",$G18&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C18)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="19" ht="42" customHeight="1">
@@ -1277,7 +1277,7 @@
         <s:f>IF($C19="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C19,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J19" t="str" s="5">
-        <s:f>IF(COUNTA($A19:$C19,$D19:$E19)=0,"",IF(OR($A19="",$B19="",$C19="",$F19="",$G19="",$D19=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C19)&gt;1,"故事名称重复",IF(OR(AND($F19&lt;&gt;"是",$F19&lt;&gt;"否"),AND($G19&lt;&gt;"是",$G19&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C19)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A19:$C19,$D19:$E19)=0,"",IF(LEFT($E19,4)="待确认：","待确认",IF(OR($A19="",$B19="",$C19="",$F19="",$G19="",$D19=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C19)&gt;1,"故事名称重复",IF(OR(AND($F19&lt;&gt;"是",$F19&lt;&gt;"否"),AND($G19&lt;&gt;"是",$G19&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C19)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="20" ht="42" customHeight="1">
@@ -1299,7 +1299,7 @@
         <s:f>IF($C20="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C20,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J20" t="str" s="5">
-        <s:f>IF(COUNTA($A20:$C20,$D20:$E20)=0,"",IF(OR($A20="",$B20="",$C20="",$F20="",$G20="",$D20=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C20)&gt;1,"故事名称重复",IF(OR(AND($F20&lt;&gt;"是",$F20&lt;&gt;"否"),AND($G20&lt;&gt;"是",$G20&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C20)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A20:$C20,$D20:$E20)=0,"",IF(LEFT($E20,4)="待确认：","待确认",IF(OR($A20="",$B20="",$C20="",$F20="",$G20="",$D20=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C20)&gt;1,"故事名称重复",IF(OR(AND($F20&lt;&gt;"是",$F20&lt;&gt;"否"),AND($G20&lt;&gt;"是",$G20&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C20)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="21" ht="42" customHeight="1">
@@ -1321,7 +1321,7 @@
         <s:f>IF($C21="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C21,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J21" t="str" s="5">
-        <s:f>IF(COUNTA($A21:$C21,$D21:$E21)=0,"",IF(OR($A21="",$B21="",$C21="",$F21="",$G21="",$D21=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C21)&gt;1,"故事名称重复",IF(OR(AND($F21&lt;&gt;"是",$F21&lt;&gt;"否"),AND($G21&lt;&gt;"是",$G21&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C21)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A21:$C21,$D21:$E21)=0,"",IF(LEFT($E21,4)="待确认：","待确认",IF(OR($A21="",$B21="",$C21="",$F21="",$G21="",$D21=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C21)&gt;1,"故事名称重复",IF(OR(AND($F21&lt;&gt;"是",$F21&lt;&gt;"否"),AND($G21&lt;&gt;"是",$G21&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C21)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="22" ht="42" customHeight="1">
@@ -1343,7 +1343,7 @@
         <s:f>IF($C22="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C22,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J22" t="str" s="5">
-        <s:f>IF(COUNTA($A22:$C22,$D22:$E22)=0,"",IF(OR($A22="",$B22="",$C22="",$F22="",$G22="",$D22=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C22)&gt;1,"故事名称重复",IF(OR(AND($F22&lt;&gt;"是",$F22&lt;&gt;"否"),AND($G22&lt;&gt;"是",$G22&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C22)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A22:$C22,$D22:$E22)=0,"",IF(LEFT($E22,4)="待确认：","待确认",IF(OR($A22="",$B22="",$C22="",$F22="",$G22="",$D22=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C22)&gt;1,"故事名称重复",IF(OR(AND($F22&lt;&gt;"是",$F22&lt;&gt;"否"),AND($G22&lt;&gt;"是",$G22&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C22)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="23" ht="42" customHeight="1">
@@ -1365,7 +1365,7 @@
         <s:f>IF($C23="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C23,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J23" t="str" s="5">
-        <s:f>IF(COUNTA($A23:$C23,$D23:$E23)=0,"",IF(OR($A23="",$B23="",$C23="",$F23="",$G23="",$D23=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C23)&gt;1,"故事名称重复",IF(OR(AND($F23&lt;&gt;"是",$F23&lt;&gt;"否"),AND($G23&lt;&gt;"是",$G23&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C23)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A23:$C23,$D23:$E23)=0,"",IF(LEFT($E23,4)="待确认：","待确认",IF(OR($A23="",$B23="",$C23="",$F23="",$G23="",$D23=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C23)&gt;1,"故事名称重复",IF(OR(AND($F23&lt;&gt;"是",$F23&lt;&gt;"否"),AND($G23&lt;&gt;"是",$G23&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C23)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="24" ht="42" customHeight="1">
@@ -1387,7 +1387,7 @@
         <s:f>IF($C24="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C24,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J24" t="str" s="5">
-        <s:f>IF(COUNTA($A24:$C24,$D24:$E24)=0,"",IF(OR($A24="",$B24="",$C24="",$F24="",$G24="",$D24=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C24)&gt;1,"故事名称重复",IF(OR(AND($F24&lt;&gt;"是",$F24&lt;&gt;"否"),AND($G24&lt;&gt;"是",$G24&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C24)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A24:$C24,$D24:$E24)=0,"",IF(LEFT($E24,4)="待确认：","待确认",IF(OR($A24="",$B24="",$C24="",$F24="",$G24="",$D24=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C24)&gt;1,"故事名称重复",IF(OR(AND($F24&lt;&gt;"是",$F24&lt;&gt;"否"),AND($G24&lt;&gt;"是",$G24&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C24)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="25" ht="42" customHeight="1">
@@ -1409,7 +1409,7 @@
         <s:f>IF($C25="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C25,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J25" t="str" s="5">
-        <s:f>IF(COUNTA($A25:$C25,$D25:$E25)=0,"",IF(OR($A25="",$B25="",$C25="",$F25="",$G25="",$D25=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C25)&gt;1,"故事名称重复",IF(OR(AND($F25&lt;&gt;"是",$F25&lt;&gt;"否"),AND($G25&lt;&gt;"是",$G25&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C25)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A25:$C25,$D25:$E25)=0,"",IF(LEFT($E25,4)="待确认：","待确认",IF(OR($A25="",$B25="",$C25="",$F25="",$G25="",$D25=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C25)&gt;1,"故事名称重复",IF(OR(AND($F25&lt;&gt;"是",$F25&lt;&gt;"否"),AND($G25&lt;&gt;"是",$G25&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C25)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="26" ht="42" customHeight="1">
@@ -1431,7 +1431,7 @@
         <s:f>IF($C26="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C26,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J26" t="str" s="5">
-        <s:f>IF(COUNTA($A26:$C26,$D26:$E26)=0,"",IF(OR($A26="",$B26="",$C26="",$F26="",$G26="",$D26=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C26)&gt;1,"故事名称重复",IF(OR(AND($F26&lt;&gt;"是",$F26&lt;&gt;"否"),AND($G26&lt;&gt;"是",$G26&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C26)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A26:$C26,$D26:$E26)=0,"",IF(LEFT($E26,4)="待确认：","待确认",IF(OR($A26="",$B26="",$C26="",$F26="",$G26="",$D26=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C26)&gt;1,"故事名称重复",IF(OR(AND($F26&lt;&gt;"是",$F26&lt;&gt;"否"),AND($G26&lt;&gt;"是",$G26&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C26)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="27" ht="42" customHeight="1">
@@ -1453,7 +1453,7 @@
         <s:f>IF($C27="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C27,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J27" t="str" s="5">
-        <s:f>IF(COUNTA($A27:$C27,$D27:$E27)=0,"",IF(OR($A27="",$B27="",$C27="",$F27="",$G27="",$D27=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C27)&gt;1,"故事名称重复",IF(OR(AND($F27&lt;&gt;"是",$F27&lt;&gt;"否"),AND($G27&lt;&gt;"是",$G27&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C27)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A27:$C27,$D27:$E27)=0,"",IF(LEFT($E27,4)="待确认：","待确认",IF(OR($A27="",$B27="",$C27="",$F27="",$G27="",$D27=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C27)&gt;1,"故事名称重复",IF(OR(AND($F27&lt;&gt;"是",$F27&lt;&gt;"否"),AND($G27&lt;&gt;"是",$G27&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C27)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="28" ht="42" customHeight="1">
@@ -1475,7 +1475,7 @@
         <s:f>IF($C28="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C28,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J28" t="str" s="5">
-        <s:f>IF(COUNTA($A28:$C28,$D28:$E28)=0,"",IF(OR($A28="",$B28="",$C28="",$F28="",$G28="",$D28=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C28)&gt;1,"故事名称重复",IF(OR(AND($F28&lt;&gt;"是",$F28&lt;&gt;"否"),AND($G28&lt;&gt;"是",$G28&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C28)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A28:$C28,$D28:$E28)=0,"",IF(LEFT($E28,4)="待确认：","待确认",IF(OR($A28="",$B28="",$C28="",$F28="",$G28="",$D28=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C28)&gt;1,"故事名称重复",IF(OR(AND($F28&lt;&gt;"是",$F28&lt;&gt;"否"),AND($G28&lt;&gt;"是",$G28&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C28)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="29" ht="42" customHeight="1">
@@ -1497,7 +1497,7 @@
         <s:f>IF($C29="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C29,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J29" t="str" s="5">
-        <s:f>IF(COUNTA($A29:$C29,$D29:$E29)=0,"",IF(OR($A29="",$B29="",$C29="",$F29="",$G29="",$D29=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C29)&gt;1,"故事名称重复",IF(OR(AND($F29&lt;&gt;"是",$F29&lt;&gt;"否"),AND($G29&lt;&gt;"是",$G29&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C29)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A29:$C29,$D29:$E29)=0,"",IF(LEFT($E29,4)="待确认：","待确认",IF(OR($A29="",$B29="",$C29="",$F29="",$G29="",$D29=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C29)&gt;1,"故事名称重复",IF(OR(AND($F29&lt;&gt;"是",$F29&lt;&gt;"否"),AND($G29&lt;&gt;"是",$G29&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C29)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="30" ht="42" customHeight="1">
@@ -1519,7 +1519,7 @@
         <s:f>IF($C30="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C30,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J30" t="str" s="5">
-        <s:f>IF(COUNTA($A30:$C30,$D30:$E30)=0,"",IF(OR($A30="",$B30="",$C30="",$F30="",$G30="",$D30=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C30)&gt;1,"故事名称重复",IF(OR(AND($F30&lt;&gt;"是",$F30&lt;&gt;"否"),AND($G30&lt;&gt;"是",$G30&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C30)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A30:$C30,$D30:$E30)=0,"",IF(LEFT($E30,4)="待确认：","待确认",IF(OR($A30="",$B30="",$C30="",$F30="",$G30="",$D30=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C30)&gt;1,"故事名称重复",IF(OR(AND($F30&lt;&gt;"是",$F30&lt;&gt;"否"),AND($G30&lt;&gt;"是",$G30&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C30)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="31" ht="42" customHeight="1">
@@ -1541,7 +1541,7 @@
         <s:f>IF($C31="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C31,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J31" t="str" s="5">
-        <s:f>IF(COUNTA($A31:$C31,$D31:$E31)=0,"",IF(OR($A31="",$B31="",$C31="",$F31="",$G31="",$D31=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C31)&gt;1,"故事名称重复",IF(OR(AND($F31&lt;&gt;"是",$F31&lt;&gt;"否"),AND($G31&lt;&gt;"是",$G31&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C31)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A31:$C31,$D31:$E31)=0,"",IF(LEFT($E31,4)="待确认：","待确认",IF(OR($A31="",$B31="",$C31="",$F31="",$G31="",$D31=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C31)&gt;1,"故事名称重复",IF(OR(AND($F31&lt;&gt;"是",$F31&lt;&gt;"否"),AND($G31&lt;&gt;"是",$G31&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C31)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="32" ht="42" customHeight="1">
@@ -1563,7 +1563,7 @@
         <s:f>IF($C32="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C32,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J32" t="str" s="5">
-        <s:f>IF(COUNTA($A32:$C32,$D32:$E32)=0,"",IF(OR($A32="",$B32="",$C32="",$F32="",$G32="",$D32=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C32)&gt;1,"故事名称重复",IF(OR(AND($F32&lt;&gt;"是",$F32&lt;&gt;"否"),AND($G32&lt;&gt;"是",$G32&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C32)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A32:$C32,$D32:$E32)=0,"",IF(LEFT($E32,4)="待确认：","待确认",IF(OR($A32="",$B32="",$C32="",$F32="",$G32="",$D32=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C32)&gt;1,"故事名称重复",IF(OR(AND($F32&lt;&gt;"是",$F32&lt;&gt;"否"),AND($G32&lt;&gt;"是",$G32&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C32)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="33" ht="42" customHeight="1">
@@ -1585,7 +1585,7 @@
         <s:f>IF($C33="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C33,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J33" t="str" s="5">
-        <s:f>IF(COUNTA($A33:$C33,$D33:$E33)=0,"",IF(OR($A33="",$B33="",$C33="",$F33="",$G33="",$D33=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C33)&gt;1,"故事名称重复",IF(OR(AND($F33&lt;&gt;"是",$F33&lt;&gt;"否"),AND($G33&lt;&gt;"是",$G33&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C33)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A33:$C33,$D33:$E33)=0,"",IF(LEFT($E33,4)="待确认：","待确认",IF(OR($A33="",$B33="",$C33="",$F33="",$G33="",$D33=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C33)&gt;1,"故事名称重复",IF(OR(AND($F33&lt;&gt;"是",$F33&lt;&gt;"否"),AND($G33&lt;&gt;"是",$G33&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C33)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="34" ht="42" customHeight="1">
@@ -1607,7 +1607,7 @@
         <s:f>IF($C34="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C34,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J34" t="str" s="5">
-        <s:f>IF(COUNTA($A34:$C34,$D34:$E34)=0,"",IF(OR($A34="",$B34="",$C34="",$F34="",$G34="",$D34=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C34)&gt;1,"故事名称重复",IF(OR(AND($F34&lt;&gt;"是",$F34&lt;&gt;"否"),AND($G34&lt;&gt;"是",$G34&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C34)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A34:$C34,$D34:$E34)=0,"",IF(LEFT($E34,4)="待确认：","待确认",IF(OR($A34="",$B34="",$C34="",$F34="",$G34="",$D34=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C34)&gt;1,"故事名称重复",IF(OR(AND($F34&lt;&gt;"是",$F34&lt;&gt;"否"),AND($G34&lt;&gt;"是",$G34&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C34)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="35" ht="42" customHeight="1">
@@ -1629,7 +1629,7 @@
         <s:f>IF($C35="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C35,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J35" t="str" s="5">
-        <s:f>IF(COUNTA($A35:$C35,$D35:$E35)=0,"",IF(OR($A35="",$B35="",$C35="",$F35="",$G35="",$D35=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C35)&gt;1,"故事名称重复",IF(OR(AND($F35&lt;&gt;"是",$F35&lt;&gt;"否"),AND($G35&lt;&gt;"是",$G35&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C35)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A35:$C35,$D35:$E35)=0,"",IF(LEFT($E35,4)="待确认：","待确认",IF(OR($A35="",$B35="",$C35="",$F35="",$G35="",$D35=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C35)&gt;1,"故事名称重复",IF(OR(AND($F35&lt;&gt;"是",$F35&lt;&gt;"否"),AND($G35&lt;&gt;"是",$G35&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C35)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="36" ht="42" customHeight="1">
@@ -1651,7 +1651,7 @@
         <s:f>IF($C36="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C36,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J36" t="str" s="5">
-        <s:f>IF(COUNTA($A36:$C36,$D36:$E36)=0,"",IF(OR($A36="",$B36="",$C36="",$F36="",$G36="",$D36=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C36)&gt;1,"故事名称重复",IF(OR(AND($F36&lt;&gt;"是",$F36&lt;&gt;"否"),AND($G36&lt;&gt;"是",$G36&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C36)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A36:$C36,$D36:$E36)=0,"",IF(LEFT($E36,4)="待确认：","待确认",IF(OR($A36="",$B36="",$C36="",$F36="",$G36="",$D36=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C36)&gt;1,"故事名称重复",IF(OR(AND($F36&lt;&gt;"是",$F36&lt;&gt;"否"),AND($G36&lt;&gt;"是",$G36&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C36)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="37" ht="42" customHeight="1">
@@ -1673,7 +1673,7 @@
         <s:f>IF($C37="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C37,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J37" t="str" s="5">
-        <s:f>IF(COUNTA($A37:$C37,$D37:$E37)=0,"",IF(OR($A37="",$B37="",$C37="",$F37="",$G37="",$D37=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C37)&gt;1,"故事名称重复",IF(OR(AND($F37&lt;&gt;"是",$F37&lt;&gt;"否"),AND($G37&lt;&gt;"是",$G37&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C37)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A37:$C37,$D37:$E37)=0,"",IF(LEFT($E37,4)="待确认：","待确认",IF(OR($A37="",$B37="",$C37="",$F37="",$G37="",$D37=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C37)&gt;1,"故事名称重复",IF(OR(AND($F37&lt;&gt;"是",$F37&lt;&gt;"否"),AND($G37&lt;&gt;"是",$G37&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C37)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="38" ht="42" customHeight="1">
@@ -1695,7 +1695,7 @@
         <s:f>IF($C38="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C38,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J38" t="str" s="5">
-        <s:f>IF(COUNTA($A38:$C38,$D38:$E38)=0,"",IF(OR($A38="",$B38="",$C38="",$F38="",$G38="",$D38=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C38)&gt;1,"故事名称重复",IF(OR(AND($F38&lt;&gt;"是",$F38&lt;&gt;"否"),AND($G38&lt;&gt;"是",$G38&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C38)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A38:$C38,$D38:$E38)=0,"",IF(LEFT($E38,4)="待确认：","待确认",IF(OR($A38="",$B38="",$C38="",$F38="",$G38="",$D38=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C38)&gt;1,"故事名称重复",IF(OR(AND($F38&lt;&gt;"是",$F38&lt;&gt;"否"),AND($G38&lt;&gt;"是",$G38&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C38)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="39" ht="42" customHeight="1">
@@ -1717,7 +1717,7 @@
         <s:f>IF($C39="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C39,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J39" t="str" s="5">
-        <s:f>IF(COUNTA($A39:$C39,$D39:$E39)=0,"",IF(OR($A39="",$B39="",$C39="",$F39="",$G39="",$D39=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C39)&gt;1,"故事名称重复",IF(OR(AND($F39&lt;&gt;"是",$F39&lt;&gt;"否"),AND($G39&lt;&gt;"是",$G39&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C39)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A39:$C39,$D39:$E39)=0,"",IF(LEFT($E39,4)="待确认：","待确认",IF(OR($A39="",$B39="",$C39="",$F39="",$G39="",$D39=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C39)&gt;1,"故事名称重复",IF(OR(AND($F39&lt;&gt;"是",$F39&lt;&gt;"否"),AND($G39&lt;&gt;"是",$G39&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C39)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="40" ht="42" customHeight="1">
@@ -1739,7 +1739,7 @@
         <s:f>IF($C40="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C40,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J40" t="str" s="5">
-        <s:f>IF(COUNTA($A40:$C40,$D40:$E40)=0,"",IF(OR($A40="",$B40="",$C40="",$F40="",$G40="",$D40=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C40)&gt;1,"故事名称重复",IF(OR(AND($F40&lt;&gt;"是",$F40&lt;&gt;"否"),AND($G40&lt;&gt;"是",$G40&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C40)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A40:$C40,$D40:$E40)=0,"",IF(LEFT($E40,4)="待确认：","待确认",IF(OR($A40="",$B40="",$C40="",$F40="",$G40="",$D40=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C40)&gt;1,"故事名称重复",IF(OR(AND($F40&lt;&gt;"是",$F40&lt;&gt;"否"),AND($G40&lt;&gt;"是",$G40&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C40)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="41" ht="42" customHeight="1">
@@ -1761,7 +1761,7 @@
         <s:f>IF($C41="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C41,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J41" t="str" s="5">
-        <s:f>IF(COUNTA($A41:$C41,$D41:$E41)=0,"",IF(OR($A41="",$B41="",$C41="",$F41="",$G41="",$D41=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C41)&gt;1,"故事名称重复",IF(OR(AND($F41&lt;&gt;"是",$F41&lt;&gt;"否"),AND($G41&lt;&gt;"是",$G41&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C41)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A41:$C41,$D41:$E41)=0,"",IF(LEFT($E41,4)="待确认：","待确认",IF(OR($A41="",$B41="",$C41="",$F41="",$G41="",$D41=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C41)&gt;1,"故事名称重复",IF(OR(AND($F41&lt;&gt;"是",$F41&lt;&gt;"否"),AND($G41&lt;&gt;"是",$G41&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C41)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="42" ht="42" customHeight="1">
@@ -1783,7 +1783,7 @@
         <s:f>IF($C42="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C42,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J42" t="str" s="5">
-        <s:f>IF(COUNTA($A42:$C42,$D42:$E42)=0,"",IF(OR($A42="",$B42="",$C42="",$F42="",$G42="",$D42=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C42)&gt;1,"故事名称重复",IF(OR(AND($F42&lt;&gt;"是",$F42&lt;&gt;"否"),AND($G42&lt;&gt;"是",$G42&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C42)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A42:$C42,$D42:$E42)=0,"",IF(LEFT($E42,4)="待确认：","待确认",IF(OR($A42="",$B42="",$C42="",$F42="",$G42="",$D42=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C42)&gt;1,"故事名称重复",IF(OR(AND($F42&lt;&gt;"是",$F42&lt;&gt;"否"),AND($G42&lt;&gt;"是",$G42&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C42)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="43" ht="42" customHeight="1">
@@ -1805,7 +1805,7 @@
         <s:f>IF($C43="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C43,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J43" t="str" s="5">
-        <s:f>IF(COUNTA($A43:$C43,$D43:$E43)=0,"",IF(OR($A43="",$B43="",$C43="",$F43="",$G43="",$D43=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C43)&gt;1,"故事名称重复",IF(OR(AND($F43&lt;&gt;"是",$F43&lt;&gt;"否"),AND($G43&lt;&gt;"是",$G43&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C43)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A43:$C43,$D43:$E43)=0,"",IF(LEFT($E43,4)="待确认：","待确认",IF(OR($A43="",$B43="",$C43="",$F43="",$G43="",$D43=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C43)&gt;1,"故事名称重复",IF(OR(AND($F43&lt;&gt;"是",$F43&lt;&gt;"否"),AND($G43&lt;&gt;"是",$G43&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C43)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="44" ht="42" customHeight="1">
@@ -1827,7 +1827,7 @@
         <s:f>IF($C44="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C44,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J44" t="str" s="5">
-        <s:f>IF(COUNTA($A44:$C44,$D44:$E44)=0,"",IF(OR($A44="",$B44="",$C44="",$F44="",$G44="",$D44=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C44)&gt;1,"故事名称重复",IF(OR(AND($F44&lt;&gt;"是",$F44&lt;&gt;"否"),AND($G44&lt;&gt;"是",$G44&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C44)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A44:$C44,$D44:$E44)=0,"",IF(LEFT($E44,4)="待确认：","待确认",IF(OR($A44="",$B44="",$C44="",$F44="",$G44="",$D44=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C44)&gt;1,"故事名称重复",IF(OR(AND($F44&lt;&gt;"是",$F44&lt;&gt;"否"),AND($G44&lt;&gt;"是",$G44&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C44)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="45" ht="42" customHeight="1">
@@ -1849,7 +1849,7 @@
         <s:f>IF($C45="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C45,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J45" t="str" s="5">
-        <s:f>IF(COUNTA($A45:$C45,$D45:$E45)=0,"",IF(OR($A45="",$B45="",$C45="",$F45="",$G45="",$D45=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C45)&gt;1,"故事名称重复",IF(OR(AND($F45&lt;&gt;"是",$F45&lt;&gt;"否"),AND($G45&lt;&gt;"是",$G45&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C45)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A45:$C45,$D45:$E45)=0,"",IF(LEFT($E45,4)="待确认：","待确认",IF(OR($A45="",$B45="",$C45="",$F45="",$G45="",$D45=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C45)&gt;1,"故事名称重复",IF(OR(AND($F45&lt;&gt;"是",$F45&lt;&gt;"否"),AND($G45&lt;&gt;"是",$G45&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C45)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="46" ht="42" customHeight="1">
@@ -1871,7 +1871,7 @@
         <s:f>IF($C46="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C46,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J46" t="str" s="5">
-        <s:f>IF(COUNTA($A46:$C46,$D46:$E46)=0,"",IF(OR($A46="",$B46="",$C46="",$F46="",$G46="",$D46=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C46)&gt;1,"故事名称重复",IF(OR(AND($F46&lt;&gt;"是",$F46&lt;&gt;"否"),AND($G46&lt;&gt;"是",$G46&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C46)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A46:$C46,$D46:$E46)=0,"",IF(LEFT($E46,4)="待确认：","待确认",IF(OR($A46="",$B46="",$C46="",$F46="",$G46="",$D46=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C46)&gt;1,"故事名称重复",IF(OR(AND($F46&lt;&gt;"是",$F46&lt;&gt;"否"),AND($G46&lt;&gt;"是",$G46&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C46)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="47" ht="42" customHeight="1">
@@ -1893,7 +1893,7 @@
         <s:f>IF($C47="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C47,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J47" t="str" s="5">
-        <s:f>IF(COUNTA($A47:$C47,$D47:$E47)=0,"",IF(OR($A47="",$B47="",$C47="",$F47="",$G47="",$D47=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C47)&gt;1,"故事名称重复",IF(OR(AND($F47&lt;&gt;"是",$F47&lt;&gt;"否"),AND($G47&lt;&gt;"是",$G47&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C47)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A47:$C47,$D47:$E47)=0,"",IF(LEFT($E47,4)="待确认：","待确认",IF(OR($A47="",$B47="",$C47="",$F47="",$G47="",$D47=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C47)&gt;1,"故事名称重复",IF(OR(AND($F47&lt;&gt;"是",$F47&lt;&gt;"否"),AND($G47&lt;&gt;"是",$G47&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C47)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="48" ht="42" customHeight="1">
@@ -1915,7 +1915,7 @@
         <s:f>IF($C48="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C48,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J48" t="str" s="5">
-        <s:f>IF(COUNTA($A48:$C48,$D48:$E48)=0,"",IF(OR($A48="",$B48="",$C48="",$F48="",$G48="",$D48=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C48)&gt;1,"故事名称重复",IF(OR(AND($F48&lt;&gt;"是",$F48&lt;&gt;"否"),AND($G48&lt;&gt;"是",$G48&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C48)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A48:$C48,$D48:$E48)=0,"",IF(LEFT($E48,4)="待确认：","待确认",IF(OR($A48="",$B48="",$C48="",$F48="",$G48="",$D48=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C48)&gt;1,"故事名称重复",IF(OR(AND($F48&lt;&gt;"是",$F48&lt;&gt;"否"),AND($G48&lt;&gt;"是",$G48&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C48)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="49" ht="42" customHeight="1">
@@ -1937,7 +1937,7 @@
         <s:f>IF($C49="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C49,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J49" t="str" s="5">
-        <s:f>IF(COUNTA($A49:$C49,$D49:$E49)=0,"",IF(OR($A49="",$B49="",$C49="",$F49="",$G49="",$D49=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C49)&gt;1,"故事名称重复",IF(OR(AND($F49&lt;&gt;"是",$F49&lt;&gt;"否"),AND($G49&lt;&gt;"是",$G49&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C49)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A49:$C49,$D49:$E49)=0,"",IF(LEFT($E49,4)="待确认：","待确认",IF(OR($A49="",$B49="",$C49="",$F49="",$G49="",$D49=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C49)&gt;1,"故事名称重复",IF(OR(AND($F49&lt;&gt;"是",$F49&lt;&gt;"否"),AND($G49&lt;&gt;"是",$G49&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C49)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="50" ht="42" customHeight="1">
@@ -1959,7 +1959,7 @@
         <s:f>IF($C50="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C50,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J50" t="str" s="5">
-        <s:f>IF(COUNTA($A50:$C50,$D50:$E50)=0,"",IF(OR($A50="",$B50="",$C50="",$F50="",$G50="",$D50=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C50)&gt;1,"故事名称重复",IF(OR(AND($F50&lt;&gt;"是",$F50&lt;&gt;"否"),AND($G50&lt;&gt;"是",$G50&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C50)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A50:$C50,$D50:$E50)=0,"",IF(LEFT($E50,4)="待确认：","待确认",IF(OR($A50="",$B50="",$C50="",$F50="",$G50="",$D50=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C50)&gt;1,"故事名称重复",IF(OR(AND($F50&lt;&gt;"是",$F50&lt;&gt;"否"),AND($G50&lt;&gt;"是",$G50&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C50)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="51" ht="42" customHeight="1">
@@ -1981,7 +1981,7 @@
         <s:f>IF($C51="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C51,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J51" t="str" s="5">
-        <s:f>IF(COUNTA($A51:$C51,$D51:$E51)=0,"",IF(OR($A51="",$B51="",$C51="",$F51="",$G51="",$D51=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C51)&gt;1,"故事名称重复",IF(OR(AND($F51&lt;&gt;"是",$F51&lt;&gt;"否"),AND($G51&lt;&gt;"是",$G51&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C51)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A51:$C51,$D51:$E51)=0,"",IF(LEFT($E51,4)="待确认：","待确认",IF(OR($A51="",$B51="",$C51="",$F51="",$G51="",$D51=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C51)&gt;1,"故事名称重复",IF(OR(AND($F51&lt;&gt;"是",$F51&lt;&gt;"否"),AND($G51&lt;&gt;"是",$G51&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C51)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="52" ht="42" customHeight="1">
@@ -2003,7 +2003,7 @@
         <s:f>IF($C52="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C52,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J52" t="str" s="5">
-        <s:f>IF(COUNTA($A52:$C52,$D52:$E52)=0,"",IF(OR($A52="",$B52="",$C52="",$F52="",$G52="",$D52=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C52)&gt;1,"故事名称重复",IF(OR(AND($F52&lt;&gt;"是",$F52&lt;&gt;"否"),AND($G52&lt;&gt;"是",$G52&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C52)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A52:$C52,$D52:$E52)=0,"",IF(LEFT($E52,4)="待确认：","待确认",IF(OR($A52="",$B52="",$C52="",$F52="",$G52="",$D52=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C52)&gt;1,"故事名称重复",IF(OR(AND($F52&lt;&gt;"是",$F52&lt;&gt;"否"),AND($G52&lt;&gt;"是",$G52&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C52)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="53" ht="42" customHeight="1">
@@ -2025,7 +2025,7 @@
         <s:f>IF($C53="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C53,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J53" t="str" s="5">
-        <s:f>IF(COUNTA($A53:$C53,$D53:$E53)=0,"",IF(OR($A53="",$B53="",$C53="",$F53="",$G53="",$D53=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C53)&gt;1,"故事名称重复",IF(OR(AND($F53&lt;&gt;"是",$F53&lt;&gt;"否"),AND($G53&lt;&gt;"是",$G53&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C53)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A53:$C53,$D53:$E53)=0,"",IF(LEFT($E53,4)="待确认：","待确认",IF(OR($A53="",$B53="",$C53="",$F53="",$G53="",$D53=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C53)&gt;1,"故事名称重复",IF(OR(AND($F53&lt;&gt;"是",$F53&lt;&gt;"否"),AND($G53&lt;&gt;"是",$G53&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C53)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="54" ht="42" customHeight="1">
@@ -2047,7 +2047,7 @@
         <s:f>IF($C54="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C54,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J54" t="str" s="5">
-        <s:f>IF(COUNTA($A54:$C54,$D54:$E54)=0,"",IF(OR($A54="",$B54="",$C54="",$F54="",$G54="",$D54=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C54)&gt;1,"故事名称重复",IF(OR(AND($F54&lt;&gt;"是",$F54&lt;&gt;"否"),AND($G54&lt;&gt;"是",$G54&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C54)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A54:$C54,$D54:$E54)=0,"",IF(LEFT($E54,4)="待确认：","待确认",IF(OR($A54="",$B54="",$C54="",$F54="",$G54="",$D54=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C54)&gt;1,"故事名称重复",IF(OR(AND($F54&lt;&gt;"是",$F54&lt;&gt;"否"),AND($G54&lt;&gt;"是",$G54&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C54)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="55" ht="42" customHeight="1">
@@ -2069,7 +2069,7 @@
         <s:f>IF($C55="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C55,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J55" t="str" s="5">
-        <s:f>IF(COUNTA($A55:$C55,$D55:$E55)=0,"",IF(OR($A55="",$B55="",$C55="",$F55="",$G55="",$D55=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C55)&gt;1,"故事名称重复",IF(OR(AND($F55&lt;&gt;"是",$F55&lt;&gt;"否"),AND($G55&lt;&gt;"是",$G55&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C55)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A55:$C55,$D55:$E55)=0,"",IF(LEFT($E55,4)="待确认：","待确认",IF(OR($A55="",$B55="",$C55="",$F55="",$G55="",$D55=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C55)&gt;1,"故事名称重复",IF(OR(AND($F55&lt;&gt;"是",$F55&lt;&gt;"否"),AND($G55&lt;&gt;"是",$G55&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C55)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="56" ht="42" customHeight="1">
@@ -2091,7 +2091,7 @@
         <s:f>IF($C56="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C56,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J56" t="str" s="5">
-        <s:f>IF(COUNTA($A56:$C56,$D56:$E56)=0,"",IF(OR($A56="",$B56="",$C56="",$F56="",$G56="",$D56=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C56)&gt;1,"故事名称重复",IF(OR(AND($F56&lt;&gt;"是",$F56&lt;&gt;"否"),AND($G56&lt;&gt;"是",$G56&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C56)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A56:$C56,$D56:$E56)=0,"",IF(LEFT($E56,4)="待确认：","待确认",IF(OR($A56="",$B56="",$C56="",$F56="",$G56="",$D56=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C56)&gt;1,"故事名称重复",IF(OR(AND($F56&lt;&gt;"是",$F56&lt;&gt;"否"),AND($G56&lt;&gt;"是",$G56&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C56)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="57" ht="42" customHeight="1">
@@ -2113,7 +2113,7 @@
         <s:f>IF($C57="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C57,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J57" t="str" s="5">
-        <s:f>IF(COUNTA($A57:$C57,$D57:$E57)=0,"",IF(OR($A57="",$B57="",$C57="",$F57="",$G57="",$D57=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C57)&gt;1,"故事名称重复",IF(OR(AND($F57&lt;&gt;"是",$F57&lt;&gt;"否"),AND($G57&lt;&gt;"是",$G57&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C57)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A57:$C57,$D57:$E57)=0,"",IF(LEFT($E57,4)="待确认：","待确认",IF(OR($A57="",$B57="",$C57="",$F57="",$G57="",$D57=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C57)&gt;1,"故事名称重复",IF(OR(AND($F57&lt;&gt;"是",$F57&lt;&gt;"否"),AND($G57&lt;&gt;"是",$G57&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C57)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="58" ht="42" customHeight="1">
@@ -2135,7 +2135,7 @@
         <s:f>IF($C58="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C58,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J58" t="str" s="5">
-        <s:f>IF(COUNTA($A58:$C58,$D58:$E58)=0,"",IF(OR($A58="",$B58="",$C58="",$F58="",$G58="",$D58=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C58)&gt;1,"故事名称重复",IF(OR(AND($F58&lt;&gt;"是",$F58&lt;&gt;"否"),AND($G58&lt;&gt;"是",$G58&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C58)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A58:$C58,$D58:$E58)=0,"",IF(LEFT($E58,4)="待确认：","待确认",IF(OR($A58="",$B58="",$C58="",$F58="",$G58="",$D58=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C58)&gt;1,"故事名称重复",IF(OR(AND($F58&lt;&gt;"是",$F58&lt;&gt;"否"),AND($G58&lt;&gt;"是",$G58&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C58)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="59" ht="42" customHeight="1">
@@ -2157,7 +2157,7 @@
         <s:f>IF($C59="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C59,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J59" t="str" s="5">
-        <s:f>IF(COUNTA($A59:$C59,$D59:$E59)=0,"",IF(OR($A59="",$B59="",$C59="",$F59="",$G59="",$D59=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C59)&gt;1,"故事名称重复",IF(OR(AND($F59&lt;&gt;"是",$F59&lt;&gt;"否"),AND($G59&lt;&gt;"是",$G59&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C59)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A59:$C59,$D59:$E59)=0,"",IF(LEFT($E59,4)="待确认：","待确认",IF(OR($A59="",$B59="",$C59="",$F59="",$G59="",$D59=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C59)&gt;1,"故事名称重复",IF(OR(AND($F59&lt;&gt;"是",$F59&lt;&gt;"否"),AND($G59&lt;&gt;"是",$G59&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C59)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="60" ht="42" customHeight="1">
@@ -2179,7 +2179,7 @@
         <s:f>IF($C60="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C60,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J60" t="str" s="5">
-        <s:f>IF(COUNTA($A60:$C60,$D60:$E60)=0,"",IF(OR($A60="",$B60="",$C60="",$F60="",$G60="",$D60=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C60)&gt;1,"故事名称重复",IF(OR(AND($F60&lt;&gt;"是",$F60&lt;&gt;"否"),AND($G60&lt;&gt;"是",$G60&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C60)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A60:$C60,$D60:$E60)=0,"",IF(LEFT($E60,4)="待确认：","待确认",IF(OR($A60="",$B60="",$C60="",$F60="",$G60="",$D60=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C60)&gt;1,"故事名称重复",IF(OR(AND($F60&lt;&gt;"是",$F60&lt;&gt;"否"),AND($G60&lt;&gt;"是",$G60&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C60)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="61" ht="42" customHeight="1">
@@ -2201,7 +2201,7 @@
         <s:f>IF($C61="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C61,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J61" t="str" s="5">
-        <s:f>IF(COUNTA($A61:$C61,$D61:$E61)=0,"",IF(OR($A61="",$B61="",$C61="",$F61="",$G61="",$D61=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C61)&gt;1,"故事名称重复",IF(OR(AND($F61&lt;&gt;"是",$F61&lt;&gt;"否"),AND($G61&lt;&gt;"是",$G61&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C61)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A61:$C61,$D61:$E61)=0,"",IF(LEFT($E61,4)="待确认：","待确认",IF(OR($A61="",$B61="",$C61="",$F61="",$G61="",$D61=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C61)&gt;1,"故事名称重复",IF(OR(AND($F61&lt;&gt;"是",$F61&lt;&gt;"否"),AND($G61&lt;&gt;"是",$G61&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C61)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="62" ht="42" customHeight="1">
@@ -2223,7 +2223,7 @@
         <s:f>IF($C62="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C62,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J62" t="str" s="5">
-        <s:f>IF(COUNTA($A62:$C62,$D62:$E62)=0,"",IF(OR($A62="",$B62="",$C62="",$F62="",$G62="",$D62=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C62)&gt;1,"故事名称重复",IF(OR(AND($F62&lt;&gt;"是",$F62&lt;&gt;"否"),AND($G62&lt;&gt;"是",$G62&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C62)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A62:$C62,$D62:$E62)=0,"",IF(LEFT($E62,4)="待确认：","待确认",IF(OR($A62="",$B62="",$C62="",$F62="",$G62="",$D62=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C62)&gt;1,"故事名称重复",IF(OR(AND($F62&lt;&gt;"是",$F62&lt;&gt;"否"),AND($G62&lt;&gt;"是",$G62&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C62)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="63" ht="42" customHeight="1">
@@ -2245,7 +2245,7 @@
         <s:f>IF($C63="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C63,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J63" t="str" s="5">
-        <s:f>IF(COUNTA($A63:$C63,$D63:$E63)=0,"",IF(OR($A63="",$B63="",$C63="",$F63="",$G63="",$D63=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C63)&gt;1,"故事名称重复",IF(OR(AND($F63&lt;&gt;"是",$F63&lt;&gt;"否"),AND($G63&lt;&gt;"是",$G63&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C63)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A63:$C63,$D63:$E63)=0,"",IF(LEFT($E63,4)="待确认：","待确认",IF(OR($A63="",$B63="",$C63="",$F63="",$G63="",$D63=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C63)&gt;1,"故事名称重复",IF(OR(AND($F63&lt;&gt;"是",$F63&lt;&gt;"否"),AND($G63&lt;&gt;"是",$G63&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C63)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="64" ht="42" customHeight="1">
@@ -2267,7 +2267,7 @@
         <s:f>IF($C64="","",CEILING(SUMIFS(TaskTable[任务人天],TaskTable[所属故事],"="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE($C64,"~","~~"),"*","~*"),"?","~?")),INDEX(ProjectParameterTable[当前值],MATCH("故事取整粒度",ProjectParameterTable[参数名称],0))))</s:f>
       </s:c>
       <s:c r="J64" t="str" s="5">
-        <s:f>IF(COUNTA($A64:$C64,$D64:$E64)=0,"",IF(OR($A64="",$B64="",$C64="",$F64="",$G64="",$D64=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C64)&gt;1,"故事名称重复",IF(OR(AND($F64&lt;&gt;"是",$F64&lt;&gt;"否"),AND($G64&lt;&gt;"是",$G64&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C64)=0,"故事缺少任务","通过")))))</s:f>
+        <s:f>IF(COUNTA($A64:$C64,$D64:$E64)=0,"",IF(LEFT($E64,4)="待确认：","待确认",IF(OR($A64="",$B64="",$C64="",$F64="",$G64="",$D64=""),"必填项缺失",IF(COUNTIF(SOWStoryTable[故事],$C64)&gt;1,"故事名称重复",IF(OR(AND($F64&lt;&gt;"是",$F64&lt;&gt;"否"),AND($G64&lt;&gt;"是",$G64&lt;&gt;"否")),"SIT/UAT适用值非法",IF(COUNTIF(TaskTable[所属故事],$C64)=0,"故事缺少任务","通过"))))))</s:f>
       </s:c>
     </s:row>
   </s:sheetData>
@@ -2335,7 +2335,7 @@
     </s:row>
     <s:row r="2" ht="34" customHeight="1">
       <s:c r="A2" t="str" s="2">
-        <s:v>工作类型按名称选择，任务名称全表唯一。仅集成类任务选择内部集成或外部集成，其他任务留空；SIT 按该集成任务计取。灰色计算列由公式维护。</s:v>
+        <s:v>工作类型按名称选择，任务名称全表唯一。仅集成类任务选择内部集成或外部集成，其他任务留空；SIT 按该集成任务计取。无待确认事项时备注留空；待确认事项以‘待确认：’开头写备注；校验结果优先显示“待确认”。灰色计算列由公式维护。</s:v>
       </s:c>
       <s:c r="B2" s="0"/>
       <s:c r="C2" s="0"/>
@@ -2422,7 +2422,7 @@
         <s:f>IF(COUNTA($A5:$G5)=0,"",IF($F5="",0,IF(NOT(ISNUMBER($I5)),"",IF($F5="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I5,1),IF($F5="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I5,1),"")))))</s:f>
       </s:c>
       <s:c r="L5" t="str" s="5">
-        <s:f>IF(COUNTA($A5:$G5)=0,"",IF(OR($A5="",$B5="",$C5="",$D5="",$E5=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B5))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A5))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E5="S",$E5="M",$E5="L")),"复杂度非法",IF(NOT(OR($F5="",$F5="内部集成",$F5="外部集成")),"集成类型非法",IF(AND($F5&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C5,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F5="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C5,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H5),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A5:$G5)=0,"",IF(LEFT($G5,4)="待确认：","待确认",IF(OR($A5="",$B5="",$C5="",$D5="",$E5=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B5))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A5))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E5="S",$E5="M",$E5="L")),"复杂度非法",IF(NOT(OR($F5="",$F5="内部集成",$F5="外部集成")),"集成类型非法",IF(AND($F5&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C5,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F5="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C5,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H5),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="6" ht="42" customHeight="1">
@@ -2446,7 +2446,7 @@
         <s:f>IF(COUNTA($A6:$G6)=0,"",IF($F6="",0,IF(NOT(ISNUMBER($I6)),"",IF($F6="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I6,1),IF($F6="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I6,1),"")))))</s:f>
       </s:c>
       <s:c r="L6" t="str" s="5">
-        <s:f>IF(COUNTA($A6:$G6)=0,"",IF(OR($A6="",$B6="",$C6="",$D6="",$E6=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B6))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A6))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E6="S",$E6="M",$E6="L")),"复杂度非法",IF(NOT(OR($F6="",$F6="内部集成",$F6="外部集成")),"集成类型非法",IF(AND($F6&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C6,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F6="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C6,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H6),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A6:$G6)=0,"",IF(LEFT($G6,4)="待确认：","待确认",IF(OR($A6="",$B6="",$C6="",$D6="",$E6=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B6))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A6))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E6="S",$E6="M",$E6="L")),"复杂度非法",IF(NOT(OR($F6="",$F6="内部集成",$F6="外部集成")),"集成类型非法",IF(AND($F6&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C6,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F6="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C6,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H6),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="7" ht="42" customHeight="1">
@@ -2470,7 +2470,7 @@
         <s:f>IF(COUNTA($A7:$G7)=0,"",IF($F7="",0,IF(NOT(ISNUMBER($I7)),"",IF($F7="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I7,1),IF($F7="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I7,1),"")))))</s:f>
       </s:c>
       <s:c r="L7" t="str" s="5">
-        <s:f>IF(COUNTA($A7:$G7)=0,"",IF(OR($A7="",$B7="",$C7="",$D7="",$E7=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B7))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A7))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E7="S",$E7="M",$E7="L")),"复杂度非法",IF(NOT(OR($F7="",$F7="内部集成",$F7="外部集成")),"集成类型非法",IF(AND($F7&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C7,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F7="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C7,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H7),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A7:$G7)=0,"",IF(LEFT($G7,4)="待确认：","待确认",IF(OR($A7="",$B7="",$C7="",$D7="",$E7=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B7))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A7))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E7="S",$E7="M",$E7="L")),"复杂度非法",IF(NOT(OR($F7="",$F7="内部集成",$F7="外部集成")),"集成类型非法",IF(AND($F7&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C7,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F7="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C7,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H7),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="8" ht="42" customHeight="1">
@@ -2494,7 +2494,7 @@
         <s:f>IF(COUNTA($A8:$G8)=0,"",IF($F8="",0,IF(NOT(ISNUMBER($I8)),"",IF($F8="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I8,1),IF($F8="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I8,1),"")))))</s:f>
       </s:c>
       <s:c r="L8" t="str" s="5">
-        <s:f>IF(COUNTA($A8:$G8)=0,"",IF(OR($A8="",$B8="",$C8="",$D8="",$E8=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B8))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A8))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E8="S",$E8="M",$E8="L")),"复杂度非法",IF(NOT(OR($F8="",$F8="内部集成",$F8="外部集成")),"集成类型非法",IF(AND($F8&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C8,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F8="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C8,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H8),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A8:$G8)=0,"",IF(LEFT($G8,4)="待确认：","待确认",IF(OR($A8="",$B8="",$C8="",$D8="",$E8=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B8))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A8))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E8="S",$E8="M",$E8="L")),"复杂度非法",IF(NOT(OR($F8="",$F8="内部集成",$F8="外部集成")),"集成类型非法",IF(AND($F8&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C8,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F8="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C8,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H8),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="9" ht="42" customHeight="1">
@@ -2518,7 +2518,7 @@
         <s:f>IF(COUNTA($A9:$G9)=0,"",IF($F9="",0,IF(NOT(ISNUMBER($I9)),"",IF($F9="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I9,1),IF($F9="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I9,1),"")))))</s:f>
       </s:c>
       <s:c r="L9" t="str" s="5">
-        <s:f>IF(COUNTA($A9:$G9)=0,"",IF(OR($A9="",$B9="",$C9="",$D9="",$E9=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B9))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A9))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E9="S",$E9="M",$E9="L")),"复杂度非法",IF(NOT(OR($F9="",$F9="内部集成",$F9="外部集成")),"集成类型非法",IF(AND($F9&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C9,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F9="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C9,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H9),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A9:$G9)=0,"",IF(LEFT($G9,4)="待确认：","待确认",IF(OR($A9="",$B9="",$C9="",$D9="",$E9=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B9))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A9))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E9="S",$E9="M",$E9="L")),"复杂度非法",IF(NOT(OR($F9="",$F9="内部集成",$F9="外部集成")),"集成类型非法",IF(AND($F9&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C9,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F9="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C9,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H9),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="10" ht="42" customHeight="1">
@@ -2542,7 +2542,7 @@
         <s:f>IF(COUNTA($A10:$G10)=0,"",IF($F10="",0,IF(NOT(ISNUMBER($I10)),"",IF($F10="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I10,1),IF($F10="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I10,1),"")))))</s:f>
       </s:c>
       <s:c r="L10" t="str" s="5">
-        <s:f>IF(COUNTA($A10:$G10)=0,"",IF(OR($A10="",$B10="",$C10="",$D10="",$E10=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B10))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A10))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E10="S",$E10="M",$E10="L")),"复杂度非法",IF(NOT(OR($F10="",$F10="内部集成",$F10="外部集成")),"集成类型非法",IF(AND($F10&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C10,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F10="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C10,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H10),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A10:$G10)=0,"",IF(LEFT($G10,4)="待确认：","待确认",IF(OR($A10="",$B10="",$C10="",$D10="",$E10=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B10))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A10))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E10="S",$E10="M",$E10="L")),"复杂度非法",IF(NOT(OR($F10="",$F10="内部集成",$F10="外部集成")),"集成类型非法",IF(AND($F10&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C10,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F10="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C10,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H10),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="11" ht="42" customHeight="1">
@@ -2566,7 +2566,7 @@
         <s:f>IF(COUNTA($A11:$G11)=0,"",IF($F11="",0,IF(NOT(ISNUMBER($I11)),"",IF($F11="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I11,1),IF($F11="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I11,1),"")))))</s:f>
       </s:c>
       <s:c r="L11" t="str" s="5">
-        <s:f>IF(COUNTA($A11:$G11)=0,"",IF(OR($A11="",$B11="",$C11="",$D11="",$E11=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B11))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A11))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E11="S",$E11="M",$E11="L")),"复杂度非法",IF(NOT(OR($F11="",$F11="内部集成",$F11="外部集成")),"集成类型非法",IF(AND($F11&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C11,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F11="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C11,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H11),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A11:$G11)=0,"",IF(LEFT($G11,4)="待确认：","待确认",IF(OR($A11="",$B11="",$C11="",$D11="",$E11=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B11))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A11))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E11="S",$E11="M",$E11="L")),"复杂度非法",IF(NOT(OR($F11="",$F11="内部集成",$F11="外部集成")),"集成类型非法",IF(AND($F11&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C11,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F11="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C11,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H11),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="12" ht="42" customHeight="1">
@@ -2590,7 +2590,7 @@
         <s:f>IF(COUNTA($A12:$G12)=0,"",IF($F12="",0,IF(NOT(ISNUMBER($I12)),"",IF($F12="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I12,1),IF($F12="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I12,1),"")))))</s:f>
       </s:c>
       <s:c r="L12" t="str" s="5">
-        <s:f>IF(COUNTA($A12:$G12)=0,"",IF(OR($A12="",$B12="",$C12="",$D12="",$E12=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B12))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A12))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E12="S",$E12="M",$E12="L")),"复杂度非法",IF(NOT(OR($F12="",$F12="内部集成",$F12="外部集成")),"集成类型非法",IF(AND($F12&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C12,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F12="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C12,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H12),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A12:$G12)=0,"",IF(LEFT($G12,4)="待确认：","待确认",IF(OR($A12="",$B12="",$C12="",$D12="",$E12=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B12))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A12))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E12="S",$E12="M",$E12="L")),"复杂度非法",IF(NOT(OR($F12="",$F12="内部集成",$F12="外部集成")),"集成类型非法",IF(AND($F12&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C12,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F12="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C12,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H12),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="13" ht="42" customHeight="1">
@@ -2614,7 +2614,7 @@
         <s:f>IF(COUNTA($A13:$G13)=0,"",IF($F13="",0,IF(NOT(ISNUMBER($I13)),"",IF($F13="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I13,1),IF($F13="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I13,1),"")))))</s:f>
       </s:c>
       <s:c r="L13" t="str" s="5">
-        <s:f>IF(COUNTA($A13:$G13)=0,"",IF(OR($A13="",$B13="",$C13="",$D13="",$E13=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B13))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A13))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E13="S",$E13="M",$E13="L")),"复杂度非法",IF(NOT(OR($F13="",$F13="内部集成",$F13="外部集成")),"集成类型非法",IF(AND($F13&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C13,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F13="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C13,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H13),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A13:$G13)=0,"",IF(LEFT($G13,4)="待确认：","待确认",IF(OR($A13="",$B13="",$C13="",$D13="",$E13=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B13))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A13))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E13="S",$E13="M",$E13="L")),"复杂度非法",IF(NOT(OR($F13="",$F13="内部集成",$F13="外部集成")),"集成类型非法",IF(AND($F13&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C13,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F13="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C13,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H13),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="14" ht="42" customHeight="1">
@@ -2638,7 +2638,7 @@
         <s:f>IF(COUNTA($A14:$G14)=0,"",IF($F14="",0,IF(NOT(ISNUMBER($I14)),"",IF($F14="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I14,1),IF($F14="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I14,1),"")))))</s:f>
       </s:c>
       <s:c r="L14" t="str" s="5">
-        <s:f>IF(COUNTA($A14:$G14)=0,"",IF(OR($A14="",$B14="",$C14="",$D14="",$E14=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B14))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A14))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E14="S",$E14="M",$E14="L")),"复杂度非法",IF(NOT(OR($F14="",$F14="内部集成",$F14="外部集成")),"集成类型非法",IF(AND($F14&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C14,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F14="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C14,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H14),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A14:$G14)=0,"",IF(LEFT($G14,4)="待确认：","待确认",IF(OR($A14="",$B14="",$C14="",$D14="",$E14=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B14))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A14))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E14="S",$E14="M",$E14="L")),"复杂度非法",IF(NOT(OR($F14="",$F14="内部集成",$F14="外部集成")),"集成类型非法",IF(AND($F14&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C14,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F14="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C14,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H14),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="15" ht="42" customHeight="1">
@@ -2662,7 +2662,7 @@
         <s:f>IF(COUNTA($A15:$G15)=0,"",IF($F15="",0,IF(NOT(ISNUMBER($I15)),"",IF($F15="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I15,1),IF($F15="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I15,1),"")))))</s:f>
       </s:c>
       <s:c r="L15" t="str" s="5">
-        <s:f>IF(COUNTA($A15:$G15)=0,"",IF(OR($A15="",$B15="",$C15="",$D15="",$E15=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B15))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A15))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E15="S",$E15="M",$E15="L")),"复杂度非法",IF(NOT(OR($F15="",$F15="内部集成",$F15="外部集成")),"集成类型非法",IF(AND($F15&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C15,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F15="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C15,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H15),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A15:$G15)=0,"",IF(LEFT($G15,4)="待确认：","待确认",IF(OR($A15="",$B15="",$C15="",$D15="",$E15=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B15))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A15))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E15="S",$E15="M",$E15="L")),"复杂度非法",IF(NOT(OR($F15="",$F15="内部集成",$F15="外部集成")),"集成类型非法",IF(AND($F15&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C15,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F15="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C15,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H15),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="16" ht="42" customHeight="1">
@@ -2686,7 +2686,7 @@
         <s:f>IF(COUNTA($A16:$G16)=0,"",IF($F16="",0,IF(NOT(ISNUMBER($I16)),"",IF($F16="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I16,1),IF($F16="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I16,1),"")))))</s:f>
       </s:c>
       <s:c r="L16" t="str" s="5">
-        <s:f>IF(COUNTA($A16:$G16)=0,"",IF(OR($A16="",$B16="",$C16="",$D16="",$E16=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B16))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A16))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E16="S",$E16="M",$E16="L")),"复杂度非法",IF(NOT(OR($F16="",$F16="内部集成",$F16="外部集成")),"集成类型非法",IF(AND($F16&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C16,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F16="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C16,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H16),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A16:$G16)=0,"",IF(LEFT($G16,4)="待确认：","待确认",IF(OR($A16="",$B16="",$C16="",$D16="",$E16=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B16))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A16))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E16="S",$E16="M",$E16="L")),"复杂度非法",IF(NOT(OR($F16="",$F16="内部集成",$F16="外部集成")),"集成类型非法",IF(AND($F16&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C16,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F16="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C16,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H16),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="17" ht="42" customHeight="1">
@@ -2710,7 +2710,7 @@
         <s:f>IF(COUNTA($A17:$G17)=0,"",IF($F17="",0,IF(NOT(ISNUMBER($I17)),"",IF($F17="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I17,1),IF($F17="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I17,1),"")))))</s:f>
       </s:c>
       <s:c r="L17" t="str" s="5">
-        <s:f>IF(COUNTA($A17:$G17)=0,"",IF(OR($A17="",$B17="",$C17="",$D17="",$E17=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B17))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A17))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E17="S",$E17="M",$E17="L")),"复杂度非法",IF(NOT(OR($F17="",$F17="内部集成",$F17="外部集成")),"集成类型非法",IF(AND($F17&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C17,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F17="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C17,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H17),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A17:$G17)=0,"",IF(LEFT($G17,4)="待确认：","待确认",IF(OR($A17="",$B17="",$C17="",$D17="",$E17=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B17))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A17))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E17="S",$E17="M",$E17="L")),"复杂度非法",IF(NOT(OR($F17="",$F17="内部集成",$F17="外部集成")),"集成类型非法",IF(AND($F17&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C17,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F17="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C17,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H17),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="18" ht="42" customHeight="1">
@@ -2734,7 +2734,7 @@
         <s:f>IF(COUNTA($A18:$G18)=0,"",IF($F18="",0,IF(NOT(ISNUMBER($I18)),"",IF($F18="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I18,1),IF($F18="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I18,1),"")))))</s:f>
       </s:c>
       <s:c r="L18" t="str" s="5">
-        <s:f>IF(COUNTA($A18:$G18)=0,"",IF(OR($A18="",$B18="",$C18="",$D18="",$E18=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B18))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A18))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E18="S",$E18="M",$E18="L")),"复杂度非法",IF(NOT(OR($F18="",$F18="内部集成",$F18="外部集成")),"集成类型非法",IF(AND($F18&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C18,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F18="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C18,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H18),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A18:$G18)=0,"",IF(LEFT($G18,4)="待确认：","待确认",IF(OR($A18="",$B18="",$C18="",$D18="",$E18=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B18))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A18))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E18="S",$E18="M",$E18="L")),"复杂度非法",IF(NOT(OR($F18="",$F18="内部集成",$F18="外部集成")),"集成类型非法",IF(AND($F18&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C18,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F18="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C18,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H18),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="19" ht="42" customHeight="1">
@@ -2758,7 +2758,7 @@
         <s:f>IF(COUNTA($A19:$G19)=0,"",IF($F19="",0,IF(NOT(ISNUMBER($I19)),"",IF($F19="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I19,1),IF($F19="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I19,1),"")))))</s:f>
       </s:c>
       <s:c r="L19" t="str" s="5">
-        <s:f>IF(COUNTA($A19:$G19)=0,"",IF(OR($A19="",$B19="",$C19="",$D19="",$E19=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B19))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A19))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E19="S",$E19="M",$E19="L")),"复杂度非法",IF(NOT(OR($F19="",$F19="内部集成",$F19="外部集成")),"集成类型非法",IF(AND($F19&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C19,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F19="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C19,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H19),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A19:$G19)=0,"",IF(LEFT($G19,4)="待确认：","待确认",IF(OR($A19="",$B19="",$C19="",$D19="",$E19=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B19))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A19))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E19="S",$E19="M",$E19="L")),"复杂度非法",IF(NOT(OR($F19="",$F19="内部集成",$F19="外部集成")),"集成类型非法",IF(AND($F19&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C19,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F19="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C19,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H19),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="20" ht="42" customHeight="1">
@@ -2782,7 +2782,7 @@
         <s:f>IF(COUNTA($A20:$G20)=0,"",IF($F20="",0,IF(NOT(ISNUMBER($I20)),"",IF($F20="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I20,1),IF($F20="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I20,1),"")))))</s:f>
       </s:c>
       <s:c r="L20" t="str" s="5">
-        <s:f>IF(COUNTA($A20:$G20)=0,"",IF(OR($A20="",$B20="",$C20="",$D20="",$E20=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B20))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A20))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E20="S",$E20="M",$E20="L")),"复杂度非法",IF(NOT(OR($F20="",$F20="内部集成",$F20="外部集成")),"集成类型非法",IF(AND($F20&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C20,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F20="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C20,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H20),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A20:$G20)=0,"",IF(LEFT($G20,4)="待确认：","待确认",IF(OR($A20="",$B20="",$C20="",$D20="",$E20=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B20))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A20))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E20="S",$E20="M",$E20="L")),"复杂度非法",IF(NOT(OR($F20="",$F20="内部集成",$F20="外部集成")),"集成类型非法",IF(AND($F20&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C20,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F20="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C20,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H20),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="21" ht="42" customHeight="1">
@@ -2806,7 +2806,7 @@
         <s:f>IF(COUNTA($A21:$G21)=0,"",IF($F21="",0,IF(NOT(ISNUMBER($I21)),"",IF($F21="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I21,1),IF($F21="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I21,1),"")))))</s:f>
       </s:c>
       <s:c r="L21" t="str" s="5">
-        <s:f>IF(COUNTA($A21:$G21)=0,"",IF(OR($A21="",$B21="",$C21="",$D21="",$E21=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B21))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A21))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E21="S",$E21="M",$E21="L")),"复杂度非法",IF(NOT(OR($F21="",$F21="内部集成",$F21="外部集成")),"集成类型非法",IF(AND($F21&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C21,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F21="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C21,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H21),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A21:$G21)=0,"",IF(LEFT($G21,4)="待确认：","待确认",IF(OR($A21="",$B21="",$C21="",$D21="",$E21=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B21))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A21))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E21="S",$E21="M",$E21="L")),"复杂度非法",IF(NOT(OR($F21="",$F21="内部集成",$F21="外部集成")),"集成类型非法",IF(AND($F21&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C21,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F21="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C21,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H21),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="22" ht="42" customHeight="1">
@@ -2830,7 +2830,7 @@
         <s:f>IF(COUNTA($A22:$G22)=0,"",IF($F22="",0,IF(NOT(ISNUMBER($I22)),"",IF($F22="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I22,1),IF($F22="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I22,1),"")))))</s:f>
       </s:c>
       <s:c r="L22" t="str" s="5">
-        <s:f>IF(COUNTA($A22:$G22)=0,"",IF(OR($A22="",$B22="",$C22="",$D22="",$E22=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B22))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A22))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E22="S",$E22="M",$E22="L")),"复杂度非法",IF(NOT(OR($F22="",$F22="内部集成",$F22="外部集成")),"集成类型非法",IF(AND($F22&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C22,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F22="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C22,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H22),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A22:$G22)=0,"",IF(LEFT($G22,4)="待确认：","待确认",IF(OR($A22="",$B22="",$C22="",$D22="",$E22=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B22))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A22))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E22="S",$E22="M",$E22="L")),"复杂度非法",IF(NOT(OR($F22="",$F22="内部集成",$F22="外部集成")),"集成类型非法",IF(AND($F22&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C22,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F22="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C22,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H22),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="23" ht="42" customHeight="1">
@@ -2854,7 +2854,7 @@
         <s:f>IF(COUNTA($A23:$G23)=0,"",IF($F23="",0,IF(NOT(ISNUMBER($I23)),"",IF($F23="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I23,1),IF($F23="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I23,1),"")))))</s:f>
       </s:c>
       <s:c r="L23" t="str" s="5">
-        <s:f>IF(COUNTA($A23:$G23)=0,"",IF(OR($A23="",$B23="",$C23="",$D23="",$E23=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B23))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A23))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E23="S",$E23="M",$E23="L")),"复杂度非法",IF(NOT(OR($F23="",$F23="内部集成",$F23="外部集成")),"集成类型非法",IF(AND($F23&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C23,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F23="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C23,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H23),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A23:$G23)=0,"",IF(LEFT($G23,4)="待确认：","待确认",IF(OR($A23="",$B23="",$C23="",$D23="",$E23=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B23))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A23))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E23="S",$E23="M",$E23="L")),"复杂度非法",IF(NOT(OR($F23="",$F23="内部集成",$F23="外部集成")),"集成类型非法",IF(AND($F23&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C23,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F23="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C23,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H23),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="24" ht="42" customHeight="1">
@@ -2878,7 +2878,7 @@
         <s:f>IF(COUNTA($A24:$G24)=0,"",IF($F24="",0,IF(NOT(ISNUMBER($I24)),"",IF($F24="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I24,1),IF($F24="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I24,1),"")))))</s:f>
       </s:c>
       <s:c r="L24" t="str" s="5">
-        <s:f>IF(COUNTA($A24:$G24)=0,"",IF(OR($A24="",$B24="",$C24="",$D24="",$E24=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B24))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A24))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E24="S",$E24="M",$E24="L")),"复杂度非法",IF(NOT(OR($F24="",$F24="内部集成",$F24="外部集成")),"集成类型非法",IF(AND($F24&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C24,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F24="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C24,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H24),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A24:$G24)=0,"",IF(LEFT($G24,4)="待确认：","待确认",IF(OR($A24="",$B24="",$C24="",$D24="",$E24=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B24))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A24))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E24="S",$E24="M",$E24="L")),"复杂度非法",IF(NOT(OR($F24="",$F24="内部集成",$F24="外部集成")),"集成类型非法",IF(AND($F24&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C24,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F24="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C24,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H24),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="25" ht="42" customHeight="1">
@@ -2902,7 +2902,7 @@
         <s:f>IF(COUNTA($A25:$G25)=0,"",IF($F25="",0,IF(NOT(ISNUMBER($I25)),"",IF($F25="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I25,1),IF($F25="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I25,1),"")))))</s:f>
       </s:c>
       <s:c r="L25" t="str" s="5">
-        <s:f>IF(COUNTA($A25:$G25)=0,"",IF(OR($A25="",$B25="",$C25="",$D25="",$E25=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B25))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A25))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E25="S",$E25="M",$E25="L")),"复杂度非法",IF(NOT(OR($F25="",$F25="内部集成",$F25="外部集成")),"集成类型非法",IF(AND($F25&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C25,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F25="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C25,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H25),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A25:$G25)=0,"",IF(LEFT($G25,4)="待确认：","待确认",IF(OR($A25="",$B25="",$C25="",$D25="",$E25=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B25))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A25))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E25="S",$E25="M",$E25="L")),"复杂度非法",IF(NOT(OR($F25="",$F25="内部集成",$F25="外部集成")),"集成类型非法",IF(AND($F25&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C25,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F25="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C25,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H25),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="26" ht="42" customHeight="1">
@@ -2926,7 +2926,7 @@
         <s:f>IF(COUNTA($A26:$G26)=0,"",IF($F26="",0,IF(NOT(ISNUMBER($I26)),"",IF($F26="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I26,1),IF($F26="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I26,1),"")))))</s:f>
       </s:c>
       <s:c r="L26" t="str" s="5">
-        <s:f>IF(COUNTA($A26:$G26)=0,"",IF(OR($A26="",$B26="",$C26="",$D26="",$E26=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B26))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A26))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E26="S",$E26="M",$E26="L")),"复杂度非法",IF(NOT(OR($F26="",$F26="内部集成",$F26="外部集成")),"集成类型非法",IF(AND($F26&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C26,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F26="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C26,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H26),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A26:$G26)=0,"",IF(LEFT($G26,4)="待确认：","待确认",IF(OR($A26="",$B26="",$C26="",$D26="",$E26=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B26))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A26))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E26="S",$E26="M",$E26="L")),"复杂度非法",IF(NOT(OR($F26="",$F26="内部集成",$F26="外部集成")),"集成类型非法",IF(AND($F26&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C26,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F26="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C26,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H26),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="27" ht="42" customHeight="1">
@@ -2950,7 +2950,7 @@
         <s:f>IF(COUNTA($A27:$G27)=0,"",IF($F27="",0,IF(NOT(ISNUMBER($I27)),"",IF($F27="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I27,1),IF($F27="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I27,1),"")))))</s:f>
       </s:c>
       <s:c r="L27" t="str" s="5">
-        <s:f>IF(COUNTA($A27:$G27)=0,"",IF(OR($A27="",$B27="",$C27="",$D27="",$E27=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B27))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A27))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E27="S",$E27="M",$E27="L")),"复杂度非法",IF(NOT(OR($F27="",$F27="内部集成",$F27="外部集成")),"集成类型非法",IF(AND($F27&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C27,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F27="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C27,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H27),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A27:$G27)=0,"",IF(LEFT($G27,4)="待确认：","待确认",IF(OR($A27="",$B27="",$C27="",$D27="",$E27=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B27))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A27))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E27="S",$E27="M",$E27="L")),"复杂度非法",IF(NOT(OR($F27="",$F27="内部集成",$F27="外部集成")),"集成类型非法",IF(AND($F27&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C27,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F27="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C27,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H27),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="28" ht="42" customHeight="1">
@@ -2974,7 +2974,7 @@
         <s:f>IF(COUNTA($A28:$G28)=0,"",IF($F28="",0,IF(NOT(ISNUMBER($I28)),"",IF($F28="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I28,1),IF($F28="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I28,1),"")))))</s:f>
       </s:c>
       <s:c r="L28" t="str" s="5">
-        <s:f>IF(COUNTA($A28:$G28)=0,"",IF(OR($A28="",$B28="",$C28="",$D28="",$E28=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B28))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A28))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E28="S",$E28="M",$E28="L")),"复杂度非法",IF(NOT(OR($F28="",$F28="内部集成",$F28="外部集成")),"集成类型非法",IF(AND($F28&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C28,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F28="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C28,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H28),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A28:$G28)=0,"",IF(LEFT($G28,4)="待确认：","待确认",IF(OR($A28="",$B28="",$C28="",$D28="",$E28=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B28))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A28))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E28="S",$E28="M",$E28="L")),"复杂度非法",IF(NOT(OR($F28="",$F28="内部集成",$F28="外部集成")),"集成类型非法",IF(AND($F28&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C28,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F28="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C28,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H28),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="29" ht="42" customHeight="1">
@@ -2998,7 +2998,7 @@
         <s:f>IF(COUNTA($A29:$G29)=0,"",IF($F29="",0,IF(NOT(ISNUMBER($I29)),"",IF($F29="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I29,1),IF($F29="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I29,1),"")))))</s:f>
       </s:c>
       <s:c r="L29" t="str" s="5">
-        <s:f>IF(COUNTA($A29:$G29)=0,"",IF(OR($A29="",$B29="",$C29="",$D29="",$E29=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B29))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A29))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E29="S",$E29="M",$E29="L")),"复杂度非法",IF(NOT(OR($F29="",$F29="内部集成",$F29="外部集成")),"集成类型非法",IF(AND($F29&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C29,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F29="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C29,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H29),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A29:$G29)=0,"",IF(LEFT($G29,4)="待确认：","待确认",IF(OR($A29="",$B29="",$C29="",$D29="",$E29=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B29))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A29))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E29="S",$E29="M",$E29="L")),"复杂度非法",IF(NOT(OR($F29="",$F29="内部集成",$F29="外部集成")),"集成类型非法",IF(AND($F29&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C29,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F29="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C29,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H29),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="30" ht="42" customHeight="1">
@@ -3022,7 +3022,7 @@
         <s:f>IF(COUNTA($A30:$G30)=0,"",IF($F30="",0,IF(NOT(ISNUMBER($I30)),"",IF($F30="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I30,1),IF($F30="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I30,1),"")))))</s:f>
       </s:c>
       <s:c r="L30" t="str" s="5">
-        <s:f>IF(COUNTA($A30:$G30)=0,"",IF(OR($A30="",$B30="",$C30="",$D30="",$E30=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B30))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A30))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E30="S",$E30="M",$E30="L")),"复杂度非法",IF(NOT(OR($F30="",$F30="内部集成",$F30="外部集成")),"集成类型非法",IF(AND($F30&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C30,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F30="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C30,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H30),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A30:$G30)=0,"",IF(LEFT($G30,4)="待确认：","待确认",IF(OR($A30="",$B30="",$C30="",$D30="",$E30=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B30))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A30))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E30="S",$E30="M",$E30="L")),"复杂度非法",IF(NOT(OR($F30="",$F30="内部集成",$F30="外部集成")),"集成类型非法",IF(AND($F30&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C30,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F30="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C30,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H30),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="31" ht="42" customHeight="1">
@@ -3046,7 +3046,7 @@
         <s:f>IF(COUNTA($A31:$G31)=0,"",IF($F31="",0,IF(NOT(ISNUMBER($I31)),"",IF($F31="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I31,1),IF($F31="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I31,1),"")))))</s:f>
       </s:c>
       <s:c r="L31" t="str" s="5">
-        <s:f>IF(COUNTA($A31:$G31)=0,"",IF(OR($A31="",$B31="",$C31="",$D31="",$E31=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B31))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A31))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E31="S",$E31="M",$E31="L")),"复杂度非法",IF(NOT(OR($F31="",$F31="内部集成",$F31="外部集成")),"集成类型非法",IF(AND($F31&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C31,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F31="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C31,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H31),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A31:$G31)=0,"",IF(LEFT($G31,4)="待确认：","待确认",IF(OR($A31="",$B31="",$C31="",$D31="",$E31=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B31))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A31))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E31="S",$E31="M",$E31="L")),"复杂度非法",IF(NOT(OR($F31="",$F31="内部集成",$F31="外部集成")),"集成类型非法",IF(AND($F31&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C31,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F31="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C31,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H31),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="32" ht="42" customHeight="1">
@@ -3070,7 +3070,7 @@
         <s:f>IF(COUNTA($A32:$G32)=0,"",IF($F32="",0,IF(NOT(ISNUMBER($I32)),"",IF($F32="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I32,1),IF($F32="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I32,1),"")))))</s:f>
       </s:c>
       <s:c r="L32" t="str" s="5">
-        <s:f>IF(COUNTA($A32:$G32)=0,"",IF(OR($A32="",$B32="",$C32="",$D32="",$E32=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B32))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A32))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E32="S",$E32="M",$E32="L")),"复杂度非法",IF(NOT(OR($F32="",$F32="内部集成",$F32="外部集成")),"集成类型非法",IF(AND($F32&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C32,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F32="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C32,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H32),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A32:$G32)=0,"",IF(LEFT($G32,4)="待确认：","待确认",IF(OR($A32="",$B32="",$C32="",$D32="",$E32=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B32))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A32))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E32="S",$E32="M",$E32="L")),"复杂度非法",IF(NOT(OR($F32="",$F32="内部集成",$F32="外部集成")),"集成类型非法",IF(AND($F32&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C32,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F32="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C32,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H32),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="33" ht="42" customHeight="1">
@@ -3094,7 +3094,7 @@
         <s:f>IF(COUNTA($A33:$G33)=0,"",IF($F33="",0,IF(NOT(ISNUMBER($I33)),"",IF($F33="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I33,1),IF($F33="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I33,1),"")))))</s:f>
       </s:c>
       <s:c r="L33" t="str" s="5">
-        <s:f>IF(COUNTA($A33:$G33)=0,"",IF(OR($A33="",$B33="",$C33="",$D33="",$E33=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B33))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A33))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E33="S",$E33="M",$E33="L")),"复杂度非法",IF(NOT(OR($F33="",$F33="内部集成",$F33="外部集成")),"集成类型非法",IF(AND($F33&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C33,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F33="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C33,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H33),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A33:$G33)=0,"",IF(LEFT($G33,4)="待确认：","待确认",IF(OR($A33="",$B33="",$C33="",$D33="",$E33=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B33))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A33))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E33="S",$E33="M",$E33="L")),"复杂度非法",IF(NOT(OR($F33="",$F33="内部集成",$F33="外部集成")),"集成类型非法",IF(AND($F33&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C33,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F33="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C33,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H33),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="34" ht="42" customHeight="1">
@@ -3118,7 +3118,7 @@
         <s:f>IF(COUNTA($A34:$G34)=0,"",IF($F34="",0,IF(NOT(ISNUMBER($I34)),"",IF($F34="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I34,1),IF($F34="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I34,1),"")))))</s:f>
       </s:c>
       <s:c r="L34" t="str" s="5">
-        <s:f>IF(COUNTA($A34:$G34)=0,"",IF(OR($A34="",$B34="",$C34="",$D34="",$E34=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B34))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A34))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E34="S",$E34="M",$E34="L")),"复杂度非法",IF(NOT(OR($F34="",$F34="内部集成",$F34="外部集成")),"集成类型非法",IF(AND($F34&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C34,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F34="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C34,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H34),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A34:$G34)=0,"",IF(LEFT($G34,4)="待确认：","待确认",IF(OR($A34="",$B34="",$C34="",$D34="",$E34=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B34))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A34))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E34="S",$E34="M",$E34="L")),"复杂度非法",IF(NOT(OR($F34="",$F34="内部集成",$F34="外部集成")),"集成类型非法",IF(AND($F34&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C34,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F34="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C34,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H34),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="35" ht="42" customHeight="1">
@@ -3142,7 +3142,7 @@
         <s:f>IF(COUNTA($A35:$G35)=0,"",IF($F35="",0,IF(NOT(ISNUMBER($I35)),"",IF($F35="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I35,1),IF($F35="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I35,1),"")))))</s:f>
       </s:c>
       <s:c r="L35" t="str" s="5">
-        <s:f>IF(COUNTA($A35:$G35)=0,"",IF(OR($A35="",$B35="",$C35="",$D35="",$E35=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B35))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A35))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E35="S",$E35="M",$E35="L")),"复杂度非法",IF(NOT(OR($F35="",$F35="内部集成",$F35="外部集成")),"集成类型非法",IF(AND($F35&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C35,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F35="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C35,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H35),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A35:$G35)=0,"",IF(LEFT($G35,4)="待确认：","待确认",IF(OR($A35="",$B35="",$C35="",$D35="",$E35=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B35))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A35))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E35="S",$E35="M",$E35="L")),"复杂度非法",IF(NOT(OR($F35="",$F35="内部集成",$F35="外部集成")),"集成类型非法",IF(AND($F35&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C35,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F35="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C35,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H35),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="36" ht="42" customHeight="1">
@@ -3166,7 +3166,7 @@
         <s:f>IF(COUNTA($A36:$G36)=0,"",IF($F36="",0,IF(NOT(ISNUMBER($I36)),"",IF($F36="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I36,1),IF($F36="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I36,1),"")))))</s:f>
       </s:c>
       <s:c r="L36" t="str" s="5">
-        <s:f>IF(COUNTA($A36:$G36)=0,"",IF(OR($A36="",$B36="",$C36="",$D36="",$E36=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B36))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A36))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E36="S",$E36="M",$E36="L")),"复杂度非法",IF(NOT(OR($F36="",$F36="内部集成",$F36="外部集成")),"集成类型非法",IF(AND($F36&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C36,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F36="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C36,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H36),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A36:$G36)=0,"",IF(LEFT($G36,4)="待确认：","待确认",IF(OR($A36="",$B36="",$C36="",$D36="",$E36=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B36))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A36))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E36="S",$E36="M",$E36="L")),"复杂度非法",IF(NOT(OR($F36="",$F36="内部集成",$F36="外部集成")),"集成类型非法",IF(AND($F36&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C36,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F36="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C36,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H36),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="37" ht="42" customHeight="1">
@@ -3190,7 +3190,7 @@
         <s:f>IF(COUNTA($A37:$G37)=0,"",IF($F37="",0,IF(NOT(ISNUMBER($I37)),"",IF($F37="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I37,1),IF($F37="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I37,1),"")))))</s:f>
       </s:c>
       <s:c r="L37" t="str" s="5">
-        <s:f>IF(COUNTA($A37:$G37)=0,"",IF(OR($A37="",$B37="",$C37="",$D37="",$E37=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B37))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A37))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E37="S",$E37="M",$E37="L")),"复杂度非法",IF(NOT(OR($F37="",$F37="内部集成",$F37="外部集成")),"集成类型非法",IF(AND($F37&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C37,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F37="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C37,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H37),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A37:$G37)=0,"",IF(LEFT($G37,4)="待确认：","待确认",IF(OR($A37="",$B37="",$C37="",$D37="",$E37=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B37))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A37))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E37="S",$E37="M",$E37="L")),"复杂度非法",IF(NOT(OR($F37="",$F37="内部集成",$F37="外部集成")),"集成类型非法",IF(AND($F37&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C37,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F37="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C37,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H37),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="38" ht="42" customHeight="1">
@@ -3214,7 +3214,7 @@
         <s:f>IF(COUNTA($A38:$G38)=0,"",IF($F38="",0,IF(NOT(ISNUMBER($I38)),"",IF($F38="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I38,1),IF($F38="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I38,1),"")))))</s:f>
       </s:c>
       <s:c r="L38" t="str" s="5">
-        <s:f>IF(COUNTA($A38:$G38)=0,"",IF(OR($A38="",$B38="",$C38="",$D38="",$E38=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B38))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A38))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E38="S",$E38="M",$E38="L")),"复杂度非法",IF(NOT(OR($F38="",$F38="内部集成",$F38="外部集成")),"集成类型非法",IF(AND($F38&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C38,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F38="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C38,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H38),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A38:$G38)=0,"",IF(LEFT($G38,4)="待确认：","待确认",IF(OR($A38="",$B38="",$C38="",$D38="",$E38=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B38))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A38))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E38="S",$E38="M",$E38="L")),"复杂度非法",IF(NOT(OR($F38="",$F38="内部集成",$F38="外部集成")),"集成类型非法",IF(AND($F38&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C38,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F38="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C38,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H38),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="39" ht="42" customHeight="1">
@@ -3238,7 +3238,7 @@
         <s:f>IF(COUNTA($A39:$G39)=0,"",IF($F39="",0,IF(NOT(ISNUMBER($I39)),"",IF($F39="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I39,1),IF($F39="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I39,1),"")))))</s:f>
       </s:c>
       <s:c r="L39" t="str" s="5">
-        <s:f>IF(COUNTA($A39:$G39)=0,"",IF(OR($A39="",$B39="",$C39="",$D39="",$E39=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B39))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A39))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E39="S",$E39="M",$E39="L")),"复杂度非法",IF(NOT(OR($F39="",$F39="内部集成",$F39="外部集成")),"集成类型非法",IF(AND($F39&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C39,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F39="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C39,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H39),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A39:$G39)=0,"",IF(LEFT($G39,4)="待确认：","待确认",IF(OR($A39="",$B39="",$C39="",$D39="",$E39=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B39))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A39))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E39="S",$E39="M",$E39="L")),"复杂度非法",IF(NOT(OR($F39="",$F39="内部集成",$F39="外部集成")),"集成类型非法",IF(AND($F39&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C39,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F39="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C39,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H39),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="40" ht="42" customHeight="1">
@@ -3262,7 +3262,7 @@
         <s:f>IF(COUNTA($A40:$G40)=0,"",IF($F40="",0,IF(NOT(ISNUMBER($I40)),"",IF($F40="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I40,1),IF($F40="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I40,1),"")))))</s:f>
       </s:c>
       <s:c r="L40" t="str" s="5">
-        <s:f>IF(COUNTA($A40:$G40)=0,"",IF(OR($A40="",$B40="",$C40="",$D40="",$E40=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B40))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A40))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E40="S",$E40="M",$E40="L")),"复杂度非法",IF(NOT(OR($F40="",$F40="内部集成",$F40="外部集成")),"集成类型非法",IF(AND($F40&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C40,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F40="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C40,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H40),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A40:$G40)=0,"",IF(LEFT($G40,4)="待确认：","待确认",IF(OR($A40="",$B40="",$C40="",$D40="",$E40=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B40))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A40))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E40="S",$E40="M",$E40="L")),"复杂度非法",IF(NOT(OR($F40="",$F40="内部集成",$F40="外部集成")),"集成类型非法",IF(AND($F40&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C40,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F40="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C40,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H40),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="41" ht="42" customHeight="1">
@@ -3286,7 +3286,7 @@
         <s:f>IF(COUNTA($A41:$G41)=0,"",IF($F41="",0,IF(NOT(ISNUMBER($I41)),"",IF($F41="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I41,1),IF($F41="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I41,1),"")))))</s:f>
       </s:c>
       <s:c r="L41" t="str" s="5">
-        <s:f>IF(COUNTA($A41:$G41)=0,"",IF(OR($A41="",$B41="",$C41="",$D41="",$E41=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B41))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A41))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E41="S",$E41="M",$E41="L")),"复杂度非法",IF(NOT(OR($F41="",$F41="内部集成",$F41="外部集成")),"集成类型非法",IF(AND($F41&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C41,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F41="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C41,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H41),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A41:$G41)=0,"",IF(LEFT($G41,4)="待确认：","待确认",IF(OR($A41="",$B41="",$C41="",$D41="",$E41=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B41))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A41))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E41="S",$E41="M",$E41="L")),"复杂度非法",IF(NOT(OR($F41="",$F41="内部集成",$F41="外部集成")),"集成类型非法",IF(AND($F41&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C41,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F41="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C41,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H41),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="42" ht="42" customHeight="1">
@@ -3310,7 +3310,7 @@
         <s:f>IF(COUNTA($A42:$G42)=0,"",IF($F42="",0,IF(NOT(ISNUMBER($I42)),"",IF($F42="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I42,1),IF($F42="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I42,1),"")))))</s:f>
       </s:c>
       <s:c r="L42" t="str" s="5">
-        <s:f>IF(COUNTA($A42:$G42)=0,"",IF(OR($A42="",$B42="",$C42="",$D42="",$E42=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B42))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A42))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E42="S",$E42="M",$E42="L")),"复杂度非法",IF(NOT(OR($F42="",$F42="内部集成",$F42="外部集成")),"集成类型非法",IF(AND($F42&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C42,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F42="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C42,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H42),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A42:$G42)=0,"",IF(LEFT($G42,4)="待确认：","待确认",IF(OR($A42="",$B42="",$C42="",$D42="",$E42=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B42))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A42))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E42="S",$E42="M",$E42="L")),"复杂度非法",IF(NOT(OR($F42="",$F42="内部集成",$F42="外部集成")),"集成类型非法",IF(AND($F42&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C42,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F42="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C42,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H42),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="43" ht="42" customHeight="1">
@@ -3334,7 +3334,7 @@
         <s:f>IF(COUNTA($A43:$G43)=0,"",IF($F43="",0,IF(NOT(ISNUMBER($I43)),"",IF($F43="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I43,1),IF($F43="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I43,1),"")))))</s:f>
       </s:c>
       <s:c r="L43" t="str" s="5">
-        <s:f>IF(COUNTA($A43:$G43)=0,"",IF(OR($A43="",$B43="",$C43="",$D43="",$E43=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B43))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A43))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E43="S",$E43="M",$E43="L")),"复杂度非法",IF(NOT(OR($F43="",$F43="内部集成",$F43="外部集成")),"集成类型非法",IF(AND($F43&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C43,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F43="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C43,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H43),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A43:$G43)=0,"",IF(LEFT($G43,4)="待确认：","待确认",IF(OR($A43="",$B43="",$C43="",$D43="",$E43=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B43))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A43))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E43="S",$E43="M",$E43="L")),"复杂度非法",IF(NOT(OR($F43="",$F43="内部集成",$F43="外部集成")),"集成类型非法",IF(AND($F43&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C43,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F43="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C43,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H43),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="44" ht="42" customHeight="1">
@@ -3358,7 +3358,7 @@
         <s:f>IF(COUNTA($A44:$G44)=0,"",IF($F44="",0,IF(NOT(ISNUMBER($I44)),"",IF($F44="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I44,1),IF($F44="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I44,1),"")))))</s:f>
       </s:c>
       <s:c r="L44" t="str" s="5">
-        <s:f>IF(COUNTA($A44:$G44)=0,"",IF(OR($A44="",$B44="",$C44="",$D44="",$E44=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B44))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A44))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E44="S",$E44="M",$E44="L")),"复杂度非法",IF(NOT(OR($F44="",$F44="内部集成",$F44="外部集成")),"集成类型非法",IF(AND($F44&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C44,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F44="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C44,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H44),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A44:$G44)=0,"",IF(LEFT($G44,4)="待确认：","待确认",IF(OR($A44="",$B44="",$C44="",$D44="",$E44=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B44))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A44))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E44="S",$E44="M",$E44="L")),"复杂度非法",IF(NOT(OR($F44="",$F44="内部集成",$F44="外部集成")),"集成类型非法",IF(AND($F44&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C44,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F44="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C44,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H44),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="45" ht="42" customHeight="1">
@@ -3382,7 +3382,7 @@
         <s:f>IF(COUNTA($A45:$G45)=0,"",IF($F45="",0,IF(NOT(ISNUMBER($I45)),"",IF($F45="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I45,1),IF($F45="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I45,1),"")))))</s:f>
       </s:c>
       <s:c r="L45" t="str" s="5">
-        <s:f>IF(COUNTA($A45:$G45)=0,"",IF(OR($A45="",$B45="",$C45="",$D45="",$E45=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B45))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A45))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E45="S",$E45="M",$E45="L")),"复杂度非法",IF(NOT(OR($F45="",$F45="内部集成",$F45="外部集成")),"集成类型非法",IF(AND($F45&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C45,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F45="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C45,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H45),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A45:$G45)=0,"",IF(LEFT($G45,4)="待确认：","待确认",IF(OR($A45="",$B45="",$C45="",$D45="",$E45=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B45))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A45))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E45="S",$E45="M",$E45="L")),"复杂度非法",IF(NOT(OR($F45="",$F45="内部集成",$F45="外部集成")),"集成类型非法",IF(AND($F45&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C45,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F45="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C45,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H45),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="46" ht="42" customHeight="1">
@@ -3406,7 +3406,7 @@
         <s:f>IF(COUNTA($A46:$G46)=0,"",IF($F46="",0,IF(NOT(ISNUMBER($I46)),"",IF($F46="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I46,1),IF($F46="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I46,1),"")))))</s:f>
       </s:c>
       <s:c r="L46" t="str" s="5">
-        <s:f>IF(COUNTA($A46:$G46)=0,"",IF(OR($A46="",$B46="",$C46="",$D46="",$E46=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B46))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A46))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E46="S",$E46="M",$E46="L")),"复杂度非法",IF(NOT(OR($F46="",$F46="内部集成",$F46="外部集成")),"集成类型非法",IF(AND($F46&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C46,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F46="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C46,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H46),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A46:$G46)=0,"",IF(LEFT($G46,4)="待确认：","待确认",IF(OR($A46="",$B46="",$C46="",$D46="",$E46=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B46))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A46))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E46="S",$E46="M",$E46="L")),"复杂度非法",IF(NOT(OR($F46="",$F46="内部集成",$F46="外部集成")),"集成类型非法",IF(AND($F46&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C46,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F46="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C46,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H46),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="47" ht="42" customHeight="1">
@@ -3430,7 +3430,7 @@
         <s:f>IF(COUNTA($A47:$G47)=0,"",IF($F47="",0,IF(NOT(ISNUMBER($I47)),"",IF($F47="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I47,1),IF($F47="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I47,1),"")))))</s:f>
       </s:c>
       <s:c r="L47" t="str" s="5">
-        <s:f>IF(COUNTA($A47:$G47)=0,"",IF(OR($A47="",$B47="",$C47="",$D47="",$E47=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B47))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A47))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E47="S",$E47="M",$E47="L")),"复杂度非法",IF(NOT(OR($F47="",$F47="内部集成",$F47="外部集成")),"集成类型非法",IF(AND($F47&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C47,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F47="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C47,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H47),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A47:$G47)=0,"",IF(LEFT($G47,4)="待确认：","待确认",IF(OR($A47="",$B47="",$C47="",$D47="",$E47=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B47))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A47))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E47="S",$E47="M",$E47="L")),"复杂度非法",IF(NOT(OR($F47="",$F47="内部集成",$F47="外部集成")),"集成类型非法",IF(AND($F47&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C47,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F47="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C47,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H47),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="48" ht="42" customHeight="1">
@@ -3454,7 +3454,7 @@
         <s:f>IF(COUNTA($A48:$G48)=0,"",IF($F48="",0,IF(NOT(ISNUMBER($I48)),"",IF($F48="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I48,1),IF($F48="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I48,1),"")))))</s:f>
       </s:c>
       <s:c r="L48" t="str" s="5">
-        <s:f>IF(COUNTA($A48:$G48)=0,"",IF(OR($A48="",$B48="",$C48="",$D48="",$E48=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B48))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A48))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E48="S",$E48="M",$E48="L")),"复杂度非法",IF(NOT(OR($F48="",$F48="内部集成",$F48="外部集成")),"集成类型非法",IF(AND($F48&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C48,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F48="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C48,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H48),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A48:$G48)=0,"",IF(LEFT($G48,4)="待确认：","待确认",IF(OR($A48="",$B48="",$C48="",$D48="",$E48=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B48))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A48))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E48="S",$E48="M",$E48="L")),"复杂度非法",IF(NOT(OR($F48="",$F48="内部集成",$F48="外部集成")),"集成类型非法",IF(AND($F48&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C48,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F48="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C48,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H48),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="49" ht="42" customHeight="1">
@@ -3478,7 +3478,7 @@
         <s:f>IF(COUNTA($A49:$G49)=0,"",IF($F49="",0,IF(NOT(ISNUMBER($I49)),"",IF($F49="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I49,1),IF($F49="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I49,1),"")))))</s:f>
       </s:c>
       <s:c r="L49" t="str" s="5">
-        <s:f>IF(COUNTA($A49:$G49)=0,"",IF(OR($A49="",$B49="",$C49="",$D49="",$E49=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B49))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A49))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E49="S",$E49="M",$E49="L")),"复杂度非法",IF(NOT(OR($F49="",$F49="内部集成",$F49="外部集成")),"集成类型非法",IF(AND($F49&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C49,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F49="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C49,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H49),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A49:$G49)=0,"",IF(LEFT($G49,4)="待确认：","待确认",IF(OR($A49="",$B49="",$C49="",$D49="",$E49=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B49))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A49))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E49="S",$E49="M",$E49="L")),"复杂度非法",IF(NOT(OR($F49="",$F49="内部集成",$F49="外部集成")),"集成类型非法",IF(AND($F49&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C49,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F49="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C49,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H49),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="50" ht="42" customHeight="1">
@@ -3502,7 +3502,7 @@
         <s:f>IF(COUNTA($A50:$G50)=0,"",IF($F50="",0,IF(NOT(ISNUMBER($I50)),"",IF($F50="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I50,1),IF($F50="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I50,1),"")))))</s:f>
       </s:c>
       <s:c r="L50" t="str" s="5">
-        <s:f>IF(COUNTA($A50:$G50)=0,"",IF(OR($A50="",$B50="",$C50="",$D50="",$E50=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B50))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A50))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E50="S",$E50="M",$E50="L")),"复杂度非法",IF(NOT(OR($F50="",$F50="内部集成",$F50="外部集成")),"集成类型非法",IF(AND($F50&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C50,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F50="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C50,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H50),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A50:$G50)=0,"",IF(LEFT($G50,4)="待确认：","待确认",IF(OR($A50="",$B50="",$C50="",$D50="",$E50=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B50))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A50))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E50="S",$E50="M",$E50="L")),"复杂度非法",IF(NOT(OR($F50="",$F50="内部集成",$F50="外部集成")),"集成类型非法",IF(AND($F50&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C50,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F50="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C50,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H50),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="51" ht="42" customHeight="1">
@@ -3526,7 +3526,7 @@
         <s:f>IF(COUNTA($A51:$G51)=0,"",IF($F51="",0,IF(NOT(ISNUMBER($I51)),"",IF($F51="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I51,1),IF($F51="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I51,1),"")))))</s:f>
       </s:c>
       <s:c r="L51" t="str" s="5">
-        <s:f>IF(COUNTA($A51:$G51)=0,"",IF(OR($A51="",$B51="",$C51="",$D51="",$E51=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B51))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A51))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E51="S",$E51="M",$E51="L")),"复杂度非法",IF(NOT(OR($F51="",$F51="内部集成",$F51="外部集成")),"集成类型非法",IF(AND($F51&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C51,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F51="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C51,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H51),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A51:$G51)=0,"",IF(LEFT($G51,4)="待确认：","待确认",IF(OR($A51="",$B51="",$C51="",$D51="",$E51=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B51))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A51))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E51="S",$E51="M",$E51="L")),"复杂度非法",IF(NOT(OR($F51="",$F51="内部集成",$F51="外部集成")),"集成类型非法",IF(AND($F51&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C51,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F51="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C51,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H51),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="52" ht="42" customHeight="1">
@@ -3550,7 +3550,7 @@
         <s:f>IF(COUNTA($A52:$G52)=0,"",IF($F52="",0,IF(NOT(ISNUMBER($I52)),"",IF($F52="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I52,1),IF($F52="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I52,1),"")))))</s:f>
       </s:c>
       <s:c r="L52" t="str" s="5">
-        <s:f>IF(COUNTA($A52:$G52)=0,"",IF(OR($A52="",$B52="",$C52="",$D52="",$E52=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B52))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A52))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E52="S",$E52="M",$E52="L")),"复杂度非法",IF(NOT(OR($F52="",$F52="内部集成",$F52="外部集成")),"集成类型非法",IF(AND($F52&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C52,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F52="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C52,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H52),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A52:$G52)=0,"",IF(LEFT($G52,4)="待确认：","待确认",IF(OR($A52="",$B52="",$C52="",$D52="",$E52=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B52))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A52))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E52="S",$E52="M",$E52="L")),"复杂度非法",IF(NOT(OR($F52="",$F52="内部集成",$F52="外部集成")),"集成类型非法",IF(AND($F52&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C52,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F52="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C52,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H52),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="53" ht="42" customHeight="1">
@@ -3574,7 +3574,7 @@
         <s:f>IF(COUNTA($A53:$G53)=0,"",IF($F53="",0,IF(NOT(ISNUMBER($I53)),"",IF($F53="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I53,1),IF($F53="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I53,1),"")))))</s:f>
       </s:c>
       <s:c r="L53" t="str" s="5">
-        <s:f>IF(COUNTA($A53:$G53)=0,"",IF(OR($A53="",$B53="",$C53="",$D53="",$E53=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B53))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A53))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E53="S",$E53="M",$E53="L")),"复杂度非法",IF(NOT(OR($F53="",$F53="内部集成",$F53="外部集成")),"集成类型非法",IF(AND($F53&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C53,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F53="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C53,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H53),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A53:$G53)=0,"",IF(LEFT($G53,4)="待确认：","待确认",IF(OR($A53="",$B53="",$C53="",$D53="",$E53=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B53))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A53))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E53="S",$E53="M",$E53="L")),"复杂度非法",IF(NOT(OR($F53="",$F53="内部集成",$F53="外部集成")),"集成类型非法",IF(AND($F53&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C53,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F53="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C53,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H53),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="54" ht="42" customHeight="1">
@@ -3598,7 +3598,7 @@
         <s:f>IF(COUNTA($A54:$G54)=0,"",IF($F54="",0,IF(NOT(ISNUMBER($I54)),"",IF($F54="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I54,1),IF($F54="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I54,1),"")))))</s:f>
       </s:c>
       <s:c r="L54" t="str" s="5">
-        <s:f>IF(COUNTA($A54:$G54)=0,"",IF(OR($A54="",$B54="",$C54="",$D54="",$E54=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B54))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A54))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E54="S",$E54="M",$E54="L")),"复杂度非法",IF(NOT(OR($F54="",$F54="内部集成",$F54="外部集成")),"集成类型非法",IF(AND($F54&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C54,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F54="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C54,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H54),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A54:$G54)=0,"",IF(LEFT($G54,4)="待确认：","待确认",IF(OR($A54="",$B54="",$C54="",$D54="",$E54=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B54))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A54))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E54="S",$E54="M",$E54="L")),"复杂度非法",IF(NOT(OR($F54="",$F54="内部集成",$F54="外部集成")),"集成类型非法",IF(AND($F54&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C54,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F54="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C54,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H54),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="55" ht="42" customHeight="1">
@@ -3622,7 +3622,7 @@
         <s:f>IF(COUNTA($A55:$G55)=0,"",IF($F55="",0,IF(NOT(ISNUMBER($I55)),"",IF($F55="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I55,1),IF($F55="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I55,1),"")))))</s:f>
       </s:c>
       <s:c r="L55" t="str" s="5">
-        <s:f>IF(COUNTA($A55:$G55)=0,"",IF(OR($A55="",$B55="",$C55="",$D55="",$E55=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B55))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A55))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E55="S",$E55="M",$E55="L")),"复杂度非法",IF(NOT(OR($F55="",$F55="内部集成",$F55="外部集成")),"集成类型非法",IF(AND($F55&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C55,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F55="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C55,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H55),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A55:$G55)=0,"",IF(LEFT($G55,4)="待确认：","待确认",IF(OR($A55="",$B55="",$C55="",$D55="",$E55=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B55))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A55))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E55="S",$E55="M",$E55="L")),"复杂度非法",IF(NOT(OR($F55="",$F55="内部集成",$F55="外部集成")),"集成类型非法",IF(AND($F55&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C55,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F55="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C55,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H55),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="56" ht="42" customHeight="1">
@@ -3646,7 +3646,7 @@
         <s:f>IF(COUNTA($A56:$G56)=0,"",IF($F56="",0,IF(NOT(ISNUMBER($I56)),"",IF($F56="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I56,1),IF($F56="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I56,1),"")))))</s:f>
       </s:c>
       <s:c r="L56" t="str" s="5">
-        <s:f>IF(COUNTA($A56:$G56)=0,"",IF(OR($A56="",$B56="",$C56="",$D56="",$E56=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B56))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A56))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E56="S",$E56="M",$E56="L")),"复杂度非法",IF(NOT(OR($F56="",$F56="内部集成",$F56="外部集成")),"集成类型非法",IF(AND($F56&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C56,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F56="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C56,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H56),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A56:$G56)=0,"",IF(LEFT($G56,4)="待确认：","待确认",IF(OR($A56="",$B56="",$C56="",$D56="",$E56=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B56))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A56))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E56="S",$E56="M",$E56="L")),"复杂度非法",IF(NOT(OR($F56="",$F56="内部集成",$F56="外部集成")),"集成类型非法",IF(AND($F56&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C56,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F56="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C56,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H56),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="57" ht="42" customHeight="1">
@@ -3670,7 +3670,7 @@
         <s:f>IF(COUNTA($A57:$G57)=0,"",IF($F57="",0,IF(NOT(ISNUMBER($I57)),"",IF($F57="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I57,1),IF($F57="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I57,1),"")))))</s:f>
       </s:c>
       <s:c r="L57" t="str" s="5">
-        <s:f>IF(COUNTA($A57:$G57)=0,"",IF(OR($A57="",$B57="",$C57="",$D57="",$E57=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B57))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A57))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E57="S",$E57="M",$E57="L")),"复杂度非法",IF(NOT(OR($F57="",$F57="内部集成",$F57="外部集成")),"集成类型非法",IF(AND($F57&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C57,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F57="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C57,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H57),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A57:$G57)=0,"",IF(LEFT($G57,4)="待确认：","待确认",IF(OR($A57="",$B57="",$C57="",$D57="",$E57=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B57))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A57))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E57="S",$E57="M",$E57="L")),"复杂度非法",IF(NOT(OR($F57="",$F57="内部集成",$F57="外部集成")),"集成类型非法",IF(AND($F57&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C57,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F57="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C57,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H57),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="58" ht="42" customHeight="1">
@@ -3694,7 +3694,7 @@
         <s:f>IF(COUNTA($A58:$G58)=0,"",IF($F58="",0,IF(NOT(ISNUMBER($I58)),"",IF($F58="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I58,1),IF($F58="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I58,1),"")))))</s:f>
       </s:c>
       <s:c r="L58" t="str" s="5">
-        <s:f>IF(COUNTA($A58:$G58)=0,"",IF(OR($A58="",$B58="",$C58="",$D58="",$E58=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B58))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A58))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E58="S",$E58="M",$E58="L")),"复杂度非法",IF(NOT(OR($F58="",$F58="内部集成",$F58="外部集成")),"集成类型非法",IF(AND($F58&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C58,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F58="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C58,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H58),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A58:$G58)=0,"",IF(LEFT($G58,4)="待确认：","待确认",IF(OR($A58="",$B58="",$C58="",$D58="",$E58=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B58))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A58))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E58="S",$E58="M",$E58="L")),"复杂度非法",IF(NOT(OR($F58="",$F58="内部集成",$F58="外部集成")),"集成类型非法",IF(AND($F58&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C58,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F58="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C58,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H58),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="59" ht="42" customHeight="1">
@@ -3718,7 +3718,7 @@
         <s:f>IF(COUNTA($A59:$G59)=0,"",IF($F59="",0,IF(NOT(ISNUMBER($I59)),"",IF($F59="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I59,1),IF($F59="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I59,1),"")))))</s:f>
       </s:c>
       <s:c r="L59" t="str" s="5">
-        <s:f>IF(COUNTA($A59:$G59)=0,"",IF(OR($A59="",$B59="",$C59="",$D59="",$E59=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B59))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A59))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E59="S",$E59="M",$E59="L")),"复杂度非法",IF(NOT(OR($F59="",$F59="内部集成",$F59="外部集成")),"集成类型非法",IF(AND($F59&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C59,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F59="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C59,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H59),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A59:$G59)=0,"",IF(LEFT($G59,4)="待确认：","待确认",IF(OR($A59="",$B59="",$C59="",$D59="",$E59=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B59))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A59))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E59="S",$E59="M",$E59="L")),"复杂度非法",IF(NOT(OR($F59="",$F59="内部集成",$F59="外部集成")),"集成类型非法",IF(AND($F59&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C59,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F59="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C59,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H59),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="60" ht="42" customHeight="1">
@@ -3742,7 +3742,7 @@
         <s:f>IF(COUNTA($A60:$G60)=0,"",IF($F60="",0,IF(NOT(ISNUMBER($I60)),"",IF($F60="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I60,1),IF($F60="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I60,1),"")))))</s:f>
       </s:c>
       <s:c r="L60" t="str" s="5">
-        <s:f>IF(COUNTA($A60:$G60)=0,"",IF(OR($A60="",$B60="",$C60="",$D60="",$E60=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B60))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A60))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E60="S",$E60="M",$E60="L")),"复杂度非法",IF(NOT(OR($F60="",$F60="内部集成",$F60="外部集成")),"集成类型非法",IF(AND($F60&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C60,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F60="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C60,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H60),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A60:$G60)=0,"",IF(LEFT($G60,4)="待确认：","待确认",IF(OR($A60="",$B60="",$C60="",$D60="",$E60=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B60))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A60))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E60="S",$E60="M",$E60="L")),"复杂度非法",IF(NOT(OR($F60="",$F60="内部集成",$F60="外部集成")),"集成类型非法",IF(AND($F60&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C60,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F60="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C60,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H60),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="61" ht="42" customHeight="1">
@@ -3766,7 +3766,7 @@
         <s:f>IF(COUNTA($A61:$G61)=0,"",IF($F61="",0,IF(NOT(ISNUMBER($I61)),"",IF($F61="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I61,1),IF($F61="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I61,1),"")))))</s:f>
       </s:c>
       <s:c r="L61" t="str" s="5">
-        <s:f>IF(COUNTA($A61:$G61)=0,"",IF(OR($A61="",$B61="",$C61="",$D61="",$E61=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B61))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A61))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E61="S",$E61="M",$E61="L")),"复杂度非法",IF(NOT(OR($F61="",$F61="内部集成",$F61="外部集成")),"集成类型非法",IF(AND($F61&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C61,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F61="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C61,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H61),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A61:$G61)=0,"",IF(LEFT($G61,4)="待确认：","待确认",IF(OR($A61="",$B61="",$C61="",$D61="",$E61=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B61))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A61))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E61="S",$E61="M",$E61="L")),"复杂度非法",IF(NOT(OR($F61="",$F61="内部集成",$F61="外部集成")),"集成类型非法",IF(AND($F61&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C61,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F61="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C61,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H61),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="62" ht="42" customHeight="1">
@@ -3790,7 +3790,7 @@
         <s:f>IF(COUNTA($A62:$G62)=0,"",IF($F62="",0,IF(NOT(ISNUMBER($I62)),"",IF($F62="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I62,1),IF($F62="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I62,1),"")))))</s:f>
       </s:c>
       <s:c r="L62" t="str" s="5">
-        <s:f>IF(COUNTA($A62:$G62)=0,"",IF(OR($A62="",$B62="",$C62="",$D62="",$E62=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B62))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A62))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E62="S",$E62="M",$E62="L")),"复杂度非法",IF(NOT(OR($F62="",$F62="内部集成",$F62="外部集成")),"集成类型非法",IF(AND($F62&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C62,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F62="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C62,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H62),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A62:$G62)=0,"",IF(LEFT($G62,4)="待确认：","待确认",IF(OR($A62="",$B62="",$C62="",$D62="",$E62=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B62))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A62))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E62="S",$E62="M",$E62="L")),"复杂度非法",IF(NOT(OR($F62="",$F62="内部集成",$F62="外部集成")),"集成类型非法",IF(AND($F62&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C62,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F62="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C62,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H62),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="63" ht="42" customHeight="1">
@@ -3814,7 +3814,7 @@
         <s:f>IF(COUNTA($A63:$G63)=0,"",IF($F63="",0,IF(NOT(ISNUMBER($I63)),"",IF($F63="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I63,1),IF($F63="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I63,1),"")))))</s:f>
       </s:c>
       <s:c r="L63" t="str" s="5">
-        <s:f>IF(COUNTA($A63:$G63)=0,"",IF(OR($A63="",$B63="",$C63="",$D63="",$E63=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B63))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A63))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E63="S",$E63="M",$E63="L")),"复杂度非法",IF(NOT(OR($F63="",$F63="内部集成",$F63="外部集成")),"集成类型非法",IF(AND($F63&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C63,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F63="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C63,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H63),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A63:$G63)=0,"",IF(LEFT($G63,4)="待确认：","待确认",IF(OR($A63="",$B63="",$C63="",$D63="",$E63=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B63))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A63))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E63="S",$E63="M",$E63="L")),"复杂度非法",IF(NOT(OR($F63="",$F63="内部集成",$F63="外部集成")),"集成类型非法",IF(AND($F63&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C63,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F63="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C63,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H63),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="64" ht="42" customHeight="1">
@@ -3838,7 +3838,7 @@
         <s:f>IF(COUNTA($A64:$G64)=0,"",IF($F64="",0,IF(NOT(ISNUMBER($I64)),"",IF($F64="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I64,1),IF($F64="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I64,1),"")))))</s:f>
       </s:c>
       <s:c r="L64" t="str" s="5">
-        <s:f>IF(COUNTA($A64:$G64)=0,"",IF(OR($A64="",$B64="",$C64="",$D64="",$E64=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B64))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A64))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E64="S",$E64="M",$E64="L")),"复杂度非法",IF(NOT(OR($F64="",$F64="内部集成",$F64="外部集成")),"集成类型非法",IF(AND($F64&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C64,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F64="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C64,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H64),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A64:$G64)=0,"",IF(LEFT($G64,4)="待确认：","待确认",IF(OR($A64="",$B64="",$C64="",$D64="",$E64=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B64))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A64))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E64="S",$E64="M",$E64="L")),"复杂度非法",IF(NOT(OR($F64="",$F64="内部集成",$F64="外部集成")),"集成类型非法",IF(AND($F64&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C64,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F64="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C64,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H64),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="65" ht="42" customHeight="1">
@@ -3862,7 +3862,7 @@
         <s:f>IF(COUNTA($A65:$G65)=0,"",IF($F65="",0,IF(NOT(ISNUMBER($I65)),"",IF($F65="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I65,1),IF($F65="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I65,1),"")))))</s:f>
       </s:c>
       <s:c r="L65" t="str" s="5">
-        <s:f>IF(COUNTA($A65:$G65)=0,"",IF(OR($A65="",$B65="",$C65="",$D65="",$E65=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B65))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A65))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E65="S",$E65="M",$E65="L")),"复杂度非法",IF(NOT(OR($F65="",$F65="内部集成",$F65="外部集成")),"集成类型非法",IF(AND($F65&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C65,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F65="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C65,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H65),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A65:$G65)=0,"",IF(LEFT($G65,4)="待确认：","待确认",IF(OR($A65="",$B65="",$C65="",$D65="",$E65=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B65))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A65))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E65="S",$E65="M",$E65="L")),"复杂度非法",IF(NOT(OR($F65="",$F65="内部集成",$F65="外部集成")),"集成类型非法",IF(AND($F65&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C65,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F65="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C65,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H65),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="66" ht="42" customHeight="1">
@@ -3886,7 +3886,7 @@
         <s:f>IF(COUNTA($A66:$G66)=0,"",IF($F66="",0,IF(NOT(ISNUMBER($I66)),"",IF($F66="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I66,1),IF($F66="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I66,1),"")))))</s:f>
       </s:c>
       <s:c r="L66" t="str" s="5">
-        <s:f>IF(COUNTA($A66:$G66)=0,"",IF(OR($A66="",$B66="",$C66="",$D66="",$E66=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B66))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A66))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E66="S",$E66="M",$E66="L")),"复杂度非法",IF(NOT(OR($F66="",$F66="内部集成",$F66="外部集成")),"集成类型非法",IF(AND($F66&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C66,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F66="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C66,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H66),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A66:$G66)=0,"",IF(LEFT($G66,4)="待确认：","待确认",IF(OR($A66="",$B66="",$C66="",$D66="",$E66=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B66))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A66))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E66="S",$E66="M",$E66="L")),"复杂度非法",IF(NOT(OR($F66="",$F66="内部集成",$F66="外部集成")),"集成类型非法",IF(AND($F66&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C66,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F66="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C66,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H66),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="67" ht="42" customHeight="1">
@@ -3910,7 +3910,7 @@
         <s:f>IF(COUNTA($A67:$G67)=0,"",IF($F67="",0,IF(NOT(ISNUMBER($I67)),"",IF($F67="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I67,1),IF($F67="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I67,1),"")))))</s:f>
       </s:c>
       <s:c r="L67" t="str" s="5">
-        <s:f>IF(COUNTA($A67:$G67)=0,"",IF(OR($A67="",$B67="",$C67="",$D67="",$E67=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B67))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A67))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E67="S",$E67="M",$E67="L")),"复杂度非法",IF(NOT(OR($F67="",$F67="内部集成",$F67="外部集成")),"集成类型非法",IF(AND($F67&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C67,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F67="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C67,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H67),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A67:$G67)=0,"",IF(LEFT($G67,4)="待确认：","待确认",IF(OR($A67="",$B67="",$C67="",$D67="",$E67=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B67))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A67))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E67="S",$E67="M",$E67="L")),"复杂度非法",IF(NOT(OR($F67="",$F67="内部集成",$F67="外部集成")),"集成类型非法",IF(AND($F67&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C67,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F67="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C67,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H67),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="68" ht="42" customHeight="1">
@@ -3934,7 +3934,7 @@
         <s:f>IF(COUNTA($A68:$G68)=0,"",IF($F68="",0,IF(NOT(ISNUMBER($I68)),"",IF($F68="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I68,1),IF($F68="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I68,1),"")))))</s:f>
       </s:c>
       <s:c r="L68" t="str" s="5">
-        <s:f>IF(COUNTA($A68:$G68)=0,"",IF(OR($A68="",$B68="",$C68="",$D68="",$E68=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B68))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A68))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E68="S",$E68="M",$E68="L")),"复杂度非法",IF(NOT(OR($F68="",$F68="内部集成",$F68="外部集成")),"集成类型非法",IF(AND($F68&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C68,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F68="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C68,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H68),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A68:$G68)=0,"",IF(LEFT($G68,4)="待确认：","待确认",IF(OR($A68="",$B68="",$C68="",$D68="",$E68=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B68))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A68))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E68="S",$E68="M",$E68="L")),"复杂度非法",IF(NOT(OR($F68="",$F68="内部集成",$F68="外部集成")),"集成类型非法",IF(AND($F68&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C68,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F68="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C68,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H68),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="69" ht="42" customHeight="1">
@@ -3958,7 +3958,7 @@
         <s:f>IF(COUNTA($A69:$G69)=0,"",IF($F69="",0,IF(NOT(ISNUMBER($I69)),"",IF($F69="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I69,1),IF($F69="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I69,1),"")))))</s:f>
       </s:c>
       <s:c r="L69" t="str" s="5">
-        <s:f>IF(COUNTA($A69:$G69)=0,"",IF(OR($A69="",$B69="",$C69="",$D69="",$E69=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B69))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A69))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E69="S",$E69="M",$E69="L")),"复杂度非法",IF(NOT(OR($F69="",$F69="内部集成",$F69="外部集成")),"集成类型非法",IF(AND($F69&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C69,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F69="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C69,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H69),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A69:$G69)=0,"",IF(LEFT($G69,4)="待确认：","待确认",IF(OR($A69="",$B69="",$C69="",$D69="",$E69=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B69))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A69))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E69="S",$E69="M",$E69="L")),"复杂度非法",IF(NOT(OR($F69="",$F69="内部集成",$F69="外部集成")),"集成类型非法",IF(AND($F69&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C69,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F69="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C69,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H69),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="70" ht="42" customHeight="1">
@@ -3982,7 +3982,7 @@
         <s:f>IF(COUNTA($A70:$G70)=0,"",IF($F70="",0,IF(NOT(ISNUMBER($I70)),"",IF($F70="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I70,1),IF($F70="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I70,1),"")))))</s:f>
       </s:c>
       <s:c r="L70" t="str" s="5">
-        <s:f>IF(COUNTA($A70:$G70)=0,"",IF(OR($A70="",$B70="",$C70="",$D70="",$E70=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B70))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A70))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E70="S",$E70="M",$E70="L")),"复杂度非法",IF(NOT(OR($F70="",$F70="内部集成",$F70="外部集成")),"集成类型非法",IF(AND($F70&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C70,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F70="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C70,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H70),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A70:$G70)=0,"",IF(LEFT($G70,4)="待确认：","待确认",IF(OR($A70="",$B70="",$C70="",$D70="",$E70=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B70))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A70))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E70="S",$E70="M",$E70="L")),"复杂度非法",IF(NOT(OR($F70="",$F70="内部集成",$F70="外部集成")),"集成类型非法",IF(AND($F70&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C70,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F70="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C70,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H70),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="71" ht="42" customHeight="1">
@@ -4006,7 +4006,7 @@
         <s:f>IF(COUNTA($A71:$G71)=0,"",IF($F71="",0,IF(NOT(ISNUMBER($I71)),"",IF($F71="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I71,1),IF($F71="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I71,1),"")))))</s:f>
       </s:c>
       <s:c r="L71" t="str" s="5">
-        <s:f>IF(COUNTA($A71:$G71)=0,"",IF(OR($A71="",$B71="",$C71="",$D71="",$E71=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B71))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A71))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E71="S",$E71="M",$E71="L")),"复杂度非法",IF(NOT(OR($F71="",$F71="内部集成",$F71="外部集成")),"集成类型非法",IF(AND($F71&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C71,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F71="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C71,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H71),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A71:$G71)=0,"",IF(LEFT($G71,4)="待确认：","待确认",IF(OR($A71="",$B71="",$C71="",$D71="",$E71=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B71))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A71))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E71="S",$E71="M",$E71="L")),"复杂度非法",IF(NOT(OR($F71="",$F71="内部集成",$F71="外部集成")),"集成类型非法",IF(AND($F71&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C71,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F71="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C71,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H71),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="72" ht="42" customHeight="1">
@@ -4030,7 +4030,7 @@
         <s:f>IF(COUNTA($A72:$G72)=0,"",IF($F72="",0,IF(NOT(ISNUMBER($I72)),"",IF($F72="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I72,1),IF($F72="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I72,1),"")))))</s:f>
       </s:c>
       <s:c r="L72" t="str" s="5">
-        <s:f>IF(COUNTA($A72:$G72)=0,"",IF(OR($A72="",$B72="",$C72="",$D72="",$E72=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B72))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A72))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E72="S",$E72="M",$E72="L")),"复杂度非法",IF(NOT(OR($F72="",$F72="内部集成",$F72="外部集成")),"集成类型非法",IF(AND($F72&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C72,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F72="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C72,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H72),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A72:$G72)=0,"",IF(LEFT($G72,4)="待确认：","待确认",IF(OR($A72="",$B72="",$C72="",$D72="",$E72=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B72))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A72))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E72="S",$E72="M",$E72="L")),"复杂度非法",IF(NOT(OR($F72="",$F72="内部集成",$F72="外部集成")),"集成类型非法",IF(AND($F72&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C72,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F72="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C72,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H72),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="73" ht="42" customHeight="1">
@@ -4054,7 +4054,7 @@
         <s:f>IF(COUNTA($A73:$G73)=0,"",IF($F73="",0,IF(NOT(ISNUMBER($I73)),"",IF($F73="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I73,1),IF($F73="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I73,1),"")))))</s:f>
       </s:c>
       <s:c r="L73" t="str" s="5">
-        <s:f>IF(COUNTA($A73:$G73)=0,"",IF(OR($A73="",$B73="",$C73="",$D73="",$E73=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B73))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A73))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E73="S",$E73="M",$E73="L")),"复杂度非法",IF(NOT(OR($F73="",$F73="内部集成",$F73="外部集成")),"集成类型非法",IF(AND($F73&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C73,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F73="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C73,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H73),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A73:$G73)=0,"",IF(LEFT($G73,4)="待确认：","待确认",IF(OR($A73="",$B73="",$C73="",$D73="",$E73=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B73))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A73))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E73="S",$E73="M",$E73="L")),"复杂度非法",IF(NOT(OR($F73="",$F73="内部集成",$F73="外部集成")),"集成类型非法",IF(AND($F73&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C73,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F73="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C73,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H73),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="74" ht="42" customHeight="1">
@@ -4078,7 +4078,7 @@
         <s:f>IF(COUNTA($A74:$G74)=0,"",IF($F74="",0,IF(NOT(ISNUMBER($I74)),"",IF($F74="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I74,1),IF($F74="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I74,1),"")))))</s:f>
       </s:c>
       <s:c r="L74" t="str" s="5">
-        <s:f>IF(COUNTA($A74:$G74)=0,"",IF(OR($A74="",$B74="",$C74="",$D74="",$E74=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B74))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A74))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E74="S",$E74="M",$E74="L")),"复杂度非法",IF(NOT(OR($F74="",$F74="内部集成",$F74="外部集成")),"集成类型非法",IF(AND($F74&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C74,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F74="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C74,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H74),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A74:$G74)=0,"",IF(LEFT($G74,4)="待确认：","待确认",IF(OR($A74="",$B74="",$C74="",$D74="",$E74=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B74))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A74))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E74="S",$E74="M",$E74="L")),"复杂度非法",IF(NOT(OR($F74="",$F74="内部集成",$F74="外部集成")),"集成类型非法",IF(AND($F74&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C74,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F74="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C74,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H74),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="75" ht="42" customHeight="1">
@@ -4102,7 +4102,7 @@
         <s:f>IF(COUNTA($A75:$G75)=0,"",IF($F75="",0,IF(NOT(ISNUMBER($I75)),"",IF($F75="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I75,1),IF($F75="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I75,1),"")))))</s:f>
       </s:c>
       <s:c r="L75" t="str" s="5">
-        <s:f>IF(COUNTA($A75:$G75)=0,"",IF(OR($A75="",$B75="",$C75="",$D75="",$E75=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B75))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A75))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E75="S",$E75="M",$E75="L")),"复杂度非法",IF(NOT(OR($F75="",$F75="内部集成",$F75="外部集成")),"集成类型非法",IF(AND($F75&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C75,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F75="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C75,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H75),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A75:$G75)=0,"",IF(LEFT($G75,4)="待确认：","待确认",IF(OR($A75="",$B75="",$C75="",$D75="",$E75=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B75))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A75))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E75="S",$E75="M",$E75="L")),"复杂度非法",IF(NOT(OR($F75="",$F75="内部集成",$F75="外部集成")),"集成类型非法",IF(AND($F75&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C75,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F75="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C75,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H75),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="76" ht="42" customHeight="1">
@@ -4126,7 +4126,7 @@
         <s:f>IF(COUNTA($A76:$G76)=0,"",IF($F76="",0,IF(NOT(ISNUMBER($I76)),"",IF($F76="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I76,1),IF($F76="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I76,1),"")))))</s:f>
       </s:c>
       <s:c r="L76" t="str" s="5">
-        <s:f>IF(COUNTA($A76:$G76)=0,"",IF(OR($A76="",$B76="",$C76="",$D76="",$E76=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B76))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A76))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E76="S",$E76="M",$E76="L")),"复杂度非法",IF(NOT(OR($F76="",$F76="内部集成",$F76="外部集成")),"集成类型非法",IF(AND($F76&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C76,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F76="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C76,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H76),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A76:$G76)=0,"",IF(LEFT($G76,4)="待确认：","待确认",IF(OR($A76="",$B76="",$C76="",$D76="",$E76=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B76))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A76))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E76="S",$E76="M",$E76="L")),"复杂度非法",IF(NOT(OR($F76="",$F76="内部集成",$F76="外部集成")),"集成类型非法",IF(AND($F76&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C76,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F76="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C76,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H76),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="77" ht="42" customHeight="1">
@@ -4150,7 +4150,7 @@
         <s:f>IF(COUNTA($A77:$G77)=0,"",IF($F77="",0,IF(NOT(ISNUMBER($I77)),"",IF($F77="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I77,1),IF($F77="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I77,1),"")))))</s:f>
       </s:c>
       <s:c r="L77" t="str" s="5">
-        <s:f>IF(COUNTA($A77:$G77)=0,"",IF(OR($A77="",$B77="",$C77="",$D77="",$E77=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B77))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A77))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E77="S",$E77="M",$E77="L")),"复杂度非法",IF(NOT(OR($F77="",$F77="内部集成",$F77="外部集成")),"集成类型非法",IF(AND($F77&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C77,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F77="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C77,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H77),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A77:$G77)=0,"",IF(LEFT($G77,4)="待确认：","待确认",IF(OR($A77="",$B77="",$C77="",$D77="",$E77=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B77))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A77))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E77="S",$E77="M",$E77="L")),"复杂度非法",IF(NOT(OR($F77="",$F77="内部集成",$F77="外部集成")),"集成类型非法",IF(AND($F77&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C77,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F77="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C77,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H77),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="78" ht="42" customHeight="1">
@@ -4174,7 +4174,7 @@
         <s:f>IF(COUNTA($A78:$G78)=0,"",IF($F78="",0,IF(NOT(ISNUMBER($I78)),"",IF($F78="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I78,1),IF($F78="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I78,1),"")))))</s:f>
       </s:c>
       <s:c r="L78" t="str" s="5">
-        <s:f>IF(COUNTA($A78:$G78)=0,"",IF(OR($A78="",$B78="",$C78="",$D78="",$E78=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B78))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A78))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E78="S",$E78="M",$E78="L")),"复杂度非法",IF(NOT(OR($F78="",$F78="内部集成",$F78="外部集成")),"集成类型非法",IF(AND($F78&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C78,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F78="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C78,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H78),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A78:$G78)=0,"",IF(LEFT($G78,4)="待确认：","待确认",IF(OR($A78="",$B78="",$C78="",$D78="",$E78=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B78))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A78))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E78="S",$E78="M",$E78="L")),"复杂度非法",IF(NOT(OR($F78="",$F78="内部集成",$F78="外部集成")),"集成类型非法",IF(AND($F78&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C78,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F78="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C78,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H78),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="79" ht="42" customHeight="1">
@@ -4198,7 +4198,7 @@
         <s:f>IF(COUNTA($A79:$G79)=0,"",IF($F79="",0,IF(NOT(ISNUMBER($I79)),"",IF($F79="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I79,1),IF($F79="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I79,1),"")))))</s:f>
       </s:c>
       <s:c r="L79" t="str" s="5">
-        <s:f>IF(COUNTA($A79:$G79)=0,"",IF(OR($A79="",$B79="",$C79="",$D79="",$E79=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B79))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A79))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E79="S",$E79="M",$E79="L")),"复杂度非法",IF(NOT(OR($F79="",$F79="内部集成",$F79="外部集成")),"集成类型非法",IF(AND($F79&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C79,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F79="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C79,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H79),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A79:$G79)=0,"",IF(LEFT($G79,4)="待确认：","待确认",IF(OR($A79="",$B79="",$C79="",$D79="",$E79=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B79))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A79))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E79="S",$E79="M",$E79="L")),"复杂度非法",IF(NOT(OR($F79="",$F79="内部集成",$F79="外部集成")),"集成类型非法",IF(AND($F79&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C79,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F79="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C79,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H79),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="80" ht="42" customHeight="1">
@@ -4222,7 +4222,7 @@
         <s:f>IF(COUNTA($A80:$G80)=0,"",IF($F80="",0,IF(NOT(ISNUMBER($I80)),"",IF($F80="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I80,1),IF($F80="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I80,1),"")))))</s:f>
       </s:c>
       <s:c r="L80" t="str" s="5">
-        <s:f>IF(COUNTA($A80:$G80)=0,"",IF(OR($A80="",$B80="",$C80="",$D80="",$E80=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B80))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A80))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E80="S",$E80="M",$E80="L")),"复杂度非法",IF(NOT(OR($F80="",$F80="内部集成",$F80="外部集成")),"集成类型非法",IF(AND($F80&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C80,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F80="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C80,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H80),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A80:$G80)=0,"",IF(LEFT($G80,4)="待确认：","待确认",IF(OR($A80="",$B80="",$C80="",$D80="",$E80=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B80))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A80))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E80="S",$E80="M",$E80="L")),"复杂度非法",IF(NOT(OR($F80="",$F80="内部集成",$F80="外部集成")),"集成类型非法",IF(AND($F80&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C80,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F80="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C80,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H80),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="81" ht="42" customHeight="1">
@@ -4246,7 +4246,7 @@
         <s:f>IF(COUNTA($A81:$G81)=0,"",IF($F81="",0,IF(NOT(ISNUMBER($I81)),"",IF($F81="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I81,1),IF($F81="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I81,1),"")))))</s:f>
       </s:c>
       <s:c r="L81" t="str" s="5">
-        <s:f>IF(COUNTA($A81:$G81)=0,"",IF(OR($A81="",$B81="",$C81="",$D81="",$E81=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B81))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A81))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E81="S",$E81="M",$E81="L")),"复杂度非法",IF(NOT(OR($F81="",$F81="内部集成",$F81="外部集成")),"集成类型非法",IF(AND($F81&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C81,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F81="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C81,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H81),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A81:$G81)=0,"",IF(LEFT($G81,4)="待确认：","待确认",IF(OR($A81="",$B81="",$C81="",$D81="",$E81=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B81))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A81))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E81="S",$E81="M",$E81="L")),"复杂度非法",IF(NOT(OR($F81="",$F81="内部集成",$F81="外部集成")),"集成类型非法",IF(AND($F81&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C81,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F81="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C81,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H81),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="82" ht="42" customHeight="1">
@@ -4270,7 +4270,7 @@
         <s:f>IF(COUNTA($A82:$G82)=0,"",IF($F82="",0,IF(NOT(ISNUMBER($I82)),"",IF($F82="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I82,1),IF($F82="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I82,1),"")))))</s:f>
       </s:c>
       <s:c r="L82" t="str" s="5">
-        <s:f>IF(COUNTA($A82:$G82)=0,"",IF(OR($A82="",$B82="",$C82="",$D82="",$E82=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B82))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A82))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E82="S",$E82="M",$E82="L")),"复杂度非法",IF(NOT(OR($F82="",$F82="内部集成",$F82="外部集成")),"集成类型非法",IF(AND($F82&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C82,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F82="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C82,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H82),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A82:$G82)=0,"",IF(LEFT($G82,4)="待确认：","待确认",IF(OR($A82="",$B82="",$C82="",$D82="",$E82=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B82))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A82))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E82="S",$E82="M",$E82="L")),"复杂度非法",IF(NOT(OR($F82="",$F82="内部集成",$F82="外部集成")),"集成类型非法",IF(AND($F82&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C82,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F82="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C82,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H82),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="83" ht="42" customHeight="1">
@@ -4294,7 +4294,7 @@
         <s:f>IF(COUNTA($A83:$G83)=0,"",IF($F83="",0,IF(NOT(ISNUMBER($I83)),"",IF($F83="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I83,1),IF($F83="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I83,1),"")))))</s:f>
       </s:c>
       <s:c r="L83" t="str" s="5">
-        <s:f>IF(COUNTA($A83:$G83)=0,"",IF(OR($A83="",$B83="",$C83="",$D83="",$E83=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B83))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A83))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E83="S",$E83="M",$E83="L")),"复杂度非法",IF(NOT(OR($F83="",$F83="内部集成",$F83="外部集成")),"集成类型非法",IF(AND($F83&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C83,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F83="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C83,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H83),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A83:$G83)=0,"",IF(LEFT($G83,4)="待确认：","待确认",IF(OR($A83="",$B83="",$C83="",$D83="",$E83=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B83))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A83))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E83="S",$E83="M",$E83="L")),"复杂度非法",IF(NOT(OR($F83="",$F83="内部集成",$F83="外部集成")),"集成类型非法",IF(AND($F83&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C83,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F83="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C83,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H83),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="84" ht="42" customHeight="1">
@@ -4318,7 +4318,7 @@
         <s:f>IF(COUNTA($A84:$G84)=0,"",IF($F84="",0,IF(NOT(ISNUMBER($I84)),"",IF($F84="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I84,1),IF($F84="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I84,1),"")))))</s:f>
       </s:c>
       <s:c r="L84" t="str" s="5">
-        <s:f>IF(COUNTA($A84:$G84)=0,"",IF(OR($A84="",$B84="",$C84="",$D84="",$E84=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B84))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A84))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E84="S",$E84="M",$E84="L")),"复杂度非法",IF(NOT(OR($F84="",$F84="内部集成",$F84="外部集成")),"集成类型非法",IF(AND($F84&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C84,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F84="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C84,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H84),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A84:$G84)=0,"",IF(LEFT($G84,4)="待确认：","待确认",IF(OR($A84="",$B84="",$C84="",$D84="",$E84=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B84))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A84))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E84="S",$E84="M",$E84="L")),"复杂度非法",IF(NOT(OR($F84="",$F84="内部集成",$F84="外部集成")),"集成类型非法",IF(AND($F84&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C84,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F84="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C84,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H84),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="85" ht="42" customHeight="1">
@@ -4342,7 +4342,7 @@
         <s:f>IF(COUNTA($A85:$G85)=0,"",IF($F85="",0,IF(NOT(ISNUMBER($I85)),"",IF($F85="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I85,1),IF($F85="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I85,1),"")))))</s:f>
       </s:c>
       <s:c r="L85" t="str" s="5">
-        <s:f>IF(COUNTA($A85:$G85)=0,"",IF(OR($A85="",$B85="",$C85="",$D85="",$E85=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B85))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A85))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E85="S",$E85="M",$E85="L")),"复杂度非法",IF(NOT(OR($F85="",$F85="内部集成",$F85="外部集成")),"集成类型非法",IF(AND($F85&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C85,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F85="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C85,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H85),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A85:$G85)=0,"",IF(LEFT($G85,4)="待确认：","待确认",IF(OR($A85="",$B85="",$C85="",$D85="",$E85=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B85))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A85))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E85="S",$E85="M",$E85="L")),"复杂度非法",IF(NOT(OR($F85="",$F85="内部集成",$F85="外部集成")),"集成类型非法",IF(AND($F85&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C85,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F85="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C85,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H85),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="86" ht="42" customHeight="1">
@@ -4366,7 +4366,7 @@
         <s:f>IF(COUNTA($A86:$G86)=0,"",IF($F86="",0,IF(NOT(ISNUMBER($I86)),"",IF($F86="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I86,1),IF($F86="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I86,1),"")))))</s:f>
       </s:c>
       <s:c r="L86" t="str" s="5">
-        <s:f>IF(COUNTA($A86:$G86)=0,"",IF(OR($A86="",$B86="",$C86="",$D86="",$E86=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B86))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A86))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E86="S",$E86="M",$E86="L")),"复杂度非法",IF(NOT(OR($F86="",$F86="内部集成",$F86="外部集成")),"集成类型非法",IF(AND($F86&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C86,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F86="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C86,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H86),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A86:$G86)=0,"",IF(LEFT($G86,4)="待确认：","待确认",IF(OR($A86="",$B86="",$C86="",$D86="",$E86=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B86))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A86))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E86="S",$E86="M",$E86="L")),"复杂度非法",IF(NOT(OR($F86="",$F86="内部集成",$F86="外部集成")),"集成类型非法",IF(AND($F86&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C86,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F86="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C86,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H86),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="87" ht="42" customHeight="1">
@@ -4390,7 +4390,7 @@
         <s:f>IF(COUNTA($A87:$G87)=0,"",IF($F87="",0,IF(NOT(ISNUMBER($I87)),"",IF($F87="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I87,1),IF($F87="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I87,1),"")))))</s:f>
       </s:c>
       <s:c r="L87" t="str" s="5">
-        <s:f>IF(COUNTA($A87:$G87)=0,"",IF(OR($A87="",$B87="",$C87="",$D87="",$E87=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B87))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A87))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E87="S",$E87="M",$E87="L")),"复杂度非法",IF(NOT(OR($F87="",$F87="内部集成",$F87="外部集成")),"集成类型非法",IF(AND($F87&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C87,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F87="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C87,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H87),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A87:$G87)=0,"",IF(LEFT($G87,4)="待确认：","待确认",IF(OR($A87="",$B87="",$C87="",$D87="",$E87=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B87))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A87))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E87="S",$E87="M",$E87="L")),"复杂度非法",IF(NOT(OR($F87="",$F87="内部集成",$F87="外部集成")),"集成类型非法",IF(AND($F87&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C87,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F87="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C87,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H87),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="88" ht="42" customHeight="1">
@@ -4414,7 +4414,7 @@
         <s:f>IF(COUNTA($A88:$G88)=0,"",IF($F88="",0,IF(NOT(ISNUMBER($I88)),"",IF($F88="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I88,1),IF($F88="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I88,1),"")))))</s:f>
       </s:c>
       <s:c r="L88" t="str" s="5">
-        <s:f>IF(COUNTA($A88:$G88)=0,"",IF(OR($A88="",$B88="",$C88="",$D88="",$E88=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B88))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A88))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E88="S",$E88="M",$E88="L")),"复杂度非法",IF(NOT(OR($F88="",$F88="内部集成",$F88="外部集成")),"集成类型非法",IF(AND($F88&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C88,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F88="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C88,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H88),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A88:$G88)=0,"",IF(LEFT($G88,4)="待确认：","待确认",IF(OR($A88="",$B88="",$C88="",$D88="",$E88=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B88))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A88))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E88="S",$E88="M",$E88="L")),"复杂度非法",IF(NOT(OR($F88="",$F88="内部集成",$F88="外部集成")),"集成类型非法",IF(AND($F88&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C88,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F88="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C88,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H88),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="89" ht="42" customHeight="1">
@@ -4438,7 +4438,7 @@
         <s:f>IF(COUNTA($A89:$G89)=0,"",IF($F89="",0,IF(NOT(ISNUMBER($I89)),"",IF($F89="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I89,1),IF($F89="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I89,1),"")))))</s:f>
       </s:c>
       <s:c r="L89" t="str" s="5">
-        <s:f>IF(COUNTA($A89:$G89)=0,"",IF(OR($A89="",$B89="",$C89="",$D89="",$E89=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B89))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A89))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E89="S",$E89="M",$E89="L")),"复杂度非法",IF(NOT(OR($F89="",$F89="内部集成",$F89="外部集成")),"集成类型非法",IF(AND($F89&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C89,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F89="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C89,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H89),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A89:$G89)=0,"",IF(LEFT($G89,4)="待确认：","待确认",IF(OR($A89="",$B89="",$C89="",$D89="",$E89=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B89))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A89))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E89="S",$E89="M",$E89="L")),"复杂度非法",IF(NOT(OR($F89="",$F89="内部集成",$F89="外部集成")),"集成类型非法",IF(AND($F89&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C89,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F89="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C89,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H89),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="90" ht="42" customHeight="1">
@@ -4462,7 +4462,7 @@
         <s:f>IF(COUNTA($A90:$G90)=0,"",IF($F90="",0,IF(NOT(ISNUMBER($I90)),"",IF($F90="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I90,1),IF($F90="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I90,1),"")))))</s:f>
       </s:c>
       <s:c r="L90" t="str" s="5">
-        <s:f>IF(COUNTA($A90:$G90)=0,"",IF(OR($A90="",$B90="",$C90="",$D90="",$E90=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B90))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A90))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E90="S",$E90="M",$E90="L")),"复杂度非法",IF(NOT(OR($F90="",$F90="内部集成",$F90="外部集成")),"集成类型非法",IF(AND($F90&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C90,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F90="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C90,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H90),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A90:$G90)=0,"",IF(LEFT($G90,4)="待确认：","待确认",IF(OR($A90="",$B90="",$C90="",$D90="",$E90=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B90))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A90))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E90="S",$E90="M",$E90="L")),"复杂度非法",IF(NOT(OR($F90="",$F90="内部集成",$F90="外部集成")),"集成类型非法",IF(AND($F90&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C90,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F90="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C90,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H90),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="91" ht="42" customHeight="1">
@@ -4486,7 +4486,7 @@
         <s:f>IF(COUNTA($A91:$G91)=0,"",IF($F91="",0,IF(NOT(ISNUMBER($I91)),"",IF($F91="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I91,1),IF($F91="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I91,1),"")))))</s:f>
       </s:c>
       <s:c r="L91" t="str" s="5">
-        <s:f>IF(COUNTA($A91:$G91)=0,"",IF(OR($A91="",$B91="",$C91="",$D91="",$E91=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B91))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A91))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E91="S",$E91="M",$E91="L")),"复杂度非法",IF(NOT(OR($F91="",$F91="内部集成",$F91="外部集成")),"集成类型非法",IF(AND($F91&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C91,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F91="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C91,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H91),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A91:$G91)=0,"",IF(LEFT($G91,4)="待确认：","待确认",IF(OR($A91="",$B91="",$C91="",$D91="",$E91=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B91))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A91))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E91="S",$E91="M",$E91="L")),"复杂度非法",IF(NOT(OR($F91="",$F91="内部集成",$F91="外部集成")),"集成类型非法",IF(AND($F91&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C91,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F91="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C91,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H91),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="92" ht="42" customHeight="1">
@@ -4510,7 +4510,7 @@
         <s:f>IF(COUNTA($A92:$G92)=0,"",IF($F92="",0,IF(NOT(ISNUMBER($I92)),"",IF($F92="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I92,1),IF($F92="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I92,1),"")))))</s:f>
       </s:c>
       <s:c r="L92" t="str" s="5">
-        <s:f>IF(COUNTA($A92:$G92)=0,"",IF(OR($A92="",$B92="",$C92="",$D92="",$E92=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B92))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A92))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E92="S",$E92="M",$E92="L")),"复杂度非法",IF(NOT(OR($F92="",$F92="内部集成",$F92="外部集成")),"集成类型非法",IF(AND($F92&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C92,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F92="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C92,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H92),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A92:$G92)=0,"",IF(LEFT($G92,4)="待确认：","待确认",IF(OR($A92="",$B92="",$C92="",$D92="",$E92=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B92))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A92))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E92="S",$E92="M",$E92="L")),"复杂度非法",IF(NOT(OR($F92="",$F92="内部集成",$F92="外部集成")),"集成类型非法",IF(AND($F92&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C92,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F92="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C92,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H92),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="93" ht="42" customHeight="1">
@@ -4534,7 +4534,7 @@
         <s:f>IF(COUNTA($A93:$G93)=0,"",IF($F93="",0,IF(NOT(ISNUMBER($I93)),"",IF($F93="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I93,1),IF($F93="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I93,1),"")))))</s:f>
       </s:c>
       <s:c r="L93" t="str" s="5">
-        <s:f>IF(COUNTA($A93:$G93)=0,"",IF(OR($A93="",$B93="",$C93="",$D93="",$E93=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B93))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A93))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E93="S",$E93="M",$E93="L")),"复杂度非法",IF(NOT(OR($F93="",$F93="内部集成",$F93="外部集成")),"集成类型非法",IF(AND($F93&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C93,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F93="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C93,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H93),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A93:$G93)=0,"",IF(LEFT($G93,4)="待确认：","待确认",IF(OR($A93="",$B93="",$C93="",$D93="",$E93=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B93))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A93))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E93="S",$E93="M",$E93="L")),"复杂度非法",IF(NOT(OR($F93="",$F93="内部集成",$F93="外部集成")),"集成类型非法",IF(AND($F93&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C93,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F93="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C93,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H93),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="94" ht="42" customHeight="1">
@@ -4558,7 +4558,7 @@
         <s:f>IF(COUNTA($A94:$G94)=0,"",IF($F94="",0,IF(NOT(ISNUMBER($I94)),"",IF($F94="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I94,1),IF($F94="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I94,1),"")))))</s:f>
       </s:c>
       <s:c r="L94" t="str" s="5">
-        <s:f>IF(COUNTA($A94:$G94)=0,"",IF(OR($A94="",$B94="",$C94="",$D94="",$E94=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B94))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A94))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E94="S",$E94="M",$E94="L")),"复杂度非法",IF(NOT(OR($F94="",$F94="内部集成",$F94="外部集成")),"集成类型非法",IF(AND($F94&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C94,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F94="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C94,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H94),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A94:$G94)=0,"",IF(LEFT($G94,4)="待确认：","待确认",IF(OR($A94="",$B94="",$C94="",$D94="",$E94=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B94))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A94))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E94="S",$E94="M",$E94="L")),"复杂度非法",IF(NOT(OR($F94="",$F94="内部集成",$F94="外部集成")),"集成类型非法",IF(AND($F94&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C94,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F94="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C94,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H94),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="95" ht="42" customHeight="1">
@@ -4582,7 +4582,7 @@
         <s:f>IF(COUNTA($A95:$G95)=0,"",IF($F95="",0,IF(NOT(ISNUMBER($I95)),"",IF($F95="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I95,1),IF($F95="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I95,1),"")))))</s:f>
       </s:c>
       <s:c r="L95" t="str" s="5">
-        <s:f>IF(COUNTA($A95:$G95)=0,"",IF(OR($A95="",$B95="",$C95="",$D95="",$E95=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B95))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A95))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E95="S",$E95="M",$E95="L")),"复杂度非法",IF(NOT(OR($F95="",$F95="内部集成",$F95="外部集成")),"集成类型非法",IF(AND($F95&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C95,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F95="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C95,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H95),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A95:$G95)=0,"",IF(LEFT($G95,4)="待确认：","待确认",IF(OR($A95="",$B95="",$C95="",$D95="",$E95=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B95))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A95))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E95="S",$E95="M",$E95="L")),"复杂度非法",IF(NOT(OR($F95="",$F95="内部集成",$F95="外部集成")),"集成类型非法",IF(AND($F95&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C95,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F95="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C95,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H95),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="96" ht="42" customHeight="1">
@@ -4606,7 +4606,7 @@
         <s:f>IF(COUNTA($A96:$G96)=0,"",IF($F96="",0,IF(NOT(ISNUMBER($I96)),"",IF($F96="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I96,1),IF($F96="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I96,1),"")))))</s:f>
       </s:c>
       <s:c r="L96" t="str" s="5">
-        <s:f>IF(COUNTA($A96:$G96)=0,"",IF(OR($A96="",$B96="",$C96="",$D96="",$E96=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B96))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A96))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E96="S",$E96="M",$E96="L")),"复杂度非法",IF(NOT(OR($F96="",$F96="内部集成",$F96="外部集成")),"集成类型非法",IF(AND($F96&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C96,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F96="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C96,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H96),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A96:$G96)=0,"",IF(LEFT($G96,4)="待确认：","待确认",IF(OR($A96="",$B96="",$C96="",$D96="",$E96=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B96))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A96))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E96="S",$E96="M",$E96="L")),"复杂度非法",IF(NOT(OR($F96="",$F96="内部集成",$F96="外部集成")),"集成类型非法",IF(AND($F96&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C96,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F96="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C96,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H96),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="97" ht="42" customHeight="1">
@@ -4630,7 +4630,7 @@
         <s:f>IF(COUNTA($A97:$G97)=0,"",IF($F97="",0,IF(NOT(ISNUMBER($I97)),"",IF($F97="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I97,1),IF($F97="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I97,1),"")))))</s:f>
       </s:c>
       <s:c r="L97" t="str" s="5">
-        <s:f>IF(COUNTA($A97:$G97)=0,"",IF(OR($A97="",$B97="",$C97="",$D97="",$E97=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B97))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A97))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E97="S",$E97="M",$E97="L")),"复杂度非法",IF(NOT(OR($F97="",$F97="内部集成",$F97="外部集成")),"集成类型非法",IF(AND($F97&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C97,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F97="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C97,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H97),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A97:$G97)=0,"",IF(LEFT($G97,4)="待确认：","待确认",IF(OR($A97="",$B97="",$C97="",$D97="",$E97=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B97))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A97))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E97="S",$E97="M",$E97="L")),"复杂度非法",IF(NOT(OR($F97="",$F97="内部集成",$F97="外部集成")),"集成类型非法",IF(AND($F97&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C97,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F97="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C97,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H97),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="98" ht="42" customHeight="1">
@@ -4654,7 +4654,7 @@
         <s:f>IF(COUNTA($A98:$G98)=0,"",IF($F98="",0,IF(NOT(ISNUMBER($I98)),"",IF($F98="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I98,1),IF($F98="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I98,1),"")))))</s:f>
       </s:c>
       <s:c r="L98" t="str" s="5">
-        <s:f>IF(COUNTA($A98:$G98)=0,"",IF(OR($A98="",$B98="",$C98="",$D98="",$E98=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B98))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A98))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E98="S",$E98="M",$E98="L")),"复杂度非法",IF(NOT(OR($F98="",$F98="内部集成",$F98="外部集成")),"集成类型非法",IF(AND($F98&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C98,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F98="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C98,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H98),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A98:$G98)=0,"",IF(LEFT($G98,4)="待确认：","待确认",IF(OR($A98="",$B98="",$C98="",$D98="",$E98=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B98))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A98))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E98="S",$E98="M",$E98="L")),"复杂度非法",IF(NOT(OR($F98="",$F98="内部集成",$F98="外部集成")),"集成类型非法",IF(AND($F98&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C98,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F98="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C98,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H98),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="99" ht="42" customHeight="1">
@@ -4678,7 +4678,7 @@
         <s:f>IF(COUNTA($A99:$G99)=0,"",IF($F99="",0,IF(NOT(ISNUMBER($I99)),"",IF($F99="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I99,1),IF($F99="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I99,1),"")))))</s:f>
       </s:c>
       <s:c r="L99" t="str" s="5">
-        <s:f>IF(COUNTA($A99:$G99)=0,"",IF(OR($A99="",$B99="",$C99="",$D99="",$E99=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B99))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A99))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E99="S",$E99="M",$E99="L")),"复杂度非法",IF(NOT(OR($F99="",$F99="内部集成",$F99="外部集成")),"集成类型非法",IF(AND($F99&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C99,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F99="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C99,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H99),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A99:$G99)=0,"",IF(LEFT($G99,4)="待确认：","待确认",IF(OR($A99="",$B99="",$C99="",$D99="",$E99=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B99))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A99))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E99="S",$E99="M",$E99="L")),"复杂度非法",IF(NOT(OR($F99="",$F99="内部集成",$F99="外部集成")),"集成类型非法",IF(AND($F99&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C99,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F99="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C99,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H99),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="100" ht="42" customHeight="1">
@@ -4702,7 +4702,7 @@
         <s:f>IF(COUNTA($A100:$G100)=0,"",IF($F100="",0,IF(NOT(ISNUMBER($I100)),"",IF($F100="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I100,1),IF($F100="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I100,1),"")))))</s:f>
       </s:c>
       <s:c r="L100" t="str" s="5">
-        <s:f>IF(COUNTA($A100:$G100)=0,"",IF(OR($A100="",$B100="",$C100="",$D100="",$E100=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B100))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A100))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E100="S",$E100="M",$E100="L")),"复杂度非法",IF(NOT(OR($F100="",$F100="内部集成",$F100="外部集成")),"集成类型非法",IF(AND($F100&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C100,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F100="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C100,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H100),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A100:$G100)=0,"",IF(LEFT($G100,4)="待确认：","待确认",IF(OR($A100="",$B100="",$C100="",$D100="",$E100=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B100))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A100))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E100="S",$E100="M",$E100="L")),"复杂度非法",IF(NOT(OR($F100="",$F100="内部集成",$F100="外部集成")),"集成类型非法",IF(AND($F100&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C100,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F100="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C100,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H100),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="101" ht="42" customHeight="1">
@@ -4726,7 +4726,7 @@
         <s:f>IF(COUNTA($A101:$G101)=0,"",IF($F101="",0,IF(NOT(ISNUMBER($I101)),"",IF($F101="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I101,1),IF($F101="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I101,1),"")))))</s:f>
       </s:c>
       <s:c r="L101" t="str" s="5">
-        <s:f>IF(COUNTA($A101:$G101)=0,"",IF(OR($A101="",$B101="",$C101="",$D101="",$E101=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B101))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A101))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E101="S",$E101="M",$E101="L")),"复杂度非法",IF(NOT(OR($F101="",$F101="内部集成",$F101="外部集成")),"集成类型非法",IF(AND($F101&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C101,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F101="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C101,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H101),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A101:$G101)=0,"",IF(LEFT($G101,4)="待确认：","待确认",IF(OR($A101="",$B101="",$C101="",$D101="",$E101=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B101))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A101))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E101="S",$E101="M",$E101="L")),"复杂度非法",IF(NOT(OR($F101="",$F101="内部集成",$F101="外部集成")),"集成类型非法",IF(AND($F101&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C101,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F101="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C101,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H101),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="102" ht="42" customHeight="1">
@@ -4750,7 +4750,7 @@
         <s:f>IF(COUNTA($A102:$G102)=0,"",IF($F102="",0,IF(NOT(ISNUMBER($I102)),"",IF($F102="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I102,1),IF($F102="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I102,1),"")))))</s:f>
       </s:c>
       <s:c r="L102" t="str" s="5">
-        <s:f>IF(COUNTA($A102:$G102)=0,"",IF(OR($A102="",$B102="",$C102="",$D102="",$E102=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B102))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A102))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E102="S",$E102="M",$E102="L")),"复杂度非法",IF(NOT(OR($F102="",$F102="内部集成",$F102="外部集成")),"集成类型非法",IF(AND($F102&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C102,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F102="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C102,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H102),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A102:$G102)=0,"",IF(LEFT($G102,4)="待确认：","待确认",IF(OR($A102="",$B102="",$C102="",$D102="",$E102=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B102))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A102))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E102="S",$E102="M",$E102="L")),"复杂度非法",IF(NOT(OR($F102="",$F102="内部集成",$F102="外部集成")),"集成类型非法",IF(AND($F102&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C102,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F102="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C102,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H102),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="103" ht="42" customHeight="1">
@@ -4774,7 +4774,7 @@
         <s:f>IF(COUNTA($A103:$G103)=0,"",IF($F103="",0,IF(NOT(ISNUMBER($I103)),"",IF($F103="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I103,1),IF($F103="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I103,1),"")))))</s:f>
       </s:c>
       <s:c r="L103" t="str" s="5">
-        <s:f>IF(COUNTA($A103:$G103)=0,"",IF(OR($A103="",$B103="",$C103="",$D103="",$E103=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B103))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A103))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E103="S",$E103="M",$E103="L")),"复杂度非法",IF(NOT(OR($F103="",$F103="内部集成",$F103="外部集成")),"集成类型非法",IF(AND($F103&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C103,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F103="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C103,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H103),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A103:$G103)=0,"",IF(LEFT($G103,4)="待确认：","待确认",IF(OR($A103="",$B103="",$C103="",$D103="",$E103=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B103))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A103))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E103="S",$E103="M",$E103="L")),"复杂度非法",IF(NOT(OR($F103="",$F103="内部集成",$F103="外部集成")),"集成类型非法",IF(AND($F103&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C103,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F103="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C103,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H103),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="104" ht="42" customHeight="1">
@@ -4798,7 +4798,7 @@
         <s:f>IF(COUNTA($A104:$G104)=0,"",IF($F104="",0,IF(NOT(ISNUMBER($I104)),"",IF($F104="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I104,1),IF($F104="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I104,1),"")))))</s:f>
       </s:c>
       <s:c r="L104" t="str" s="5">
-        <s:f>IF(COUNTA($A104:$G104)=0,"",IF(OR($A104="",$B104="",$C104="",$D104="",$E104=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B104))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A104))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E104="S",$E104="M",$E104="L")),"复杂度非法",IF(NOT(OR($F104="",$F104="内部集成",$F104="外部集成")),"集成类型非法",IF(AND($F104&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C104,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F104="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C104,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H104),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A104:$G104)=0,"",IF(LEFT($G104,4)="待确认：","待确认",IF(OR($A104="",$B104="",$C104="",$D104="",$E104=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B104))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A104))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E104="S",$E104="M",$E104="L")),"复杂度非法",IF(NOT(OR($F104="",$F104="内部集成",$F104="外部集成")),"集成类型非法",IF(AND($F104&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C104,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F104="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C104,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H104),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="105" ht="42" customHeight="1">
@@ -4822,7 +4822,7 @@
         <s:f>IF(COUNTA($A105:$G105)=0,"",IF($F105="",0,IF(NOT(ISNUMBER($I105)),"",IF($F105="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I105,1),IF($F105="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I105,1),"")))))</s:f>
       </s:c>
       <s:c r="L105" t="str" s="5">
-        <s:f>IF(COUNTA($A105:$G105)=0,"",IF(OR($A105="",$B105="",$C105="",$D105="",$E105=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B105))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A105))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E105="S",$E105="M",$E105="L")),"复杂度非法",IF(NOT(OR($F105="",$F105="内部集成",$F105="外部集成")),"集成类型非法",IF(AND($F105&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C105,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F105="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C105,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H105),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A105:$G105)=0,"",IF(LEFT($G105,4)="待确认：","待确认",IF(OR($A105="",$B105="",$C105="",$D105="",$E105=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B105))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A105))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E105="S",$E105="M",$E105="L")),"复杂度非法",IF(NOT(OR($F105="",$F105="内部集成",$F105="外部集成")),"集成类型非法",IF(AND($F105&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C105,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F105="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C105,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H105),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="106" ht="42" customHeight="1">
@@ -4846,7 +4846,7 @@
         <s:f>IF(COUNTA($A106:$G106)=0,"",IF($F106="",0,IF(NOT(ISNUMBER($I106)),"",IF($F106="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I106,1),IF($F106="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I106,1),"")))))</s:f>
       </s:c>
       <s:c r="L106" t="str" s="5">
-        <s:f>IF(COUNTA($A106:$G106)=0,"",IF(OR($A106="",$B106="",$C106="",$D106="",$E106=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B106))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A106))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E106="S",$E106="M",$E106="L")),"复杂度非法",IF(NOT(OR($F106="",$F106="内部集成",$F106="外部集成")),"集成类型非法",IF(AND($F106&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C106,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F106="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C106,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H106),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A106:$G106)=0,"",IF(LEFT($G106,4)="待确认：","待确认",IF(OR($A106="",$B106="",$C106="",$D106="",$E106=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B106))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A106))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E106="S",$E106="M",$E106="L")),"复杂度非法",IF(NOT(OR($F106="",$F106="内部集成",$F106="外部集成")),"集成类型非法",IF(AND($F106&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C106,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F106="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C106,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H106),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="107" ht="42" customHeight="1">
@@ -4870,7 +4870,7 @@
         <s:f>IF(COUNTA($A107:$G107)=0,"",IF($F107="",0,IF(NOT(ISNUMBER($I107)),"",IF($F107="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I107,1),IF($F107="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I107,1),"")))))</s:f>
       </s:c>
       <s:c r="L107" t="str" s="5">
-        <s:f>IF(COUNTA($A107:$G107)=0,"",IF(OR($A107="",$B107="",$C107="",$D107="",$E107=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B107))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A107))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E107="S",$E107="M",$E107="L")),"复杂度非法",IF(NOT(OR($F107="",$F107="内部集成",$F107="外部集成")),"集成类型非法",IF(AND($F107&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C107,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F107="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C107,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H107),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A107:$G107)=0,"",IF(LEFT($G107,4)="待确认：","待确认",IF(OR($A107="",$B107="",$C107="",$D107="",$E107=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B107))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A107))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E107="S",$E107="M",$E107="L")),"复杂度非法",IF(NOT(OR($F107="",$F107="内部集成",$F107="外部集成")),"集成类型非法",IF(AND($F107&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C107,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F107="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C107,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H107),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="108" ht="42" customHeight="1">
@@ -4894,7 +4894,7 @@
         <s:f>IF(COUNTA($A108:$G108)=0,"",IF($F108="",0,IF(NOT(ISNUMBER($I108)),"",IF($F108="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I108,1),IF($F108="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I108,1),"")))))</s:f>
       </s:c>
       <s:c r="L108" t="str" s="5">
-        <s:f>IF(COUNTA($A108:$G108)=0,"",IF(OR($A108="",$B108="",$C108="",$D108="",$E108=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B108))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A108))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E108="S",$E108="M",$E108="L")),"复杂度非法",IF(NOT(OR($F108="",$F108="内部集成",$F108="外部集成")),"集成类型非法",IF(AND($F108&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C108,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F108="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C108,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H108),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A108:$G108)=0,"",IF(LEFT($G108,4)="待确认：","待确认",IF(OR($A108="",$B108="",$C108="",$D108="",$E108=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B108))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A108))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E108="S",$E108="M",$E108="L")),"复杂度非法",IF(NOT(OR($F108="",$F108="内部集成",$F108="外部集成")),"集成类型非法",IF(AND($F108&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C108,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F108="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C108,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H108),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="109" ht="42" customHeight="1">
@@ -4918,7 +4918,7 @@
         <s:f>IF(COUNTA($A109:$G109)=0,"",IF($F109="",0,IF(NOT(ISNUMBER($I109)),"",IF($F109="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I109,1),IF($F109="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I109,1),"")))))</s:f>
       </s:c>
       <s:c r="L109" t="str" s="5">
-        <s:f>IF(COUNTA($A109:$G109)=0,"",IF(OR($A109="",$B109="",$C109="",$D109="",$E109=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B109))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A109))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E109="S",$E109="M",$E109="L")),"复杂度非法",IF(NOT(OR($F109="",$F109="内部集成",$F109="外部集成")),"集成类型非法",IF(AND($F109&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C109,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F109="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C109,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H109),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A109:$G109)=0,"",IF(LEFT($G109,4)="待确认：","待确认",IF(OR($A109="",$B109="",$C109="",$D109="",$E109=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B109))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A109))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E109="S",$E109="M",$E109="L")),"复杂度非法",IF(NOT(OR($F109="",$F109="内部集成",$F109="外部集成")),"集成类型非法",IF(AND($F109&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C109,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F109="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C109,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H109),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="110" ht="42" customHeight="1">
@@ -4942,7 +4942,7 @@
         <s:f>IF(COUNTA($A110:$G110)=0,"",IF($F110="",0,IF(NOT(ISNUMBER($I110)),"",IF($F110="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I110,1),IF($F110="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I110,1),"")))))</s:f>
       </s:c>
       <s:c r="L110" t="str" s="5">
-        <s:f>IF(COUNTA($A110:$G110)=0,"",IF(OR($A110="",$B110="",$C110="",$D110="",$E110=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B110))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A110))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E110="S",$E110="M",$E110="L")),"复杂度非法",IF(NOT(OR($F110="",$F110="内部集成",$F110="外部集成")),"集成类型非法",IF(AND($F110&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C110,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F110="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C110,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H110),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A110:$G110)=0,"",IF(LEFT($G110,4)="待确认：","待确认",IF(OR($A110="",$B110="",$C110="",$D110="",$E110=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B110))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A110))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E110="S",$E110="M",$E110="L")),"复杂度非法",IF(NOT(OR($F110="",$F110="内部集成",$F110="外部集成")),"集成类型非法",IF(AND($F110&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C110,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F110="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C110,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H110),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="111" ht="42" customHeight="1">
@@ -4966,7 +4966,7 @@
         <s:f>IF(COUNTA($A111:$G111)=0,"",IF($F111="",0,IF(NOT(ISNUMBER($I111)),"",IF($F111="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I111,1),IF($F111="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I111,1),"")))))</s:f>
       </s:c>
       <s:c r="L111" t="str" s="5">
-        <s:f>IF(COUNTA($A111:$G111)=0,"",IF(OR($A111="",$B111="",$C111="",$D111="",$E111=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B111))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A111))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E111="S",$E111="M",$E111="L")),"复杂度非法",IF(NOT(OR($F111="",$F111="内部集成",$F111="外部集成")),"集成类型非法",IF(AND($F111&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C111,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F111="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C111,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H111),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A111:$G111)=0,"",IF(LEFT($G111,4)="待确认：","待确认",IF(OR($A111="",$B111="",$C111="",$D111="",$E111=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B111))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A111))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E111="S",$E111="M",$E111="L")),"复杂度非法",IF(NOT(OR($F111="",$F111="内部集成",$F111="外部集成")),"集成类型非法",IF(AND($F111&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C111,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F111="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C111,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H111),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="112" ht="42" customHeight="1">
@@ -4990,7 +4990,7 @@
         <s:f>IF(COUNTA($A112:$G112)=0,"",IF($F112="",0,IF(NOT(ISNUMBER($I112)),"",IF($F112="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I112,1),IF($F112="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I112,1),"")))))</s:f>
       </s:c>
       <s:c r="L112" t="str" s="5">
-        <s:f>IF(COUNTA($A112:$G112)=0,"",IF(OR($A112="",$B112="",$C112="",$D112="",$E112=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B112))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A112))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E112="S",$E112="M",$E112="L")),"复杂度非法",IF(NOT(OR($F112="",$F112="内部集成",$F112="外部集成")),"集成类型非法",IF(AND($F112&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C112,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F112="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C112,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H112),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A112:$G112)=0,"",IF(LEFT($G112,4)="待确认：","待确认",IF(OR($A112="",$B112="",$C112="",$D112="",$E112=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B112))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A112))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E112="S",$E112="M",$E112="L")),"复杂度非法",IF(NOT(OR($F112="",$F112="内部集成",$F112="外部集成")),"集成类型非法",IF(AND($F112&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C112,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F112="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C112,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H112),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="113" ht="42" customHeight="1">
@@ -5014,7 +5014,7 @@
         <s:f>IF(COUNTA($A113:$G113)=0,"",IF($F113="",0,IF(NOT(ISNUMBER($I113)),"",IF($F113="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I113,1),IF($F113="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I113,1),"")))))</s:f>
       </s:c>
       <s:c r="L113" t="str" s="5">
-        <s:f>IF(COUNTA($A113:$G113)=0,"",IF(OR($A113="",$B113="",$C113="",$D113="",$E113=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B113))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A113))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E113="S",$E113="M",$E113="L")),"复杂度非法",IF(NOT(OR($F113="",$F113="内部集成",$F113="外部集成")),"集成类型非法",IF(AND($F113&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C113,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F113="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C113,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H113),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A113:$G113)=0,"",IF(LEFT($G113,4)="待确认：","待确认",IF(OR($A113="",$B113="",$C113="",$D113="",$E113=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B113))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A113))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E113="S",$E113="M",$E113="L")),"复杂度非法",IF(NOT(OR($F113="",$F113="内部集成",$F113="外部集成")),"集成类型非法",IF(AND($F113&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C113,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F113="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C113,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H113),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="114" ht="42" customHeight="1">
@@ -5038,7 +5038,7 @@
         <s:f>IF(COUNTA($A114:$G114)=0,"",IF($F114="",0,IF(NOT(ISNUMBER($I114)),"",IF($F114="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I114,1),IF($F114="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I114,1),"")))))</s:f>
       </s:c>
       <s:c r="L114" t="str" s="5">
-        <s:f>IF(COUNTA($A114:$G114)=0,"",IF(OR($A114="",$B114="",$C114="",$D114="",$E114=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B114))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A114))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E114="S",$E114="M",$E114="L")),"复杂度非法",IF(NOT(OR($F114="",$F114="内部集成",$F114="外部集成")),"集成类型非法",IF(AND($F114&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C114,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F114="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C114,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H114),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A114:$G114)=0,"",IF(LEFT($G114,4)="待确认：","待确认",IF(OR($A114="",$B114="",$C114="",$D114="",$E114=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B114))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A114))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E114="S",$E114="M",$E114="L")),"复杂度非法",IF(NOT(OR($F114="",$F114="内部集成",$F114="外部集成")),"集成类型非法",IF(AND($F114&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C114,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F114="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C114,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H114),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="115" ht="42" customHeight="1">
@@ -5062,7 +5062,7 @@
         <s:f>IF(COUNTA($A115:$G115)=0,"",IF($F115="",0,IF(NOT(ISNUMBER($I115)),"",IF($F115="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I115,1),IF($F115="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I115,1),"")))))</s:f>
       </s:c>
       <s:c r="L115" t="str" s="5">
-        <s:f>IF(COUNTA($A115:$G115)=0,"",IF(OR($A115="",$B115="",$C115="",$D115="",$E115=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B115))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A115))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E115="S",$E115="M",$E115="L")),"复杂度非法",IF(NOT(OR($F115="",$F115="内部集成",$F115="外部集成")),"集成类型非法",IF(AND($F115&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C115,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F115="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C115,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H115),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A115:$G115)=0,"",IF(LEFT($G115,4)="待确认：","待确认",IF(OR($A115="",$B115="",$C115="",$D115="",$E115=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B115))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A115))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E115="S",$E115="M",$E115="L")),"复杂度非法",IF(NOT(OR($F115="",$F115="内部集成",$F115="外部集成")),"集成类型非法",IF(AND($F115&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C115,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F115="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C115,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H115),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="116" ht="42" customHeight="1">
@@ -5086,7 +5086,7 @@
         <s:f>IF(COUNTA($A116:$G116)=0,"",IF($F116="",0,IF(NOT(ISNUMBER($I116)),"",IF($F116="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I116,1),IF($F116="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I116,1),"")))))</s:f>
       </s:c>
       <s:c r="L116" t="str" s="5">
-        <s:f>IF(COUNTA($A116:$G116)=0,"",IF(OR($A116="",$B116="",$C116="",$D116="",$E116=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B116))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A116))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E116="S",$E116="M",$E116="L")),"复杂度非法",IF(NOT(OR($F116="",$F116="内部集成",$F116="外部集成")),"集成类型非法",IF(AND($F116&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C116,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F116="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C116,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H116),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A116:$G116)=0,"",IF(LEFT($G116,4)="待确认：","待确认",IF(OR($A116="",$B116="",$C116="",$D116="",$E116=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B116))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A116))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E116="S",$E116="M",$E116="L")),"复杂度非法",IF(NOT(OR($F116="",$F116="内部集成",$F116="外部集成")),"集成类型非法",IF(AND($F116&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C116,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F116="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C116,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H116),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="117" ht="42" customHeight="1">
@@ -5110,7 +5110,7 @@
         <s:f>IF(COUNTA($A117:$G117)=0,"",IF($F117="",0,IF(NOT(ISNUMBER($I117)),"",IF($F117="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I117,1),IF($F117="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I117,1),"")))))</s:f>
       </s:c>
       <s:c r="L117" t="str" s="5">
-        <s:f>IF(COUNTA($A117:$G117)=0,"",IF(OR($A117="",$B117="",$C117="",$D117="",$E117=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B117))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A117))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E117="S",$E117="M",$E117="L")),"复杂度非法",IF(NOT(OR($F117="",$F117="内部集成",$F117="外部集成")),"集成类型非法",IF(AND($F117&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C117,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F117="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C117,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H117),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A117:$G117)=0,"",IF(LEFT($G117,4)="待确认：","待确认",IF(OR($A117="",$B117="",$C117="",$D117="",$E117=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B117))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A117))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E117="S",$E117="M",$E117="L")),"复杂度非法",IF(NOT(OR($F117="",$F117="内部集成",$F117="外部集成")),"集成类型非法",IF(AND($F117&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C117,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F117="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C117,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H117),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="118" ht="42" customHeight="1">
@@ -5134,7 +5134,7 @@
         <s:f>IF(COUNTA($A118:$G118)=0,"",IF($F118="",0,IF(NOT(ISNUMBER($I118)),"",IF($F118="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I118,1),IF($F118="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I118,1),"")))))</s:f>
       </s:c>
       <s:c r="L118" t="str" s="5">
-        <s:f>IF(COUNTA($A118:$G118)=0,"",IF(OR($A118="",$B118="",$C118="",$D118="",$E118=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B118))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A118))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E118="S",$E118="M",$E118="L")),"复杂度非法",IF(NOT(OR($F118="",$F118="内部集成",$F118="外部集成")),"集成类型非法",IF(AND($F118&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C118,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F118="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C118,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H118),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A118:$G118)=0,"",IF(LEFT($G118,4)="待确认：","待确认",IF(OR($A118="",$B118="",$C118="",$D118="",$E118=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B118))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A118))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E118="S",$E118="M",$E118="L")),"复杂度非法",IF(NOT(OR($F118="",$F118="内部集成",$F118="外部集成")),"集成类型非法",IF(AND($F118&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C118,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F118="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C118,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H118),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="119" ht="42" customHeight="1">
@@ -5158,7 +5158,7 @@
         <s:f>IF(COUNTA($A119:$G119)=0,"",IF($F119="",0,IF(NOT(ISNUMBER($I119)),"",IF($F119="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I119,1),IF($F119="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I119,1),"")))))</s:f>
       </s:c>
       <s:c r="L119" t="str" s="5">
-        <s:f>IF(COUNTA($A119:$G119)=0,"",IF(OR($A119="",$B119="",$C119="",$D119="",$E119=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B119))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A119))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E119="S",$E119="M",$E119="L")),"复杂度非法",IF(NOT(OR($F119="",$F119="内部集成",$F119="外部集成")),"集成类型非法",IF(AND($F119&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C119,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F119="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C119,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H119),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A119:$G119)=0,"",IF(LEFT($G119,4)="待确认：","待确认",IF(OR($A119="",$B119="",$C119="",$D119="",$E119=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B119))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A119))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E119="S",$E119="M",$E119="L")),"复杂度非法",IF(NOT(OR($F119="",$F119="内部集成",$F119="外部集成")),"集成类型非法",IF(AND($F119&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C119,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F119="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C119,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H119),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="120" ht="42" customHeight="1">
@@ -5182,7 +5182,7 @@
         <s:f>IF(COUNTA($A120:$G120)=0,"",IF($F120="",0,IF(NOT(ISNUMBER($I120)),"",IF($F120="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I120,1),IF($F120="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I120,1),"")))))</s:f>
       </s:c>
       <s:c r="L120" t="str" s="5">
-        <s:f>IF(COUNTA($A120:$G120)=0,"",IF(OR($A120="",$B120="",$C120="",$D120="",$E120=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B120))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A120))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E120="S",$E120="M",$E120="L")),"复杂度非法",IF(NOT(OR($F120="",$F120="内部集成",$F120="外部集成")),"集成类型非法",IF(AND($F120&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C120,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F120="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C120,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H120),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A120:$G120)=0,"",IF(LEFT($G120,4)="待确认：","待确认",IF(OR($A120="",$B120="",$C120="",$D120="",$E120=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B120))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A120))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E120="S",$E120="M",$E120="L")),"复杂度非法",IF(NOT(OR($F120="",$F120="内部集成",$F120="外部集成")),"集成类型非法",IF(AND($F120&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C120,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F120="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C120,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H120),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="121" ht="42" customHeight="1">
@@ -5206,7 +5206,7 @@
         <s:f>IF(COUNTA($A121:$G121)=0,"",IF($F121="",0,IF(NOT(ISNUMBER($I121)),"",IF($F121="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I121,1),IF($F121="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I121,1),"")))))</s:f>
       </s:c>
       <s:c r="L121" t="str" s="5">
-        <s:f>IF(COUNTA($A121:$G121)=0,"",IF(OR($A121="",$B121="",$C121="",$D121="",$E121=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B121))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A121))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E121="S",$E121="M",$E121="L")),"复杂度非法",IF(NOT(OR($F121="",$F121="内部集成",$F121="外部集成")),"集成类型非法",IF(AND($F121&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C121,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F121="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C121,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H121),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A121:$G121)=0,"",IF(LEFT($G121,4)="待确认：","待确认",IF(OR($A121="",$B121="",$C121="",$D121="",$E121=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B121))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A121))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E121="S",$E121="M",$E121="L")),"复杂度非法",IF(NOT(OR($F121="",$F121="内部集成",$F121="外部集成")),"集成类型非法",IF(AND($F121&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C121,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F121="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C121,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H121),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="122" ht="42" customHeight="1">
@@ -5230,7 +5230,7 @@
         <s:f>IF(COUNTA($A122:$G122)=0,"",IF($F122="",0,IF(NOT(ISNUMBER($I122)),"",IF($F122="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I122,1),IF($F122="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I122,1),"")))))</s:f>
       </s:c>
       <s:c r="L122" t="str" s="5">
-        <s:f>IF(COUNTA($A122:$G122)=0,"",IF(OR($A122="",$B122="",$C122="",$D122="",$E122=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B122))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A122))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E122="S",$E122="M",$E122="L")),"复杂度非法",IF(NOT(OR($F122="",$F122="内部集成",$F122="外部集成")),"集成类型非法",IF(AND($F122&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C122,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F122="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C122,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H122),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A122:$G122)=0,"",IF(LEFT($G122,4)="待确认：","待确认",IF(OR($A122="",$B122="",$C122="",$D122="",$E122=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B122))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A122))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E122="S",$E122="M",$E122="L")),"复杂度非法",IF(NOT(OR($F122="",$F122="内部集成",$F122="外部集成")),"集成类型非法",IF(AND($F122&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C122,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F122="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C122,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H122),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="123" ht="42" customHeight="1">
@@ -5254,7 +5254,7 @@
         <s:f>IF(COUNTA($A123:$G123)=0,"",IF($F123="",0,IF(NOT(ISNUMBER($I123)),"",IF($F123="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I123,1),IF($F123="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I123,1),"")))))</s:f>
       </s:c>
       <s:c r="L123" t="str" s="5">
-        <s:f>IF(COUNTA($A123:$G123)=0,"",IF(OR($A123="",$B123="",$C123="",$D123="",$E123=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B123))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A123))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E123="S",$E123="M",$E123="L")),"复杂度非法",IF(NOT(OR($F123="",$F123="内部集成",$F123="外部集成")),"集成类型非法",IF(AND($F123&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C123,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F123="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C123,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H123),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A123:$G123)=0,"",IF(LEFT($G123,4)="待确认：","待确认",IF(OR($A123="",$B123="",$C123="",$D123="",$E123=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B123))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A123))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E123="S",$E123="M",$E123="L")),"复杂度非法",IF(NOT(OR($F123="",$F123="内部集成",$F123="外部集成")),"集成类型非法",IF(AND($F123&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C123,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F123="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C123,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H123),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="124" ht="42" customHeight="1">
@@ -5278,7 +5278,7 @@
         <s:f>IF(COUNTA($A124:$G124)=0,"",IF($F124="",0,IF(NOT(ISNUMBER($I124)),"",IF($F124="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I124,1),IF($F124="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I124,1),"")))))</s:f>
       </s:c>
       <s:c r="L124" t="str" s="5">
-        <s:f>IF(COUNTA($A124:$G124)=0,"",IF(OR($A124="",$B124="",$C124="",$D124="",$E124=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B124))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A124))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E124="S",$E124="M",$E124="L")),"复杂度非法",IF(NOT(OR($F124="",$F124="内部集成",$F124="外部集成")),"集成类型非法",IF(AND($F124&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C124,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F124="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C124,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H124),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A124:$G124)=0,"",IF(LEFT($G124,4)="待确认：","待确认",IF(OR($A124="",$B124="",$C124="",$D124="",$E124=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B124))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A124))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E124="S",$E124="M",$E124="L")),"复杂度非法",IF(NOT(OR($F124="",$F124="内部集成",$F124="外部集成")),"集成类型非法",IF(AND($F124&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C124,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F124="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C124,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H124),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="125" ht="42" customHeight="1">
@@ -5302,7 +5302,7 @@
         <s:f>IF(COUNTA($A125:$G125)=0,"",IF($F125="",0,IF(NOT(ISNUMBER($I125)),"",IF($F125="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I125,1),IF($F125="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I125,1),"")))))</s:f>
       </s:c>
       <s:c r="L125" t="str" s="5">
-        <s:f>IF(COUNTA($A125:$G125)=0,"",IF(OR($A125="",$B125="",$C125="",$D125="",$E125=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B125))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A125))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E125="S",$E125="M",$E125="L")),"复杂度非法",IF(NOT(OR($F125="",$F125="内部集成",$F125="外部集成")),"集成类型非法",IF(AND($F125&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C125,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F125="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C125,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H125),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A125:$G125)=0,"",IF(LEFT($G125,4)="待确认：","待确认",IF(OR($A125="",$B125="",$C125="",$D125="",$E125=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B125))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A125))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E125="S",$E125="M",$E125="L")),"复杂度非法",IF(NOT(OR($F125="",$F125="内部集成",$F125="外部集成")),"集成类型非法",IF(AND($F125&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C125,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F125="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C125,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H125),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="126" ht="42" customHeight="1">
@@ -5326,7 +5326,7 @@
         <s:f>IF(COUNTA($A126:$G126)=0,"",IF($F126="",0,IF(NOT(ISNUMBER($I126)),"",IF($F126="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I126,1),IF($F126="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I126,1),"")))))</s:f>
       </s:c>
       <s:c r="L126" t="str" s="5">
-        <s:f>IF(COUNTA($A126:$G126)=0,"",IF(OR($A126="",$B126="",$C126="",$D126="",$E126=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B126))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A126))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E126="S",$E126="M",$E126="L")),"复杂度非法",IF(NOT(OR($F126="",$F126="内部集成",$F126="外部集成")),"集成类型非法",IF(AND($F126&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C126,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F126="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C126,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H126),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A126:$G126)=0,"",IF(LEFT($G126,4)="待确认：","待确认",IF(OR($A126="",$B126="",$C126="",$D126="",$E126=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B126))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A126))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E126="S",$E126="M",$E126="L")),"复杂度非法",IF(NOT(OR($F126="",$F126="内部集成",$F126="外部集成")),"集成类型非法",IF(AND($F126&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C126,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F126="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C126,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H126),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="127" ht="42" customHeight="1">
@@ -5350,7 +5350,7 @@
         <s:f>IF(COUNTA($A127:$G127)=0,"",IF($F127="",0,IF(NOT(ISNUMBER($I127)),"",IF($F127="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I127,1),IF($F127="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I127,1),"")))))</s:f>
       </s:c>
       <s:c r="L127" t="str" s="5">
-        <s:f>IF(COUNTA($A127:$G127)=0,"",IF(OR($A127="",$B127="",$C127="",$D127="",$E127=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B127))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A127))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E127="S",$E127="M",$E127="L")),"复杂度非法",IF(NOT(OR($F127="",$F127="内部集成",$F127="外部集成")),"集成类型非法",IF(AND($F127&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C127,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F127="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C127,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H127),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A127:$G127)=0,"",IF(LEFT($G127,4)="待确认：","待确认",IF(OR($A127="",$B127="",$C127="",$D127="",$E127=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B127))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A127))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E127="S",$E127="M",$E127="L")),"复杂度非法",IF(NOT(OR($F127="",$F127="内部集成",$F127="外部集成")),"集成类型非法",IF(AND($F127&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C127,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F127="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C127,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H127),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="128" ht="42" customHeight="1">
@@ -5374,7 +5374,7 @@
         <s:f>IF(COUNTA($A128:$G128)=0,"",IF($F128="",0,IF(NOT(ISNUMBER($I128)),"",IF($F128="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I128,1),IF($F128="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I128,1),"")))))</s:f>
       </s:c>
       <s:c r="L128" t="str" s="5">
-        <s:f>IF(COUNTA($A128:$G128)=0,"",IF(OR($A128="",$B128="",$C128="",$D128="",$E128=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B128))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A128))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E128="S",$E128="M",$E128="L")),"复杂度非法",IF(NOT(OR($F128="",$F128="内部集成",$F128="外部集成")),"集成类型非法",IF(AND($F128&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C128,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F128="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C128,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H128),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A128:$G128)=0,"",IF(LEFT($G128,4)="待确认：","待确认",IF(OR($A128="",$B128="",$C128="",$D128="",$E128=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B128))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A128))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E128="S",$E128="M",$E128="L")),"复杂度非法",IF(NOT(OR($F128="",$F128="内部集成",$F128="外部集成")),"集成类型非法",IF(AND($F128&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C128,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F128="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C128,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H128),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="129" ht="42" customHeight="1">
@@ -5398,7 +5398,7 @@
         <s:f>IF(COUNTA($A129:$G129)=0,"",IF($F129="",0,IF(NOT(ISNUMBER($I129)),"",IF($F129="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I129,1),IF($F129="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I129,1),"")))))</s:f>
       </s:c>
       <s:c r="L129" t="str" s="5">
-        <s:f>IF(COUNTA($A129:$G129)=0,"",IF(OR($A129="",$B129="",$C129="",$D129="",$E129=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B129))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A129))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E129="S",$E129="M",$E129="L")),"复杂度非法",IF(NOT(OR($F129="",$F129="内部集成",$F129="外部集成")),"集成类型非法",IF(AND($F129&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C129,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F129="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C129,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H129),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A129:$G129)=0,"",IF(LEFT($G129,4)="待确认：","待确认",IF(OR($A129="",$B129="",$C129="",$D129="",$E129=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B129))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A129))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E129="S",$E129="M",$E129="L")),"复杂度非法",IF(NOT(OR($F129="",$F129="内部集成",$F129="外部集成")),"集成类型非法",IF(AND($F129&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C129,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F129="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C129,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H129),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="130" ht="42" customHeight="1">
@@ -5422,7 +5422,7 @@
         <s:f>IF(COUNTA($A130:$G130)=0,"",IF($F130="",0,IF(NOT(ISNUMBER($I130)),"",IF($F130="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I130,1),IF($F130="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I130,1),"")))))</s:f>
       </s:c>
       <s:c r="L130" t="str" s="5">
-        <s:f>IF(COUNTA($A130:$G130)=0,"",IF(OR($A130="",$B130="",$C130="",$D130="",$E130=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B130))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A130))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E130="S",$E130="M",$E130="L")),"复杂度非法",IF(NOT(OR($F130="",$F130="内部集成",$F130="外部集成")),"集成类型非法",IF(AND($F130&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C130,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F130="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C130,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H130),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A130:$G130)=0,"",IF(LEFT($G130,4)="待确认：","待确认",IF(OR($A130="",$B130="",$C130="",$D130="",$E130=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B130))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A130))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E130="S",$E130="M",$E130="L")),"复杂度非法",IF(NOT(OR($F130="",$F130="内部集成",$F130="外部集成")),"集成类型非法",IF(AND($F130&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C130,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F130="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C130,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H130),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="131" ht="42" customHeight="1">
@@ -5446,7 +5446,7 @@
         <s:f>IF(COUNTA($A131:$G131)=0,"",IF($F131="",0,IF(NOT(ISNUMBER($I131)),"",IF($F131="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I131,1),IF($F131="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I131,1),"")))))</s:f>
       </s:c>
       <s:c r="L131" t="str" s="5">
-        <s:f>IF(COUNTA($A131:$G131)=0,"",IF(OR($A131="",$B131="",$C131="",$D131="",$E131=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B131))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A131))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E131="S",$E131="M",$E131="L")),"复杂度非法",IF(NOT(OR($F131="",$F131="内部集成",$F131="外部集成")),"集成类型非法",IF(AND($F131&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C131,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F131="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C131,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H131),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A131:$G131)=0,"",IF(LEFT($G131,4)="待确认：","待确认",IF(OR($A131="",$B131="",$C131="",$D131="",$E131=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B131))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A131))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E131="S",$E131="M",$E131="L")),"复杂度非法",IF(NOT(OR($F131="",$F131="内部集成",$F131="外部集成")),"集成类型非法",IF(AND($F131&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C131,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F131="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C131,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H131),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="132" ht="42" customHeight="1">
@@ -5470,7 +5470,7 @@
         <s:f>IF(COUNTA($A132:$G132)=0,"",IF($F132="",0,IF(NOT(ISNUMBER($I132)),"",IF($F132="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I132,1),IF($F132="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I132,1),"")))))</s:f>
       </s:c>
       <s:c r="L132" t="str" s="5">
-        <s:f>IF(COUNTA($A132:$G132)=0,"",IF(OR($A132="",$B132="",$C132="",$D132="",$E132=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B132))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A132))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E132="S",$E132="M",$E132="L")),"复杂度非法",IF(NOT(OR($F132="",$F132="内部集成",$F132="外部集成")),"集成类型非法",IF(AND($F132&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C132,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F132="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C132,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H132),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A132:$G132)=0,"",IF(LEFT($G132,4)="待确认：","待确认",IF(OR($A132="",$B132="",$C132="",$D132="",$E132=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B132))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A132))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E132="S",$E132="M",$E132="L")),"复杂度非法",IF(NOT(OR($F132="",$F132="内部集成",$F132="外部集成")),"集成类型非法",IF(AND($F132&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C132,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F132="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C132,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H132),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="133" ht="42" customHeight="1">
@@ -5494,7 +5494,7 @@
         <s:f>IF(COUNTA($A133:$G133)=0,"",IF($F133="",0,IF(NOT(ISNUMBER($I133)),"",IF($F133="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I133,1),IF($F133="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I133,1),"")))))</s:f>
       </s:c>
       <s:c r="L133" t="str" s="5">
-        <s:f>IF(COUNTA($A133:$G133)=0,"",IF(OR($A133="",$B133="",$C133="",$D133="",$E133=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B133))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A133))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E133="S",$E133="M",$E133="L")),"复杂度非法",IF(NOT(OR($F133="",$F133="内部集成",$F133="外部集成")),"集成类型非法",IF(AND($F133&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C133,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F133="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C133,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H133),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A133:$G133)=0,"",IF(LEFT($G133,4)="待确认：","待确认",IF(OR($A133="",$B133="",$C133="",$D133="",$E133=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B133))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A133))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E133="S",$E133="M",$E133="L")),"复杂度非法",IF(NOT(OR($F133="",$F133="内部集成",$F133="外部集成")),"集成类型非法",IF(AND($F133&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C133,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F133="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C133,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H133),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="134" ht="42" customHeight="1">
@@ -5518,7 +5518,7 @@
         <s:f>IF(COUNTA($A134:$G134)=0,"",IF($F134="",0,IF(NOT(ISNUMBER($I134)),"",IF($F134="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I134,1),IF($F134="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I134,1),"")))))</s:f>
       </s:c>
       <s:c r="L134" t="str" s="5">
-        <s:f>IF(COUNTA($A134:$G134)=0,"",IF(OR($A134="",$B134="",$C134="",$D134="",$E134=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B134))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A134))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E134="S",$E134="M",$E134="L")),"复杂度非法",IF(NOT(OR($F134="",$F134="内部集成",$F134="外部集成")),"集成类型非法",IF(AND($F134&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C134,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F134="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C134,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H134),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A134:$G134)=0,"",IF(LEFT($G134,4)="待确认：","待确认",IF(OR($A134="",$B134="",$C134="",$D134="",$E134=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B134))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A134))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E134="S",$E134="M",$E134="L")),"复杂度非法",IF(NOT(OR($F134="",$F134="内部集成",$F134="外部集成")),"集成类型非法",IF(AND($F134&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C134,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F134="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C134,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H134),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="135" ht="42" customHeight="1">
@@ -5542,7 +5542,7 @@
         <s:f>IF(COUNTA($A135:$G135)=0,"",IF($F135="",0,IF(NOT(ISNUMBER($I135)),"",IF($F135="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I135,1),IF($F135="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I135,1),"")))))</s:f>
       </s:c>
       <s:c r="L135" t="str" s="5">
-        <s:f>IF(COUNTA($A135:$G135)=0,"",IF(OR($A135="",$B135="",$C135="",$D135="",$E135=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B135))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A135))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E135="S",$E135="M",$E135="L")),"复杂度非法",IF(NOT(OR($F135="",$F135="内部集成",$F135="外部集成")),"集成类型非法",IF(AND($F135&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C135,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F135="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C135,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H135),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A135:$G135)=0,"",IF(LEFT($G135,4)="待确认：","待确认",IF(OR($A135="",$B135="",$C135="",$D135="",$E135=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B135))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A135))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E135="S",$E135="M",$E135="L")),"复杂度非法",IF(NOT(OR($F135="",$F135="内部集成",$F135="外部集成")),"集成类型非法",IF(AND($F135&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C135,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F135="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C135,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H135),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="136" ht="42" customHeight="1">
@@ -5566,7 +5566,7 @@
         <s:f>IF(COUNTA($A136:$G136)=0,"",IF($F136="",0,IF(NOT(ISNUMBER($I136)),"",IF($F136="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I136,1),IF($F136="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I136,1),"")))))</s:f>
       </s:c>
       <s:c r="L136" t="str" s="5">
-        <s:f>IF(COUNTA($A136:$G136)=0,"",IF(OR($A136="",$B136="",$C136="",$D136="",$E136=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B136))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A136))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E136="S",$E136="M",$E136="L")),"复杂度非法",IF(NOT(OR($F136="",$F136="内部集成",$F136="外部集成")),"集成类型非法",IF(AND($F136&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C136,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F136="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C136,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H136),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A136:$G136)=0,"",IF(LEFT($G136,4)="待确认：","待确认",IF(OR($A136="",$B136="",$C136="",$D136="",$E136=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B136))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A136))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E136="S",$E136="M",$E136="L")),"复杂度非法",IF(NOT(OR($F136="",$F136="内部集成",$F136="外部集成")),"集成类型非法",IF(AND($F136&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C136,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F136="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C136,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H136),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="137" ht="42" customHeight="1">
@@ -5590,7 +5590,7 @@
         <s:f>IF(COUNTA($A137:$G137)=0,"",IF($F137="",0,IF(NOT(ISNUMBER($I137)),"",IF($F137="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I137,1),IF($F137="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I137,1),"")))))</s:f>
       </s:c>
       <s:c r="L137" t="str" s="5">
-        <s:f>IF(COUNTA($A137:$G137)=0,"",IF(OR($A137="",$B137="",$C137="",$D137="",$E137=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B137))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A137))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E137="S",$E137="M",$E137="L")),"复杂度非法",IF(NOT(OR($F137="",$F137="内部集成",$F137="外部集成")),"集成类型非法",IF(AND($F137&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C137,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F137="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C137,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H137),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A137:$G137)=0,"",IF(LEFT($G137,4)="待确认：","待确认",IF(OR($A137="",$B137="",$C137="",$D137="",$E137=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B137))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A137))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E137="S",$E137="M",$E137="L")),"复杂度非法",IF(NOT(OR($F137="",$F137="内部集成",$F137="外部集成")),"集成类型非法",IF(AND($F137&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C137,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F137="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C137,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H137),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="138" ht="42" customHeight="1">
@@ -5614,7 +5614,7 @@
         <s:f>IF(COUNTA($A138:$G138)=0,"",IF($F138="",0,IF(NOT(ISNUMBER($I138)),"",IF($F138="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I138,1),IF($F138="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I138,1),"")))))</s:f>
       </s:c>
       <s:c r="L138" t="str" s="5">
-        <s:f>IF(COUNTA($A138:$G138)=0,"",IF(OR($A138="",$B138="",$C138="",$D138="",$E138=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B138))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A138))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E138="S",$E138="M",$E138="L")),"复杂度非法",IF(NOT(OR($F138="",$F138="内部集成",$F138="外部集成")),"集成类型非法",IF(AND($F138&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C138,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F138="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C138,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H138),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A138:$G138)=0,"",IF(LEFT($G138,4)="待确认：","待确认",IF(OR($A138="",$B138="",$C138="",$D138="",$E138=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B138))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A138))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E138="S",$E138="M",$E138="L")),"复杂度非法",IF(NOT(OR($F138="",$F138="内部集成",$F138="外部集成")),"集成类型非法",IF(AND($F138&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C138,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F138="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C138,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H138),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="139" ht="42" customHeight="1">
@@ -5638,7 +5638,7 @@
         <s:f>IF(COUNTA($A139:$G139)=0,"",IF($F139="",0,IF(NOT(ISNUMBER($I139)),"",IF($F139="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I139,1),IF($F139="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I139,1),"")))))</s:f>
       </s:c>
       <s:c r="L139" t="str" s="5">
-        <s:f>IF(COUNTA($A139:$G139)=0,"",IF(OR($A139="",$B139="",$C139="",$D139="",$E139=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B139))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A139))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E139="S",$E139="M",$E139="L")),"复杂度非法",IF(NOT(OR($F139="",$F139="内部集成",$F139="外部集成")),"集成类型非法",IF(AND($F139&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C139,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F139="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C139,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H139),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A139:$G139)=0,"",IF(LEFT($G139,4)="待确认：","待确认",IF(OR($A139="",$B139="",$C139="",$D139="",$E139=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B139))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A139))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E139="S",$E139="M",$E139="L")),"复杂度非法",IF(NOT(OR($F139="",$F139="内部集成",$F139="外部集成")),"集成类型非法",IF(AND($F139&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C139,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F139="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C139,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H139),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="140" ht="42" customHeight="1">
@@ -5662,7 +5662,7 @@
         <s:f>IF(COUNTA($A140:$G140)=0,"",IF($F140="",0,IF(NOT(ISNUMBER($I140)),"",IF($F140="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I140,1),IF($F140="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I140,1),"")))))</s:f>
       </s:c>
       <s:c r="L140" t="str" s="5">
-        <s:f>IF(COUNTA($A140:$G140)=0,"",IF(OR($A140="",$B140="",$C140="",$D140="",$E140=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B140))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A140))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E140="S",$E140="M",$E140="L")),"复杂度非法",IF(NOT(OR($F140="",$F140="内部集成",$F140="外部集成")),"集成类型非法",IF(AND($F140&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C140,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F140="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C140,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H140),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A140:$G140)=0,"",IF(LEFT($G140,4)="待确认：","待确认",IF(OR($A140="",$B140="",$C140="",$D140="",$E140=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B140))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A140))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E140="S",$E140="M",$E140="L")),"复杂度非法",IF(NOT(OR($F140="",$F140="内部集成",$F140="外部集成")),"集成类型非法",IF(AND($F140&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C140,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F140="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C140,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H140),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="141" ht="42" customHeight="1">
@@ -5686,7 +5686,7 @@
         <s:f>IF(COUNTA($A141:$G141)=0,"",IF($F141="",0,IF(NOT(ISNUMBER($I141)),"",IF($F141="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I141,1),IF($F141="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I141,1),"")))))</s:f>
       </s:c>
       <s:c r="L141" t="str" s="5">
-        <s:f>IF(COUNTA($A141:$G141)=0,"",IF(OR($A141="",$B141="",$C141="",$D141="",$E141=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B141))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A141))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E141="S",$E141="M",$E141="L")),"复杂度非法",IF(NOT(OR($F141="",$F141="内部集成",$F141="外部集成")),"集成类型非法",IF(AND($F141&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C141,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F141="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C141,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H141),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A141:$G141)=0,"",IF(LEFT($G141,4)="待确认：","待确认",IF(OR($A141="",$B141="",$C141="",$D141="",$E141=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B141))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A141))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E141="S",$E141="M",$E141="L")),"复杂度非法",IF(NOT(OR($F141="",$F141="内部集成",$F141="外部集成")),"集成类型非法",IF(AND($F141&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C141,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F141="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C141,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H141),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="142" ht="42" customHeight="1">
@@ -5710,7 +5710,7 @@
         <s:f>IF(COUNTA($A142:$G142)=0,"",IF($F142="",0,IF(NOT(ISNUMBER($I142)),"",IF($F142="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I142,1),IF($F142="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I142,1),"")))))</s:f>
       </s:c>
       <s:c r="L142" t="str" s="5">
-        <s:f>IF(COUNTA($A142:$G142)=0,"",IF(OR($A142="",$B142="",$C142="",$D142="",$E142=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B142))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A142))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E142="S",$E142="M",$E142="L")),"复杂度非法",IF(NOT(OR($F142="",$F142="内部集成",$F142="外部集成")),"集成类型非法",IF(AND($F142&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C142,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F142="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C142,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H142),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A142:$G142)=0,"",IF(LEFT($G142,4)="待确认：","待确认",IF(OR($A142="",$B142="",$C142="",$D142="",$E142=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B142))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A142))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E142="S",$E142="M",$E142="L")),"复杂度非法",IF(NOT(OR($F142="",$F142="内部集成",$F142="外部集成")),"集成类型非法",IF(AND($F142&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C142,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F142="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C142,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H142),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="143" ht="42" customHeight="1">
@@ -5734,7 +5734,7 @@
         <s:f>IF(COUNTA($A143:$G143)=0,"",IF($F143="",0,IF(NOT(ISNUMBER($I143)),"",IF($F143="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I143,1),IF($F143="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I143,1),"")))))</s:f>
       </s:c>
       <s:c r="L143" t="str" s="5">
-        <s:f>IF(COUNTA($A143:$G143)=0,"",IF(OR($A143="",$B143="",$C143="",$D143="",$E143=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B143))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A143))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E143="S",$E143="M",$E143="L")),"复杂度非法",IF(NOT(OR($F143="",$F143="内部集成",$F143="外部集成")),"集成类型非法",IF(AND($F143&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C143,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F143="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C143,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H143),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A143:$G143)=0,"",IF(LEFT($G143,4)="待确认：","待确认",IF(OR($A143="",$B143="",$C143="",$D143="",$E143=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B143))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A143))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E143="S",$E143="M",$E143="L")),"复杂度非法",IF(NOT(OR($F143="",$F143="内部集成",$F143="外部集成")),"集成类型非法",IF(AND($F143&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C143,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F143="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C143,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H143),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="144" ht="42" customHeight="1">
@@ -5758,7 +5758,7 @@
         <s:f>IF(COUNTA($A144:$G144)=0,"",IF($F144="",0,IF(NOT(ISNUMBER($I144)),"",IF($F144="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I144,1),IF($F144="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I144,1),"")))))</s:f>
       </s:c>
       <s:c r="L144" t="str" s="5">
-        <s:f>IF(COUNTA($A144:$G144)=0,"",IF(OR($A144="",$B144="",$C144="",$D144="",$E144=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B144))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A144))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E144="S",$E144="M",$E144="L")),"复杂度非法",IF(NOT(OR($F144="",$F144="内部集成",$F144="外部集成")),"集成类型非法",IF(AND($F144&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C144,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F144="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C144,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H144),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A144:$G144)=0,"",IF(LEFT($G144,4)="待确认：","待确认",IF(OR($A144="",$B144="",$C144="",$D144="",$E144=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B144))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A144))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E144="S",$E144="M",$E144="L")),"复杂度非法",IF(NOT(OR($F144="",$F144="内部集成",$F144="外部集成")),"集成类型非法",IF(AND($F144&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C144,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F144="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C144,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H144),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="145" ht="42" customHeight="1">
@@ -5782,7 +5782,7 @@
         <s:f>IF(COUNTA($A145:$G145)=0,"",IF($F145="",0,IF(NOT(ISNUMBER($I145)),"",IF($F145="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I145,1),IF($F145="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I145,1),"")))))</s:f>
       </s:c>
       <s:c r="L145" t="str" s="5">
-        <s:f>IF(COUNTA($A145:$G145)=0,"",IF(OR($A145="",$B145="",$C145="",$D145="",$E145=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B145))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A145))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E145="S",$E145="M",$E145="L")),"复杂度非法",IF(NOT(OR($F145="",$F145="内部集成",$F145="外部集成")),"集成类型非法",IF(AND($F145&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C145,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F145="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C145,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H145),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A145:$G145)=0,"",IF(LEFT($G145,4)="待确认：","待确认",IF(OR($A145="",$B145="",$C145="",$D145="",$E145=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B145))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A145))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E145="S",$E145="M",$E145="L")),"复杂度非法",IF(NOT(OR($F145="",$F145="内部集成",$F145="外部集成")),"集成类型非法",IF(AND($F145&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C145,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F145="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C145,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H145),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="146" ht="42" customHeight="1">
@@ -5806,7 +5806,7 @@
         <s:f>IF(COUNTA($A146:$G146)=0,"",IF($F146="",0,IF(NOT(ISNUMBER($I146)),"",IF($F146="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I146,1),IF($F146="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I146,1),"")))))</s:f>
       </s:c>
       <s:c r="L146" t="str" s="5">
-        <s:f>IF(COUNTA($A146:$G146)=0,"",IF(OR($A146="",$B146="",$C146="",$D146="",$E146=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B146))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A146))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E146="S",$E146="M",$E146="L")),"复杂度非法",IF(NOT(OR($F146="",$F146="内部集成",$F146="外部集成")),"集成类型非法",IF(AND($F146&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C146,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F146="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C146,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H146),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A146:$G146)=0,"",IF(LEFT($G146,4)="待确认：","待确认",IF(OR($A146="",$B146="",$C146="",$D146="",$E146=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B146))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A146))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E146="S",$E146="M",$E146="L")),"复杂度非法",IF(NOT(OR($F146="",$F146="内部集成",$F146="外部集成")),"集成类型非法",IF(AND($F146&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C146,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F146="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C146,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H146),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="147" ht="42" customHeight="1">
@@ -5830,7 +5830,7 @@
         <s:f>IF(COUNTA($A147:$G147)=0,"",IF($F147="",0,IF(NOT(ISNUMBER($I147)),"",IF($F147="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I147,1),IF($F147="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I147,1),"")))))</s:f>
       </s:c>
       <s:c r="L147" t="str" s="5">
-        <s:f>IF(COUNTA($A147:$G147)=0,"",IF(OR($A147="",$B147="",$C147="",$D147="",$E147=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B147))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A147))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E147="S",$E147="M",$E147="L")),"复杂度非法",IF(NOT(OR($F147="",$F147="内部集成",$F147="外部集成")),"集成类型非法",IF(AND($F147&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C147,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F147="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C147,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H147),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A147:$G147)=0,"",IF(LEFT($G147,4)="待确认：","待确认",IF(OR($A147="",$B147="",$C147="",$D147="",$E147=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B147))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A147))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E147="S",$E147="M",$E147="L")),"复杂度非法",IF(NOT(OR($F147="",$F147="内部集成",$F147="外部集成")),"集成类型非法",IF(AND($F147&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C147,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F147="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C147,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H147),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="148" ht="42" customHeight="1">
@@ -5854,7 +5854,7 @@
         <s:f>IF(COUNTA($A148:$G148)=0,"",IF($F148="",0,IF(NOT(ISNUMBER($I148)),"",IF($F148="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I148,1),IF($F148="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I148,1),"")))))</s:f>
       </s:c>
       <s:c r="L148" t="str" s="5">
-        <s:f>IF(COUNTA($A148:$G148)=0,"",IF(OR($A148="",$B148="",$C148="",$D148="",$E148=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B148))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A148))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E148="S",$E148="M",$E148="L")),"复杂度非法",IF(NOT(OR($F148="",$F148="内部集成",$F148="外部集成")),"集成类型非法",IF(AND($F148&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C148,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F148="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C148,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H148),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A148:$G148)=0,"",IF(LEFT($G148,4)="待确认：","待确认",IF(OR($A148="",$B148="",$C148="",$D148="",$E148=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B148))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A148))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E148="S",$E148="M",$E148="L")),"复杂度非法",IF(NOT(OR($F148="",$F148="内部集成",$F148="外部集成")),"集成类型非法",IF(AND($F148&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C148,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F148="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C148,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H148),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="149" ht="42" customHeight="1">
@@ -5878,7 +5878,7 @@
         <s:f>IF(COUNTA($A149:$G149)=0,"",IF($F149="",0,IF(NOT(ISNUMBER($I149)),"",IF($F149="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I149,1),IF($F149="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I149,1),"")))))</s:f>
       </s:c>
       <s:c r="L149" t="str" s="5">
-        <s:f>IF(COUNTA($A149:$G149)=0,"",IF(OR($A149="",$B149="",$C149="",$D149="",$E149=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B149))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A149))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E149="S",$E149="M",$E149="L")),"复杂度非法",IF(NOT(OR($F149="",$F149="内部集成",$F149="外部集成")),"集成类型非法",IF(AND($F149&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C149,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F149="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C149,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H149),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A149:$G149)=0,"",IF(LEFT($G149,4)="待确认：","待确认",IF(OR($A149="",$B149="",$C149="",$D149="",$E149=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B149))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A149))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E149="S",$E149="M",$E149="L")),"复杂度非法",IF(NOT(OR($F149="",$F149="内部集成",$F149="外部集成")),"集成类型非法",IF(AND($F149&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C149,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F149="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C149,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H149),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="150" ht="42" customHeight="1">
@@ -5902,7 +5902,7 @@
         <s:f>IF(COUNTA($A150:$G150)=0,"",IF($F150="",0,IF(NOT(ISNUMBER($I150)),"",IF($F150="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I150,1),IF($F150="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I150,1),"")))))</s:f>
       </s:c>
       <s:c r="L150" t="str" s="5">
-        <s:f>IF(COUNTA($A150:$G150)=0,"",IF(OR($A150="",$B150="",$C150="",$D150="",$E150=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B150))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A150))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E150="S",$E150="M",$E150="L")),"复杂度非法",IF(NOT(OR($F150="",$F150="内部集成",$F150="外部集成")),"集成类型非法",IF(AND($F150&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C150,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F150="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C150,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H150),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A150:$G150)=0,"",IF(LEFT($G150,4)="待确认：","待确认",IF(OR($A150="",$B150="",$C150="",$D150="",$E150=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B150))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A150))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E150="S",$E150="M",$E150="L")),"复杂度非法",IF(NOT(OR($F150="",$F150="内部集成",$F150="外部集成")),"集成类型非法",IF(AND($F150&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C150,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F150="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C150,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H150),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="151" ht="42" customHeight="1">
@@ -5926,7 +5926,7 @@
         <s:f>IF(COUNTA($A151:$G151)=0,"",IF($F151="",0,IF(NOT(ISNUMBER($I151)),"",IF($F151="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I151,1),IF($F151="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I151,1),"")))))</s:f>
       </s:c>
       <s:c r="L151" t="str" s="5">
-        <s:f>IF(COUNTA($A151:$G151)=0,"",IF(OR($A151="",$B151="",$C151="",$D151="",$E151=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B151))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A151))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E151="S",$E151="M",$E151="L")),"复杂度非法",IF(NOT(OR($F151="",$F151="内部集成",$F151="外部集成")),"集成类型非法",IF(AND($F151&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C151,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F151="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C151,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H151),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A151:$G151)=0,"",IF(LEFT($G151,4)="待确认：","待确认",IF(OR($A151="",$B151="",$C151="",$D151="",$E151=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B151))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A151))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E151="S",$E151="M",$E151="L")),"复杂度非法",IF(NOT(OR($F151="",$F151="内部集成",$F151="外部集成")),"集成类型非法",IF(AND($F151&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C151,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F151="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C151,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H151),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="152" ht="42" customHeight="1">
@@ -5950,7 +5950,7 @@
         <s:f>IF(COUNTA($A152:$G152)=0,"",IF($F152="",0,IF(NOT(ISNUMBER($I152)),"",IF($F152="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I152,1),IF($F152="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I152,1),"")))))</s:f>
       </s:c>
       <s:c r="L152" t="str" s="5">
-        <s:f>IF(COUNTA($A152:$G152)=0,"",IF(OR($A152="",$B152="",$C152="",$D152="",$E152=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B152))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A152))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E152="S",$E152="M",$E152="L")),"复杂度非法",IF(NOT(OR($F152="",$F152="内部集成",$F152="外部集成")),"集成类型非法",IF(AND($F152&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C152,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F152="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C152,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H152),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A152:$G152)=0,"",IF(LEFT($G152,4)="待确认：","待确认",IF(OR($A152="",$B152="",$C152="",$D152="",$E152=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B152))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A152))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E152="S",$E152="M",$E152="L")),"复杂度非法",IF(NOT(OR($F152="",$F152="内部集成",$F152="外部集成")),"集成类型非法",IF(AND($F152&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C152,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F152="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C152,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H152),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="153" ht="42" customHeight="1">
@@ -5974,7 +5974,7 @@
         <s:f>IF(COUNTA($A153:$G153)=0,"",IF($F153="",0,IF(NOT(ISNUMBER($I153)),"",IF($F153="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I153,1),IF($F153="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I153,1),"")))))</s:f>
       </s:c>
       <s:c r="L153" t="str" s="5">
-        <s:f>IF(COUNTA($A153:$G153)=0,"",IF(OR($A153="",$B153="",$C153="",$D153="",$E153=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B153))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A153))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E153="S",$E153="M",$E153="L")),"复杂度非法",IF(NOT(OR($F153="",$F153="内部集成",$F153="外部集成")),"集成类型非法",IF(AND($F153&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C153,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F153="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C153,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H153),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A153:$G153)=0,"",IF(LEFT($G153,4)="待确认：","待确认",IF(OR($A153="",$B153="",$C153="",$D153="",$E153=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B153))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A153))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E153="S",$E153="M",$E153="L")),"复杂度非法",IF(NOT(OR($F153="",$F153="内部集成",$F153="外部集成")),"集成类型非法",IF(AND($F153&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C153,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F153="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C153,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H153),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="154" ht="42" customHeight="1">
@@ -5998,7 +5998,7 @@
         <s:f>IF(COUNTA($A154:$G154)=0,"",IF($F154="",0,IF(NOT(ISNUMBER($I154)),"",IF($F154="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I154,1),IF($F154="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I154,1),"")))))</s:f>
       </s:c>
       <s:c r="L154" t="str" s="5">
-        <s:f>IF(COUNTA($A154:$G154)=0,"",IF(OR($A154="",$B154="",$C154="",$D154="",$E154=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B154))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A154))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E154="S",$E154="M",$E154="L")),"复杂度非法",IF(NOT(OR($F154="",$F154="内部集成",$F154="外部集成")),"集成类型非法",IF(AND($F154&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C154,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F154="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C154,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H154),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A154:$G154)=0,"",IF(LEFT($G154,4)="待确认：","待确认",IF(OR($A154="",$B154="",$C154="",$D154="",$E154=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B154))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A154))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E154="S",$E154="M",$E154="L")),"复杂度非法",IF(NOT(OR($F154="",$F154="内部集成",$F154="外部集成")),"集成类型非法",IF(AND($F154&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C154,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F154="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C154,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H154),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="155" ht="42" customHeight="1">
@@ -6022,7 +6022,7 @@
         <s:f>IF(COUNTA($A155:$G155)=0,"",IF($F155="",0,IF(NOT(ISNUMBER($I155)),"",IF($F155="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I155,1),IF($F155="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I155,1),"")))))</s:f>
       </s:c>
       <s:c r="L155" t="str" s="5">
-        <s:f>IF(COUNTA($A155:$G155)=0,"",IF(OR($A155="",$B155="",$C155="",$D155="",$E155=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B155))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A155))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E155="S",$E155="M",$E155="L")),"复杂度非法",IF(NOT(OR($F155="",$F155="内部集成",$F155="外部集成")),"集成类型非法",IF(AND($F155&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C155,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F155="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C155,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H155),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A155:$G155)=0,"",IF(LEFT($G155,4)="待确认：","待确认",IF(OR($A155="",$B155="",$C155="",$D155="",$E155=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B155))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A155))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E155="S",$E155="M",$E155="L")),"复杂度非法",IF(NOT(OR($F155="",$F155="内部集成",$F155="外部集成")),"集成类型非法",IF(AND($F155&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C155,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F155="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C155,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H155),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="156" ht="42" customHeight="1">
@@ -6046,7 +6046,7 @@
         <s:f>IF(COUNTA($A156:$G156)=0,"",IF($F156="",0,IF(NOT(ISNUMBER($I156)),"",IF($F156="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I156,1),IF($F156="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I156,1),"")))))</s:f>
       </s:c>
       <s:c r="L156" t="str" s="5">
-        <s:f>IF(COUNTA($A156:$G156)=0,"",IF(OR($A156="",$B156="",$C156="",$D156="",$E156=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B156))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A156))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E156="S",$E156="M",$E156="L")),"复杂度非法",IF(NOT(OR($F156="",$F156="内部集成",$F156="外部集成")),"集成类型非法",IF(AND($F156&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C156,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F156="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C156,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H156),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A156:$G156)=0,"",IF(LEFT($G156,4)="待确认：","待确认",IF(OR($A156="",$B156="",$C156="",$D156="",$E156=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B156))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A156))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E156="S",$E156="M",$E156="L")),"复杂度非法",IF(NOT(OR($F156="",$F156="内部集成",$F156="外部集成")),"集成类型非法",IF(AND($F156&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C156,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F156="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C156,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H156),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="157" ht="42" customHeight="1">
@@ -6070,7 +6070,7 @@
         <s:f>IF(COUNTA($A157:$G157)=0,"",IF($F157="",0,IF(NOT(ISNUMBER($I157)),"",IF($F157="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I157,1),IF($F157="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I157,1),"")))))</s:f>
       </s:c>
       <s:c r="L157" t="str" s="5">
-        <s:f>IF(COUNTA($A157:$G157)=0,"",IF(OR($A157="",$B157="",$C157="",$D157="",$E157=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B157))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A157))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E157="S",$E157="M",$E157="L")),"复杂度非法",IF(NOT(OR($F157="",$F157="内部集成",$F157="外部集成")),"集成类型非法",IF(AND($F157&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C157,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F157="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C157,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H157),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A157:$G157)=0,"",IF(LEFT($G157,4)="待确认：","待确认",IF(OR($A157="",$B157="",$C157="",$D157="",$E157=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B157))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A157))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E157="S",$E157="M",$E157="L")),"复杂度非法",IF(NOT(OR($F157="",$F157="内部集成",$F157="外部集成")),"集成类型非法",IF(AND($F157&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C157,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F157="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C157,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H157),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="158" ht="42" customHeight="1">
@@ -6094,7 +6094,7 @@
         <s:f>IF(COUNTA($A158:$G158)=0,"",IF($F158="",0,IF(NOT(ISNUMBER($I158)),"",IF($F158="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I158,1),IF($F158="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I158,1),"")))))</s:f>
       </s:c>
       <s:c r="L158" t="str" s="5">
-        <s:f>IF(COUNTA($A158:$G158)=0,"",IF(OR($A158="",$B158="",$C158="",$D158="",$E158=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B158))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A158))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E158="S",$E158="M",$E158="L")),"复杂度非法",IF(NOT(OR($F158="",$F158="内部集成",$F158="外部集成")),"集成类型非法",IF(AND($F158&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C158,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F158="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C158,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H158),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A158:$G158)=0,"",IF(LEFT($G158,4)="待确认：","待确认",IF(OR($A158="",$B158="",$C158="",$D158="",$E158=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B158))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A158))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E158="S",$E158="M",$E158="L")),"复杂度非法",IF(NOT(OR($F158="",$F158="内部集成",$F158="外部集成")),"集成类型非法",IF(AND($F158&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C158,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F158="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C158,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H158),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="159" ht="42" customHeight="1">
@@ -6118,7 +6118,7 @@
         <s:f>IF(COUNTA($A159:$G159)=0,"",IF($F159="",0,IF(NOT(ISNUMBER($I159)),"",IF($F159="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I159,1),IF($F159="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I159,1),"")))))</s:f>
       </s:c>
       <s:c r="L159" t="str" s="5">
-        <s:f>IF(COUNTA($A159:$G159)=0,"",IF(OR($A159="",$B159="",$C159="",$D159="",$E159=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B159))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A159))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E159="S",$E159="M",$E159="L")),"复杂度非法",IF(NOT(OR($F159="",$F159="内部集成",$F159="外部集成")),"集成类型非法",IF(AND($F159&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C159,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F159="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C159,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H159),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A159:$G159)=0,"",IF(LEFT($G159,4)="待确认：","待确认",IF(OR($A159="",$B159="",$C159="",$D159="",$E159=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B159))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A159))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E159="S",$E159="M",$E159="L")),"复杂度非法",IF(NOT(OR($F159="",$F159="内部集成",$F159="外部集成")),"集成类型非法",IF(AND($F159&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C159,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F159="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C159,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H159),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="160" ht="42" customHeight="1">
@@ -6142,7 +6142,7 @@
         <s:f>IF(COUNTA($A160:$G160)=0,"",IF($F160="",0,IF(NOT(ISNUMBER($I160)),"",IF($F160="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I160,1),IF($F160="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I160,1),"")))))</s:f>
       </s:c>
       <s:c r="L160" t="str" s="5">
-        <s:f>IF(COUNTA($A160:$G160)=0,"",IF(OR($A160="",$B160="",$C160="",$D160="",$E160=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B160))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A160))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E160="S",$E160="M",$E160="L")),"复杂度非法",IF(NOT(OR($F160="",$F160="内部集成",$F160="外部集成")),"集成类型非法",IF(AND($F160&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C160,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F160="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C160,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H160),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A160:$G160)=0,"",IF(LEFT($G160,4)="待确认：","待确认",IF(OR($A160="",$B160="",$C160="",$D160="",$E160=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B160))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A160))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E160="S",$E160="M",$E160="L")),"复杂度非法",IF(NOT(OR($F160="",$F160="内部集成",$F160="外部集成")),"集成类型非法",IF(AND($F160&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C160,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F160="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C160,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H160),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="161" ht="42" customHeight="1">
@@ -6166,7 +6166,7 @@
         <s:f>IF(COUNTA($A161:$G161)=0,"",IF($F161="",0,IF(NOT(ISNUMBER($I161)),"",IF($F161="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I161,1),IF($F161="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I161,1),"")))))</s:f>
       </s:c>
       <s:c r="L161" t="str" s="5">
-        <s:f>IF(COUNTA($A161:$G161)=0,"",IF(OR($A161="",$B161="",$C161="",$D161="",$E161=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B161))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A161))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E161="S",$E161="M",$E161="L")),"复杂度非法",IF(NOT(OR($F161="",$F161="内部集成",$F161="外部集成")),"集成类型非法",IF(AND($F161&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C161,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F161="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C161,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H161),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A161:$G161)=0,"",IF(LEFT($G161,4)="待确认：","待确认",IF(OR($A161="",$B161="",$C161="",$D161="",$E161=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B161))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A161))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E161="S",$E161="M",$E161="L")),"复杂度非法",IF(NOT(OR($F161="",$F161="内部集成",$F161="外部集成")),"集成类型非法",IF(AND($F161&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C161,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F161="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C161,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H161),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="162" ht="42" customHeight="1">
@@ -6190,7 +6190,7 @@
         <s:f>IF(COUNTA($A162:$G162)=0,"",IF($F162="",0,IF(NOT(ISNUMBER($I162)),"",IF($F162="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I162,1),IF($F162="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I162,1),"")))))</s:f>
       </s:c>
       <s:c r="L162" t="str" s="5">
-        <s:f>IF(COUNTA($A162:$G162)=0,"",IF(OR($A162="",$B162="",$C162="",$D162="",$E162=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B162))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A162))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E162="S",$E162="M",$E162="L")),"复杂度非法",IF(NOT(OR($F162="",$F162="内部集成",$F162="外部集成")),"集成类型非法",IF(AND($F162&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C162,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F162="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C162,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H162),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A162:$G162)=0,"",IF(LEFT($G162,4)="待确认：","待确认",IF(OR($A162="",$B162="",$C162="",$D162="",$E162=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B162))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A162))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E162="S",$E162="M",$E162="L")),"复杂度非法",IF(NOT(OR($F162="",$F162="内部集成",$F162="外部集成")),"集成类型非法",IF(AND($F162&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C162,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F162="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C162,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H162),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="163" ht="42" customHeight="1">
@@ -6214,7 +6214,7 @@
         <s:f>IF(COUNTA($A163:$G163)=0,"",IF($F163="",0,IF(NOT(ISNUMBER($I163)),"",IF($F163="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I163,1),IF($F163="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I163,1),"")))))</s:f>
       </s:c>
       <s:c r="L163" t="str" s="5">
-        <s:f>IF(COUNTA($A163:$G163)=0,"",IF(OR($A163="",$B163="",$C163="",$D163="",$E163=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B163))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A163))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E163="S",$E163="M",$E163="L")),"复杂度非法",IF(NOT(OR($F163="",$F163="内部集成",$F163="外部集成")),"集成类型非法",IF(AND($F163&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C163,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F163="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C163,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H163),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A163:$G163)=0,"",IF(LEFT($G163,4)="待确认：","待确认",IF(OR($A163="",$B163="",$C163="",$D163="",$E163=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B163))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A163))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E163="S",$E163="M",$E163="L")),"复杂度非法",IF(NOT(OR($F163="",$F163="内部集成",$F163="外部集成")),"集成类型非法",IF(AND($F163&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C163,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F163="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C163,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H163),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="164" ht="42" customHeight="1">
@@ -6238,7 +6238,7 @@
         <s:f>IF(COUNTA($A164:$G164)=0,"",IF($F164="",0,IF(NOT(ISNUMBER($I164)),"",IF($F164="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I164,1),IF($F164="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I164,1),"")))))</s:f>
       </s:c>
       <s:c r="L164" t="str" s="5">
-        <s:f>IF(COUNTA($A164:$G164)=0,"",IF(OR($A164="",$B164="",$C164="",$D164="",$E164=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B164))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A164))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E164="S",$E164="M",$E164="L")),"复杂度非法",IF(NOT(OR($F164="",$F164="内部集成",$F164="外部集成")),"集成类型非法",IF(AND($F164&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C164,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F164="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C164,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H164),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A164:$G164)=0,"",IF(LEFT($G164,4)="待确认：","待确认",IF(OR($A164="",$B164="",$C164="",$D164="",$E164=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B164))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A164))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E164="S",$E164="M",$E164="L")),"复杂度非法",IF(NOT(OR($F164="",$F164="内部集成",$F164="外部集成")),"集成类型非法",IF(AND($F164&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C164,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F164="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C164,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H164),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="165" ht="42" customHeight="1">
@@ -6262,7 +6262,7 @@
         <s:f>IF(COUNTA($A165:$G165)=0,"",IF($F165="",0,IF(NOT(ISNUMBER($I165)),"",IF($F165="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I165,1),IF($F165="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I165,1),"")))))</s:f>
       </s:c>
       <s:c r="L165" t="str" s="5">
-        <s:f>IF(COUNTA($A165:$G165)=0,"",IF(OR($A165="",$B165="",$C165="",$D165="",$E165=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B165))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A165))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E165="S",$E165="M",$E165="L")),"复杂度非法",IF(NOT(OR($F165="",$F165="内部集成",$F165="外部集成")),"集成类型非法",IF(AND($F165&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C165,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F165="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C165,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H165),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A165:$G165)=0,"",IF(LEFT($G165,4)="待确认：","待确认",IF(OR($A165="",$B165="",$C165="",$D165="",$E165=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B165))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A165))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E165="S",$E165="M",$E165="L")),"复杂度非法",IF(NOT(OR($F165="",$F165="内部集成",$F165="外部集成")),"集成类型非法",IF(AND($F165&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C165,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F165="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C165,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H165),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="166" ht="42" customHeight="1">
@@ -6286,7 +6286,7 @@
         <s:f>IF(COUNTA($A166:$G166)=0,"",IF($F166="",0,IF(NOT(ISNUMBER($I166)),"",IF($F166="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I166,1),IF($F166="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I166,1),"")))))</s:f>
       </s:c>
       <s:c r="L166" t="str" s="5">
-        <s:f>IF(COUNTA($A166:$G166)=0,"",IF(OR($A166="",$B166="",$C166="",$D166="",$E166=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B166))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A166))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E166="S",$E166="M",$E166="L")),"复杂度非法",IF(NOT(OR($F166="",$F166="内部集成",$F166="外部集成")),"集成类型非法",IF(AND($F166&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C166,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F166="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C166,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H166),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A166:$G166)=0,"",IF(LEFT($G166,4)="待确认：","待确认",IF(OR($A166="",$B166="",$C166="",$D166="",$E166=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B166))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A166))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E166="S",$E166="M",$E166="L")),"复杂度非法",IF(NOT(OR($F166="",$F166="内部集成",$F166="外部集成")),"集成类型非法",IF(AND($F166&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C166,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F166="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C166,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H166),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="167" ht="42" customHeight="1">
@@ -6310,7 +6310,7 @@
         <s:f>IF(COUNTA($A167:$G167)=0,"",IF($F167="",0,IF(NOT(ISNUMBER($I167)),"",IF($F167="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I167,1),IF($F167="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I167,1),"")))))</s:f>
       </s:c>
       <s:c r="L167" t="str" s="5">
-        <s:f>IF(COUNTA($A167:$G167)=0,"",IF(OR($A167="",$B167="",$C167="",$D167="",$E167=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B167))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A167))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E167="S",$E167="M",$E167="L")),"复杂度非法",IF(NOT(OR($F167="",$F167="内部集成",$F167="外部集成")),"集成类型非法",IF(AND($F167&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C167,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F167="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C167,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H167),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A167:$G167)=0,"",IF(LEFT($G167,4)="待确认：","待确认",IF(OR($A167="",$B167="",$C167="",$D167="",$E167=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B167))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A167))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E167="S",$E167="M",$E167="L")),"复杂度非法",IF(NOT(OR($F167="",$F167="内部集成",$F167="外部集成")),"集成类型非法",IF(AND($F167&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C167,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F167="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C167,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H167),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="168" ht="42" customHeight="1">
@@ -6334,7 +6334,7 @@
         <s:f>IF(COUNTA($A168:$G168)=0,"",IF($F168="",0,IF(NOT(ISNUMBER($I168)),"",IF($F168="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I168,1),IF($F168="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I168,1),"")))))</s:f>
       </s:c>
       <s:c r="L168" t="str" s="5">
-        <s:f>IF(COUNTA($A168:$G168)=0,"",IF(OR($A168="",$B168="",$C168="",$D168="",$E168=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B168))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A168))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E168="S",$E168="M",$E168="L")),"复杂度非法",IF(NOT(OR($F168="",$F168="内部集成",$F168="外部集成")),"集成类型非法",IF(AND($F168&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C168,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F168="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C168,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H168),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A168:$G168)=0,"",IF(LEFT($G168,4)="待确认：","待确认",IF(OR($A168="",$B168="",$C168="",$D168="",$E168=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B168))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A168))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E168="S",$E168="M",$E168="L")),"复杂度非法",IF(NOT(OR($F168="",$F168="内部集成",$F168="外部集成")),"集成类型非法",IF(AND($F168&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C168,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F168="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C168,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H168),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="169" ht="42" customHeight="1">
@@ -6358,7 +6358,7 @@
         <s:f>IF(COUNTA($A169:$G169)=0,"",IF($F169="",0,IF(NOT(ISNUMBER($I169)),"",IF($F169="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I169,1),IF($F169="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I169,1),"")))))</s:f>
       </s:c>
       <s:c r="L169" t="str" s="5">
-        <s:f>IF(COUNTA($A169:$G169)=0,"",IF(OR($A169="",$B169="",$C169="",$D169="",$E169=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B169))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A169))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E169="S",$E169="M",$E169="L")),"复杂度非法",IF(NOT(OR($F169="",$F169="内部集成",$F169="外部集成")),"集成类型非法",IF(AND($F169&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C169,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F169="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C169,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H169),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A169:$G169)=0,"",IF(LEFT($G169,4)="待确认：","待确认",IF(OR($A169="",$B169="",$C169="",$D169="",$E169=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B169))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A169))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E169="S",$E169="M",$E169="L")),"复杂度非法",IF(NOT(OR($F169="",$F169="内部集成",$F169="外部集成")),"集成类型非法",IF(AND($F169&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C169,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F169="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C169,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H169),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="170" ht="42" customHeight="1">
@@ -6382,7 +6382,7 @@
         <s:f>IF(COUNTA($A170:$G170)=0,"",IF($F170="",0,IF(NOT(ISNUMBER($I170)),"",IF($F170="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I170,1),IF($F170="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I170,1),"")))))</s:f>
       </s:c>
       <s:c r="L170" t="str" s="5">
-        <s:f>IF(COUNTA($A170:$G170)=0,"",IF(OR($A170="",$B170="",$C170="",$D170="",$E170=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B170))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A170))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E170="S",$E170="M",$E170="L")),"复杂度非法",IF(NOT(OR($F170="",$F170="内部集成",$F170="外部集成")),"集成类型非法",IF(AND($F170&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C170,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F170="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C170,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H170),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A170:$G170)=0,"",IF(LEFT($G170,4)="待确认：","待确认",IF(OR($A170="",$B170="",$C170="",$D170="",$E170=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B170))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A170))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E170="S",$E170="M",$E170="L")),"复杂度非法",IF(NOT(OR($F170="",$F170="内部集成",$F170="外部集成")),"集成类型非法",IF(AND($F170&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C170,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F170="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C170,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H170),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="171" ht="42" customHeight="1">
@@ -6406,7 +6406,7 @@
         <s:f>IF(COUNTA($A171:$G171)=0,"",IF($F171="",0,IF(NOT(ISNUMBER($I171)),"",IF($F171="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I171,1),IF($F171="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I171,1),"")))))</s:f>
       </s:c>
       <s:c r="L171" t="str" s="5">
-        <s:f>IF(COUNTA($A171:$G171)=0,"",IF(OR($A171="",$B171="",$C171="",$D171="",$E171=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B171))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A171))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E171="S",$E171="M",$E171="L")),"复杂度非法",IF(NOT(OR($F171="",$F171="内部集成",$F171="外部集成")),"集成类型非法",IF(AND($F171&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C171,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F171="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C171,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H171),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A171:$G171)=0,"",IF(LEFT($G171,4)="待确认：","待确认",IF(OR($A171="",$B171="",$C171="",$D171="",$E171=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B171))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A171))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E171="S",$E171="M",$E171="L")),"复杂度非法",IF(NOT(OR($F171="",$F171="内部集成",$F171="外部集成")),"集成类型非法",IF(AND($F171&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C171,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F171="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C171,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H171),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="172" ht="42" customHeight="1">
@@ -6430,7 +6430,7 @@
         <s:f>IF(COUNTA($A172:$G172)=0,"",IF($F172="",0,IF(NOT(ISNUMBER($I172)),"",IF($F172="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I172,1),IF($F172="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I172,1),"")))))</s:f>
       </s:c>
       <s:c r="L172" t="str" s="5">
-        <s:f>IF(COUNTA($A172:$G172)=0,"",IF(OR($A172="",$B172="",$C172="",$D172="",$E172=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B172))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A172))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E172="S",$E172="M",$E172="L")),"复杂度非法",IF(NOT(OR($F172="",$F172="内部集成",$F172="外部集成")),"集成类型非法",IF(AND($F172&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C172,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F172="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C172,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H172),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A172:$G172)=0,"",IF(LEFT($G172,4)="待确认：","待确认",IF(OR($A172="",$B172="",$C172="",$D172="",$E172=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B172))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A172))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E172="S",$E172="M",$E172="L")),"复杂度非法",IF(NOT(OR($F172="",$F172="内部集成",$F172="外部集成")),"集成类型非法",IF(AND($F172&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C172,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F172="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C172,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H172),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="173" ht="42" customHeight="1">
@@ -6454,7 +6454,7 @@
         <s:f>IF(COUNTA($A173:$G173)=0,"",IF($F173="",0,IF(NOT(ISNUMBER($I173)),"",IF($F173="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I173,1),IF($F173="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I173,1),"")))))</s:f>
       </s:c>
       <s:c r="L173" t="str" s="5">
-        <s:f>IF(COUNTA($A173:$G173)=0,"",IF(OR($A173="",$B173="",$C173="",$D173="",$E173=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B173))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A173))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E173="S",$E173="M",$E173="L")),"复杂度非法",IF(NOT(OR($F173="",$F173="内部集成",$F173="外部集成")),"集成类型非法",IF(AND($F173&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C173,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F173="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C173,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H173),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A173:$G173)=0,"",IF(LEFT($G173,4)="待确认：","待确认",IF(OR($A173="",$B173="",$C173="",$D173="",$E173=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B173))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A173))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E173="S",$E173="M",$E173="L")),"复杂度非法",IF(NOT(OR($F173="",$F173="内部集成",$F173="外部集成")),"集成类型非法",IF(AND($F173&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C173,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F173="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C173,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H173),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="174" ht="42" customHeight="1">
@@ -6478,7 +6478,7 @@
         <s:f>IF(COUNTA($A174:$G174)=0,"",IF($F174="",0,IF(NOT(ISNUMBER($I174)),"",IF($F174="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I174,1),IF($F174="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I174,1),"")))))</s:f>
       </s:c>
       <s:c r="L174" t="str" s="5">
-        <s:f>IF(COUNTA($A174:$G174)=0,"",IF(OR($A174="",$B174="",$C174="",$D174="",$E174=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B174))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A174))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E174="S",$E174="M",$E174="L")),"复杂度非法",IF(NOT(OR($F174="",$F174="内部集成",$F174="外部集成")),"集成类型非法",IF(AND($F174&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C174,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F174="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C174,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H174),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A174:$G174)=0,"",IF(LEFT($G174,4)="待确认：","待确认",IF(OR($A174="",$B174="",$C174="",$D174="",$E174=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B174))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A174))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E174="S",$E174="M",$E174="L")),"复杂度非法",IF(NOT(OR($F174="",$F174="内部集成",$F174="外部集成")),"集成类型非法",IF(AND($F174&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C174,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F174="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C174,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H174),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="175" ht="42" customHeight="1">
@@ -6502,7 +6502,7 @@
         <s:f>IF(COUNTA($A175:$G175)=0,"",IF($F175="",0,IF(NOT(ISNUMBER($I175)),"",IF($F175="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I175,1),IF($F175="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I175,1),"")))))</s:f>
       </s:c>
       <s:c r="L175" t="str" s="5">
-        <s:f>IF(COUNTA($A175:$G175)=0,"",IF(OR($A175="",$B175="",$C175="",$D175="",$E175=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B175))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A175))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E175="S",$E175="M",$E175="L")),"复杂度非法",IF(NOT(OR($F175="",$F175="内部集成",$F175="外部集成")),"集成类型非法",IF(AND($F175&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C175,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F175="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C175,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H175),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A175:$G175)=0,"",IF(LEFT($G175,4)="待确认：","待确认",IF(OR($A175="",$B175="",$C175="",$D175="",$E175=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B175))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A175))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E175="S",$E175="M",$E175="L")),"复杂度非法",IF(NOT(OR($F175="",$F175="内部集成",$F175="外部集成")),"集成类型非法",IF(AND($F175&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C175,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F175="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C175,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H175),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="176" ht="42" customHeight="1">
@@ -6526,7 +6526,7 @@
         <s:f>IF(COUNTA($A176:$G176)=0,"",IF($F176="",0,IF(NOT(ISNUMBER($I176)),"",IF($F176="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I176,1),IF($F176="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I176,1),"")))))</s:f>
       </s:c>
       <s:c r="L176" t="str" s="5">
-        <s:f>IF(COUNTA($A176:$G176)=0,"",IF(OR($A176="",$B176="",$C176="",$D176="",$E176=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B176))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A176))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E176="S",$E176="M",$E176="L")),"复杂度非法",IF(NOT(OR($F176="",$F176="内部集成",$F176="外部集成")),"集成类型非法",IF(AND($F176&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C176,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F176="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C176,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H176),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A176:$G176)=0,"",IF(LEFT($G176,4)="待确认：","待确认",IF(OR($A176="",$B176="",$C176="",$D176="",$E176=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B176))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A176))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E176="S",$E176="M",$E176="L")),"复杂度非法",IF(NOT(OR($F176="",$F176="内部集成",$F176="外部集成")),"集成类型非法",IF(AND($F176&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C176,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F176="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C176,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H176),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="177" ht="42" customHeight="1">
@@ -6550,7 +6550,7 @@
         <s:f>IF(COUNTA($A177:$G177)=0,"",IF($F177="",0,IF(NOT(ISNUMBER($I177)),"",IF($F177="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I177,1),IF($F177="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I177,1),"")))))</s:f>
       </s:c>
       <s:c r="L177" t="str" s="5">
-        <s:f>IF(COUNTA($A177:$G177)=0,"",IF(OR($A177="",$B177="",$C177="",$D177="",$E177=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B177))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A177))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E177="S",$E177="M",$E177="L")),"复杂度非法",IF(NOT(OR($F177="",$F177="内部集成",$F177="外部集成")),"集成类型非法",IF(AND($F177&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C177,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F177="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C177,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H177),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A177:$G177)=0,"",IF(LEFT($G177,4)="待确认：","待确认",IF(OR($A177="",$B177="",$C177="",$D177="",$E177=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B177))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A177))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E177="S",$E177="M",$E177="L")),"复杂度非法",IF(NOT(OR($F177="",$F177="内部集成",$F177="外部集成")),"集成类型非法",IF(AND($F177&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C177,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F177="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C177,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H177),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="178" ht="42" customHeight="1">
@@ -6574,7 +6574,7 @@
         <s:f>IF(COUNTA($A178:$G178)=0,"",IF($F178="",0,IF(NOT(ISNUMBER($I178)),"",IF($F178="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I178,1),IF($F178="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I178,1),"")))))</s:f>
       </s:c>
       <s:c r="L178" t="str" s="5">
-        <s:f>IF(COUNTA($A178:$G178)=0,"",IF(OR($A178="",$B178="",$C178="",$D178="",$E178=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B178))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A178))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E178="S",$E178="M",$E178="L")),"复杂度非法",IF(NOT(OR($F178="",$F178="内部集成",$F178="外部集成")),"集成类型非法",IF(AND($F178&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C178,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F178="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C178,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H178),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A178:$G178)=0,"",IF(LEFT($G178,4)="待确认：","待确认",IF(OR($A178="",$B178="",$C178="",$D178="",$E178=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B178))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A178))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E178="S",$E178="M",$E178="L")),"复杂度非法",IF(NOT(OR($F178="",$F178="内部集成",$F178="外部集成")),"集成类型非法",IF(AND($F178&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C178,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F178="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C178,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H178),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="179" ht="42" customHeight="1">
@@ -6598,7 +6598,7 @@
         <s:f>IF(COUNTA($A179:$G179)=0,"",IF($F179="",0,IF(NOT(ISNUMBER($I179)),"",IF($F179="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I179,1),IF($F179="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I179,1),"")))))</s:f>
       </s:c>
       <s:c r="L179" t="str" s="5">
-        <s:f>IF(COUNTA($A179:$G179)=0,"",IF(OR($A179="",$B179="",$C179="",$D179="",$E179=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B179))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A179))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E179="S",$E179="M",$E179="L")),"复杂度非法",IF(NOT(OR($F179="",$F179="内部集成",$F179="外部集成")),"集成类型非法",IF(AND($F179&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C179,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F179="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C179,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H179),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A179:$G179)=0,"",IF(LEFT($G179,4)="待确认：","待确认",IF(OR($A179="",$B179="",$C179="",$D179="",$E179=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B179))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A179))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E179="S",$E179="M",$E179="L")),"复杂度非法",IF(NOT(OR($F179="",$F179="内部集成",$F179="外部集成")),"集成类型非法",IF(AND($F179&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C179,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F179="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C179,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H179),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="180" ht="42" customHeight="1">
@@ -6622,7 +6622,7 @@
         <s:f>IF(COUNTA($A180:$G180)=0,"",IF($F180="",0,IF(NOT(ISNUMBER($I180)),"",IF($F180="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I180,1),IF($F180="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I180,1),"")))))</s:f>
       </s:c>
       <s:c r="L180" t="str" s="5">
-        <s:f>IF(COUNTA($A180:$G180)=0,"",IF(OR($A180="",$B180="",$C180="",$D180="",$E180=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B180))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A180))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E180="S",$E180="M",$E180="L")),"复杂度非法",IF(NOT(OR($F180="",$F180="内部集成",$F180="外部集成")),"集成类型非法",IF(AND($F180&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C180,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F180="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C180,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H180),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A180:$G180)=0,"",IF(LEFT($G180,4)="待确认：","待确认",IF(OR($A180="",$B180="",$C180="",$D180="",$E180=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B180))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A180))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E180="S",$E180="M",$E180="L")),"复杂度非法",IF(NOT(OR($F180="",$F180="内部集成",$F180="外部集成")),"集成类型非法",IF(AND($F180&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C180,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F180="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C180,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H180),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="181" ht="42" customHeight="1">
@@ -6646,7 +6646,7 @@
         <s:f>IF(COUNTA($A181:$G181)=0,"",IF($F181="",0,IF(NOT(ISNUMBER($I181)),"",IF($F181="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I181,1),IF($F181="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I181,1),"")))))</s:f>
       </s:c>
       <s:c r="L181" t="str" s="5">
-        <s:f>IF(COUNTA($A181:$G181)=0,"",IF(OR($A181="",$B181="",$C181="",$D181="",$E181=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B181))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A181))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E181="S",$E181="M",$E181="L")),"复杂度非法",IF(NOT(OR($F181="",$F181="内部集成",$F181="外部集成")),"集成类型非法",IF(AND($F181&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C181,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F181="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C181,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H181),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A181:$G181)=0,"",IF(LEFT($G181,4)="待确认：","待确认",IF(OR($A181="",$B181="",$C181="",$D181="",$E181=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B181))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A181))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E181="S",$E181="M",$E181="L")),"复杂度非法",IF(NOT(OR($F181="",$F181="内部集成",$F181="外部集成")),"集成类型非法",IF(AND($F181&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C181,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F181="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C181,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H181),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="182" ht="42" customHeight="1">
@@ -6670,7 +6670,7 @@
         <s:f>IF(COUNTA($A182:$G182)=0,"",IF($F182="",0,IF(NOT(ISNUMBER($I182)),"",IF($F182="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I182,1),IF($F182="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I182,1),"")))))</s:f>
       </s:c>
       <s:c r="L182" t="str" s="5">
-        <s:f>IF(COUNTA($A182:$G182)=0,"",IF(OR($A182="",$B182="",$C182="",$D182="",$E182=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B182))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A182))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E182="S",$E182="M",$E182="L")),"复杂度非法",IF(NOT(OR($F182="",$F182="内部集成",$F182="外部集成")),"集成类型非法",IF(AND($F182&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C182,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F182="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C182,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H182),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A182:$G182)=0,"",IF(LEFT($G182,4)="待确认：","待确认",IF(OR($A182="",$B182="",$C182="",$D182="",$E182=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B182))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A182))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E182="S",$E182="M",$E182="L")),"复杂度非法",IF(NOT(OR($F182="",$F182="内部集成",$F182="外部集成")),"集成类型非法",IF(AND($F182&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C182,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F182="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C182,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H182),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="183" ht="42" customHeight="1">
@@ -6694,7 +6694,7 @@
         <s:f>IF(COUNTA($A183:$G183)=0,"",IF($F183="",0,IF(NOT(ISNUMBER($I183)),"",IF($F183="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I183,1),IF($F183="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I183,1),"")))))</s:f>
       </s:c>
       <s:c r="L183" t="str" s="5">
-        <s:f>IF(COUNTA($A183:$G183)=0,"",IF(OR($A183="",$B183="",$C183="",$D183="",$E183=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B183))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A183))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E183="S",$E183="M",$E183="L")),"复杂度非法",IF(NOT(OR($F183="",$F183="内部集成",$F183="外部集成")),"集成类型非法",IF(AND($F183&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C183,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F183="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C183,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H183),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A183:$G183)=0,"",IF(LEFT($G183,4)="待确认：","待确认",IF(OR($A183="",$B183="",$C183="",$D183="",$E183=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B183))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A183))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E183="S",$E183="M",$E183="L")),"复杂度非法",IF(NOT(OR($F183="",$F183="内部集成",$F183="外部集成")),"集成类型非法",IF(AND($F183&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C183,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F183="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C183,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H183),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="184" ht="42" customHeight="1">
@@ -6718,7 +6718,7 @@
         <s:f>IF(COUNTA($A184:$G184)=0,"",IF($F184="",0,IF(NOT(ISNUMBER($I184)),"",IF($F184="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I184,1),IF($F184="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I184,1),"")))))</s:f>
       </s:c>
       <s:c r="L184" t="str" s="5">
-        <s:f>IF(COUNTA($A184:$G184)=0,"",IF(OR($A184="",$B184="",$C184="",$D184="",$E184=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B184))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A184))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E184="S",$E184="M",$E184="L")),"复杂度非法",IF(NOT(OR($F184="",$F184="内部集成",$F184="外部集成")),"集成类型非法",IF(AND($F184&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C184,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F184="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C184,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H184),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A184:$G184)=0,"",IF(LEFT($G184,4)="待确认：","待确认",IF(OR($A184="",$B184="",$C184="",$D184="",$E184=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B184))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A184))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E184="S",$E184="M",$E184="L")),"复杂度非法",IF(NOT(OR($F184="",$F184="内部集成",$F184="外部集成")),"集成类型非法",IF(AND($F184&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C184,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F184="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C184,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H184),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="185" ht="42" customHeight="1">
@@ -6742,7 +6742,7 @@
         <s:f>IF(COUNTA($A185:$G185)=0,"",IF($F185="",0,IF(NOT(ISNUMBER($I185)),"",IF($F185="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I185,1),IF($F185="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I185,1),"")))))</s:f>
       </s:c>
       <s:c r="L185" t="str" s="5">
-        <s:f>IF(COUNTA($A185:$G185)=0,"",IF(OR($A185="",$B185="",$C185="",$D185="",$E185=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B185))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A185))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E185="S",$E185="M",$E185="L")),"复杂度非法",IF(NOT(OR($F185="",$F185="内部集成",$F185="外部集成")),"集成类型非法",IF(AND($F185&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C185,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F185="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C185,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H185),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A185:$G185)=0,"",IF(LEFT($G185,4)="待确认：","待确认",IF(OR($A185="",$B185="",$C185="",$D185="",$E185=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B185))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A185))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E185="S",$E185="M",$E185="L")),"复杂度非法",IF(NOT(OR($F185="",$F185="内部集成",$F185="外部集成")),"集成类型非法",IF(AND($F185&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C185,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F185="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C185,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H185),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="186" ht="42" customHeight="1">
@@ -6766,7 +6766,7 @@
         <s:f>IF(COUNTA($A186:$G186)=0,"",IF($F186="",0,IF(NOT(ISNUMBER($I186)),"",IF($F186="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I186,1),IF($F186="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I186,1),"")))))</s:f>
       </s:c>
       <s:c r="L186" t="str" s="5">
-        <s:f>IF(COUNTA($A186:$G186)=0,"",IF(OR($A186="",$B186="",$C186="",$D186="",$E186=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B186))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A186))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E186="S",$E186="M",$E186="L")),"复杂度非法",IF(NOT(OR($F186="",$F186="内部集成",$F186="外部集成")),"集成类型非法",IF(AND($F186&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C186,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F186="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C186,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H186),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A186:$G186)=0,"",IF(LEFT($G186,4)="待确认：","待确认",IF(OR($A186="",$B186="",$C186="",$D186="",$E186=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B186))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A186))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E186="S",$E186="M",$E186="L")),"复杂度非法",IF(NOT(OR($F186="",$F186="内部集成",$F186="外部集成")),"集成类型非法",IF(AND($F186&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C186,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F186="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C186,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H186),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="187" ht="42" customHeight="1">
@@ -6790,7 +6790,7 @@
         <s:f>IF(COUNTA($A187:$G187)=0,"",IF($F187="",0,IF(NOT(ISNUMBER($I187)),"",IF($F187="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I187,1),IF($F187="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I187,1),"")))))</s:f>
       </s:c>
       <s:c r="L187" t="str" s="5">
-        <s:f>IF(COUNTA($A187:$G187)=0,"",IF(OR($A187="",$B187="",$C187="",$D187="",$E187=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B187))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A187))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E187="S",$E187="M",$E187="L")),"复杂度非法",IF(NOT(OR($F187="",$F187="内部集成",$F187="外部集成")),"集成类型非法",IF(AND($F187&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C187,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F187="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C187,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H187),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A187:$G187)=0,"",IF(LEFT($G187,4)="待确认：","待确认",IF(OR($A187="",$B187="",$C187="",$D187="",$E187=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B187))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A187))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E187="S",$E187="M",$E187="L")),"复杂度非法",IF(NOT(OR($F187="",$F187="内部集成",$F187="外部集成")),"集成类型非法",IF(AND($F187&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C187,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F187="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C187,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H187),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="188" ht="42" customHeight="1">
@@ -6814,7 +6814,7 @@
         <s:f>IF(COUNTA($A188:$G188)=0,"",IF($F188="",0,IF(NOT(ISNUMBER($I188)),"",IF($F188="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I188,1),IF($F188="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I188,1),"")))))</s:f>
       </s:c>
       <s:c r="L188" t="str" s="5">
-        <s:f>IF(COUNTA($A188:$G188)=0,"",IF(OR($A188="",$B188="",$C188="",$D188="",$E188=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B188))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A188))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E188="S",$E188="M",$E188="L")),"复杂度非法",IF(NOT(OR($F188="",$F188="内部集成",$F188="外部集成")),"集成类型非法",IF(AND($F188&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C188,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F188="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C188,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H188),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A188:$G188)=0,"",IF(LEFT($G188,4)="待确认：","待确认",IF(OR($A188="",$B188="",$C188="",$D188="",$E188=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B188))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A188))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E188="S",$E188="M",$E188="L")),"复杂度非法",IF(NOT(OR($F188="",$F188="内部集成",$F188="外部集成")),"集成类型非法",IF(AND($F188&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C188,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F188="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C188,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H188),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="189" ht="42" customHeight="1">
@@ -6838,7 +6838,7 @@
         <s:f>IF(COUNTA($A189:$G189)=0,"",IF($F189="",0,IF(NOT(ISNUMBER($I189)),"",IF($F189="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I189,1),IF($F189="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I189,1),"")))))</s:f>
       </s:c>
       <s:c r="L189" t="str" s="5">
-        <s:f>IF(COUNTA($A189:$G189)=0,"",IF(OR($A189="",$B189="",$C189="",$D189="",$E189=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B189))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A189))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E189="S",$E189="M",$E189="L")),"复杂度非法",IF(NOT(OR($F189="",$F189="内部集成",$F189="外部集成")),"集成类型非法",IF(AND($F189&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C189,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F189="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C189,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H189),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A189:$G189)=0,"",IF(LEFT($G189,4)="待确认：","待确认",IF(OR($A189="",$B189="",$C189="",$D189="",$E189=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B189))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A189))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E189="S",$E189="M",$E189="L")),"复杂度非法",IF(NOT(OR($F189="",$F189="内部集成",$F189="外部集成")),"集成类型非法",IF(AND($F189&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C189,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F189="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C189,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H189),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="190" ht="42" customHeight="1">
@@ -6862,7 +6862,7 @@
         <s:f>IF(COUNTA($A190:$G190)=0,"",IF($F190="",0,IF(NOT(ISNUMBER($I190)),"",IF($F190="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I190,1),IF($F190="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I190,1),"")))))</s:f>
       </s:c>
       <s:c r="L190" t="str" s="5">
-        <s:f>IF(COUNTA($A190:$G190)=0,"",IF(OR($A190="",$B190="",$C190="",$D190="",$E190=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B190))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A190))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E190="S",$E190="M",$E190="L")),"复杂度非法",IF(NOT(OR($F190="",$F190="内部集成",$F190="外部集成")),"集成类型非法",IF(AND($F190&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C190,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F190="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C190,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H190),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A190:$G190)=0,"",IF(LEFT($G190,4)="待确认：","待确认",IF(OR($A190="",$B190="",$C190="",$D190="",$E190=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B190))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A190))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E190="S",$E190="M",$E190="L")),"复杂度非法",IF(NOT(OR($F190="",$F190="内部集成",$F190="外部集成")),"集成类型非法",IF(AND($F190&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C190,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F190="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C190,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H190),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="191" ht="42" customHeight="1">
@@ -6886,7 +6886,7 @@
         <s:f>IF(COUNTA($A191:$G191)=0,"",IF($F191="",0,IF(NOT(ISNUMBER($I191)),"",IF($F191="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I191,1),IF($F191="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I191,1),"")))))</s:f>
       </s:c>
       <s:c r="L191" t="str" s="5">
-        <s:f>IF(COUNTA($A191:$G191)=0,"",IF(OR($A191="",$B191="",$C191="",$D191="",$E191=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B191))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A191))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E191="S",$E191="M",$E191="L")),"复杂度非法",IF(NOT(OR($F191="",$F191="内部集成",$F191="外部集成")),"集成类型非法",IF(AND($F191&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C191,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F191="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C191,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H191),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A191:$G191)=0,"",IF(LEFT($G191,4)="待确认：","待确认",IF(OR($A191="",$B191="",$C191="",$D191="",$E191=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B191))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A191))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E191="S",$E191="M",$E191="L")),"复杂度非法",IF(NOT(OR($F191="",$F191="内部集成",$F191="外部集成")),"集成类型非法",IF(AND($F191&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C191,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F191="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C191,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H191),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="192" ht="42" customHeight="1">
@@ -6910,7 +6910,7 @@
         <s:f>IF(COUNTA($A192:$G192)=0,"",IF($F192="",0,IF(NOT(ISNUMBER($I192)),"",IF($F192="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I192,1),IF($F192="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I192,1),"")))))</s:f>
       </s:c>
       <s:c r="L192" t="str" s="5">
-        <s:f>IF(COUNTA($A192:$G192)=0,"",IF(OR($A192="",$B192="",$C192="",$D192="",$E192=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B192))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A192))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E192="S",$E192="M",$E192="L")),"复杂度非法",IF(NOT(OR($F192="",$F192="内部集成",$F192="外部集成")),"集成类型非法",IF(AND($F192&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C192,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F192="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C192,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H192),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A192:$G192)=0,"",IF(LEFT($G192,4)="待确认：","待确认",IF(OR($A192="",$B192="",$C192="",$D192="",$E192=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B192))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A192))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E192="S",$E192="M",$E192="L")),"复杂度非法",IF(NOT(OR($F192="",$F192="内部集成",$F192="外部集成")),"集成类型非法",IF(AND($F192&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C192,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F192="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C192,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H192),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="193" ht="42" customHeight="1">
@@ -6934,7 +6934,7 @@
         <s:f>IF(COUNTA($A193:$G193)=0,"",IF($F193="",0,IF(NOT(ISNUMBER($I193)),"",IF($F193="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I193,1),IF($F193="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I193,1),"")))))</s:f>
       </s:c>
       <s:c r="L193" t="str" s="5">
-        <s:f>IF(COUNTA($A193:$G193)=0,"",IF(OR($A193="",$B193="",$C193="",$D193="",$E193=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B193))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A193))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E193="S",$E193="M",$E193="L")),"复杂度非法",IF(NOT(OR($F193="",$F193="内部集成",$F193="外部集成")),"集成类型非法",IF(AND($F193&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C193,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F193="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C193,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H193),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A193:$G193)=0,"",IF(LEFT($G193,4)="待确认：","待确认",IF(OR($A193="",$B193="",$C193="",$D193="",$E193=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B193))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A193))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E193="S",$E193="M",$E193="L")),"复杂度非法",IF(NOT(OR($F193="",$F193="内部集成",$F193="外部集成")),"集成类型非法",IF(AND($F193&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C193,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F193="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C193,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H193),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="194" ht="42" customHeight="1">
@@ -6958,7 +6958,7 @@
         <s:f>IF(COUNTA($A194:$G194)=0,"",IF($F194="",0,IF(NOT(ISNUMBER($I194)),"",IF($F194="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I194,1),IF($F194="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I194,1),"")))))</s:f>
       </s:c>
       <s:c r="L194" t="str" s="5">
-        <s:f>IF(COUNTA($A194:$G194)=0,"",IF(OR($A194="",$B194="",$C194="",$D194="",$E194=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B194))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A194))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E194="S",$E194="M",$E194="L")),"复杂度非法",IF(NOT(OR($F194="",$F194="内部集成",$F194="外部集成")),"集成类型非法",IF(AND($F194&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C194,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F194="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C194,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H194),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A194:$G194)=0,"",IF(LEFT($G194,4)="待确认：","待确认",IF(OR($A194="",$B194="",$C194="",$D194="",$E194=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B194))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A194))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E194="S",$E194="M",$E194="L")),"复杂度非法",IF(NOT(OR($F194="",$F194="内部集成",$F194="外部集成")),"集成类型非法",IF(AND($F194&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C194,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F194="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C194,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H194),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="195" ht="42" customHeight="1">
@@ -6982,7 +6982,7 @@
         <s:f>IF(COUNTA($A195:$G195)=0,"",IF($F195="",0,IF(NOT(ISNUMBER($I195)),"",IF($F195="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I195,1),IF($F195="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I195,1),"")))))</s:f>
       </s:c>
       <s:c r="L195" t="str" s="5">
-        <s:f>IF(COUNTA($A195:$G195)=0,"",IF(OR($A195="",$B195="",$C195="",$D195="",$E195=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B195))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A195))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E195="S",$E195="M",$E195="L")),"复杂度非法",IF(NOT(OR($F195="",$F195="内部集成",$F195="外部集成")),"集成类型非法",IF(AND($F195&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C195,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F195="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C195,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H195),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A195:$G195)=0,"",IF(LEFT($G195,4)="待确认：","待确认",IF(OR($A195="",$B195="",$C195="",$D195="",$E195=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B195))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A195))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E195="S",$E195="M",$E195="L")),"复杂度非法",IF(NOT(OR($F195="",$F195="内部集成",$F195="外部集成")),"集成类型非法",IF(AND($F195&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C195,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F195="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C195,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H195),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="196" ht="42" customHeight="1">
@@ -7006,7 +7006,7 @@
         <s:f>IF(COUNTA($A196:$G196)=0,"",IF($F196="",0,IF(NOT(ISNUMBER($I196)),"",IF($F196="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I196,1),IF($F196="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I196,1),"")))))</s:f>
       </s:c>
       <s:c r="L196" t="str" s="5">
-        <s:f>IF(COUNTA($A196:$G196)=0,"",IF(OR($A196="",$B196="",$C196="",$D196="",$E196=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B196))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A196))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E196="S",$E196="M",$E196="L")),"复杂度非法",IF(NOT(OR($F196="",$F196="内部集成",$F196="外部集成")),"集成类型非法",IF(AND($F196&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C196,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F196="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C196,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H196),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A196:$G196)=0,"",IF(LEFT($G196,4)="待确认：","待确认",IF(OR($A196="",$B196="",$C196="",$D196="",$E196=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B196))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A196))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E196="S",$E196="M",$E196="L")),"复杂度非法",IF(NOT(OR($F196="",$F196="内部集成",$F196="外部集成")),"集成类型非法",IF(AND($F196&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C196,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F196="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C196,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H196),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="197" ht="42" customHeight="1">
@@ -7030,7 +7030,7 @@
         <s:f>IF(COUNTA($A197:$G197)=0,"",IF($F197="",0,IF(NOT(ISNUMBER($I197)),"",IF($F197="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I197,1),IF($F197="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I197,1),"")))))</s:f>
       </s:c>
       <s:c r="L197" t="str" s="5">
-        <s:f>IF(COUNTA($A197:$G197)=0,"",IF(OR($A197="",$B197="",$C197="",$D197="",$E197=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B197))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A197))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E197="S",$E197="M",$E197="L")),"复杂度非法",IF(NOT(OR($F197="",$F197="内部集成",$F197="外部集成")),"集成类型非法",IF(AND($F197&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C197,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F197="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C197,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H197),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A197:$G197)=0,"",IF(LEFT($G197,4)="待确认：","待确认",IF(OR($A197="",$B197="",$C197="",$D197="",$E197=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B197))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A197))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E197="S",$E197="M",$E197="L")),"复杂度非法",IF(NOT(OR($F197="",$F197="内部集成",$F197="外部集成")),"集成类型非法",IF(AND($F197&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C197,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F197="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C197,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H197),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="198" ht="42" customHeight="1">
@@ -7054,7 +7054,7 @@
         <s:f>IF(COUNTA($A198:$G198)=0,"",IF($F198="",0,IF(NOT(ISNUMBER($I198)),"",IF($F198="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I198,1),IF($F198="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I198,1),"")))))</s:f>
       </s:c>
       <s:c r="L198" t="str" s="5">
-        <s:f>IF(COUNTA($A198:$G198)=0,"",IF(OR($A198="",$B198="",$C198="",$D198="",$E198=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B198))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A198))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E198="S",$E198="M",$E198="L")),"复杂度非法",IF(NOT(OR($F198="",$F198="内部集成",$F198="外部集成")),"集成类型非法",IF(AND($F198&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C198,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F198="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C198,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H198),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A198:$G198)=0,"",IF(LEFT($G198,4)="待确认：","待确认",IF(OR($A198="",$B198="",$C198="",$D198="",$E198=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B198))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A198))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E198="S",$E198="M",$E198="L")),"复杂度非法",IF(NOT(OR($F198="",$F198="内部集成",$F198="外部集成")),"集成类型非法",IF(AND($F198&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C198,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F198="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C198,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H198),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="199" ht="42" customHeight="1">
@@ -7078,7 +7078,7 @@
         <s:f>IF(COUNTA($A199:$G199)=0,"",IF($F199="",0,IF(NOT(ISNUMBER($I199)),"",IF($F199="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I199,1),IF($F199="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I199,1),"")))))</s:f>
       </s:c>
       <s:c r="L199" t="str" s="5">
-        <s:f>IF(COUNTA($A199:$G199)=0,"",IF(OR($A199="",$B199="",$C199="",$D199="",$E199=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B199))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A199))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E199="S",$E199="M",$E199="L")),"复杂度非法",IF(NOT(OR($F199="",$F199="内部集成",$F199="外部集成")),"集成类型非法",IF(AND($F199&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C199,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F199="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C199,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H199),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A199:$G199)=0,"",IF(LEFT($G199,4)="待确认：","待确认",IF(OR($A199="",$B199="",$C199="",$D199="",$E199=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B199))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A199))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E199="S",$E199="M",$E199="L")),"复杂度非法",IF(NOT(OR($F199="",$F199="内部集成",$F199="外部集成")),"集成类型非法",IF(AND($F199&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C199,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F199="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C199,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H199),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="200" ht="42" customHeight="1">
@@ -7102,7 +7102,7 @@
         <s:f>IF(COUNTA($A200:$G200)=0,"",IF($F200="",0,IF(NOT(ISNUMBER($I200)),"",IF($F200="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I200,1),IF($F200="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I200,1),"")))))</s:f>
       </s:c>
       <s:c r="L200" t="str" s="5">
-        <s:f>IF(COUNTA($A200:$G200)=0,"",IF(OR($A200="",$B200="",$C200="",$D200="",$E200=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B200))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A200))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E200="S",$E200="M",$E200="L")),"复杂度非法",IF(NOT(OR($F200="",$F200="内部集成",$F200="外部集成")),"集成类型非法",IF(AND($F200&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C200,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F200="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C200,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H200),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A200:$G200)=0,"",IF(LEFT($G200,4)="待确认：","待确认",IF(OR($A200="",$B200="",$C200="",$D200="",$E200=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B200))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A200))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E200="S",$E200="M",$E200="L")),"复杂度非法",IF(NOT(OR($F200="",$F200="内部集成",$F200="外部集成")),"集成类型非法",IF(AND($F200&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C200,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F200="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C200,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H200),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="201" ht="42" customHeight="1">
@@ -7126,7 +7126,7 @@
         <s:f>IF(COUNTA($A201:$G201)=0,"",IF($F201="",0,IF(NOT(ISNUMBER($I201)),"",IF($F201="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I201,1),IF($F201="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I201,1),"")))))</s:f>
       </s:c>
       <s:c r="L201" t="str" s="5">
-        <s:f>IF(COUNTA($A201:$G201)=0,"",IF(OR($A201="",$B201="",$C201="",$D201="",$E201=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B201))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A201))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E201="S",$E201="M",$E201="L")),"复杂度非法",IF(NOT(OR($F201="",$F201="内部集成",$F201="外部集成")),"集成类型非法",IF(AND($F201&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C201,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F201="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C201,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H201),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A201:$G201)=0,"",IF(LEFT($G201,4)="待确认：","待确认",IF(OR($A201="",$B201="",$C201="",$D201="",$E201=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B201))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A201))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E201="S",$E201="M",$E201="L")),"复杂度非法",IF(NOT(OR($F201="",$F201="内部集成",$F201="外部集成")),"集成类型非法",IF(AND($F201&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C201,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F201="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C201,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H201),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="202" ht="42" customHeight="1">
@@ -7150,7 +7150,7 @@
         <s:f>IF(COUNTA($A202:$G202)=0,"",IF($F202="",0,IF(NOT(ISNUMBER($I202)),"",IF($F202="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I202,1),IF($F202="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I202,1),"")))))</s:f>
       </s:c>
       <s:c r="L202" t="str" s="5">
-        <s:f>IF(COUNTA($A202:$G202)=0,"",IF(OR($A202="",$B202="",$C202="",$D202="",$E202=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B202))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A202))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E202="S",$E202="M",$E202="L")),"复杂度非法",IF(NOT(OR($F202="",$F202="内部集成",$F202="外部集成")),"集成类型非法",IF(AND($F202&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C202,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F202="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C202,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H202),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A202:$G202)=0,"",IF(LEFT($G202,4)="待确认：","待确认",IF(OR($A202="",$B202="",$C202="",$D202="",$E202=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B202))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A202))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E202="S",$E202="M",$E202="L")),"复杂度非法",IF(NOT(OR($F202="",$F202="内部集成",$F202="外部集成")),"集成类型非法",IF(AND($F202&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C202,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F202="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C202,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H202),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="203" ht="42" customHeight="1">
@@ -7174,7 +7174,7 @@
         <s:f>IF(COUNTA($A203:$G203)=0,"",IF($F203="",0,IF(NOT(ISNUMBER($I203)),"",IF($F203="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I203,1),IF($F203="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I203,1),"")))))</s:f>
       </s:c>
       <s:c r="L203" t="str" s="5">
-        <s:f>IF(COUNTA($A203:$G203)=0,"",IF(OR($A203="",$B203="",$C203="",$D203="",$E203=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B203))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A203))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E203="S",$E203="M",$E203="L")),"复杂度非法",IF(NOT(OR($F203="",$F203="内部集成",$F203="外部集成")),"集成类型非法",IF(AND($F203&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C203,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F203="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C203,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H203),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A203:$G203)=0,"",IF(LEFT($G203,4)="待确认：","待确认",IF(OR($A203="",$B203="",$C203="",$D203="",$E203=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B203))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A203))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E203="S",$E203="M",$E203="L")),"复杂度非法",IF(NOT(OR($F203="",$F203="内部集成",$F203="外部集成")),"集成类型非法",IF(AND($F203&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C203,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F203="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C203,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H203),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
     <s:row r="204" ht="42" customHeight="1">
@@ -7198,7 +7198,7 @@
         <s:f>IF(COUNTA($A204:$G204)=0,"",IF($F204="",0,IF(NOT(ISNUMBER($I204)),"",IF($F204="内部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("内部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I204,1),IF($F204="外部集成",ROUND(INDEX(ProjectParameterTable[当前值],MATCH("外部集成点SIT支持",ProjectParameterTable[参数名称],0))*$I204,1),"")))))</s:f>
       </s:c>
       <s:c r="L204" t="str" s="5">
-        <s:f>IF(COUNTA($A204:$G204)=0,"",IF(OR($A204="",$B204="",$C204="",$D204="",$E204=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B204))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A204))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E204="S",$E204="M",$E204="L")),"复杂度非法",IF(NOT(OR($F204="",$F204="内部集成",$F204="外部集成")),"集成类型非法",IF(AND($F204&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C204,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F204="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C204,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H204),"通过","工作类型与工作方式不适用")))))))))</s:f>
+        <s:f>IF(COUNTA($A204:$G204)=0,"",IF(LEFT($G204,4)="待确认：","待确认",IF(OR($A204="",$B204="",$C204="",$D204="",$E204=""),"必填项缺失",IF(SUMPRODUCT(--(TaskTable[任务名称]=$B204))&gt;1,"任务名称重复",IF(SUMPRODUCT(--(SOWStoryTable[故事]=$A204))&lt;&gt;1,"所属故事未知",IF(NOT(OR($E204="S",$E204="M",$E204="L")),"复杂度非法",IF(NOT(OR($F204="",$F204="内部集成",$F204="外部集成")),"集成类型非法",IF(AND($F204&lt;&gt;"",NOT(IFERROR(INDEX(TaskStandardTable[分类],MATCH($C204,TaskStandardTable[工作类型],0)),"")="系统集成")),"非集成任务不应填写集成类型",IF(AND($F204="",IFERROR(INDEX(TaskStandardTable[分类],MATCH($C204,TaskStandardTable[工作类型],0)),"")="系统集成"),"集成类型缺失",IF(ISNUMBER($H204),"通过","工作类型与工作方式不适用"))))))))))</s:f>
       </s:c>
     </s:row>
   </s:sheetData>

</xml_diff>